<commit_message>
Fix catalog integrity and monitoring safeguards
</commit_message>
<xml_diff>
--- a/catalog/quality_catalog.xlsx
+++ b/catalog/quality_catalog.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rae5a21efee29404f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search" sheetId="2" r:id="R3063a38750c946c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="3" r:id="R1852161fef5d4078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="4" r:id="R7e67daac967b44eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="5" r:id="R5e3bdd8dc8354839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="6" r:id="Rd9e1c11848c1461b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PSU" sheetId="7" r:id="R3b43fb0b26ef452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motherboard" sheetId="8" r:id="Rba49ce058d99438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitor" sheetId="9" r:id="R7639385d055b483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifiers" sheetId="10" r:id="Rd05a207adc4749c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="11" r:id="Rd26a81cd60154115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="12" r:id="Rdd2e623c14f34fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="13" r:id="Rafd545fe0cf74310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="14" r:id="Rf4acd1b59f07428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" r:id="R61601278cc6740aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SheetDefinitions" sheetId="16" r:id="Ree1ba347fbb84ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDefinitions" sheetId="17" r:id="R838bca49b6234ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" r:id="R56f49ce0527e46d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPUChips" sheetId="19" r:id="R1ff1194fd9ae4008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R09c47f1f21614974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search" sheetId="2" r:id="R97835d0666cf4df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="3" r:id="Ra362d31abacf4598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="4" r:id="Rd89dc71bee4c43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="5" r:id="R0a50948d92124688"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="6" r:id="R6c96d6ff06ba4fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PSU" sheetId="7" r:id="R7e3b40c22657474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motherboard" sheetId="8" r:id="R86bac745f273485e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitor" sheetId="9" r:id="Ra67db51a50674f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifiers" sheetId="10" r:id="R617d0ab61d524d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="11" r:id="R913c5df0f03b4637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="12" r:id="R7d5a66584dda4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="13" r:id="R5e10acd8fdd24f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="14" r:id="R402a3a2cc7df4190"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" r:id="R836bde92f0fe4283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SheetDefinitions" sheetId="16" r:id="Rfc5d49b8c49b419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDefinitions" sheetId="17" r:id="R944dc2fe72c04b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" r:id="R080cf0bc2c4a4ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPUChips" sheetId="19" r:id="Rb69935859f914bf8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2044,7 +2044,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf83fce68bab4e0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81bd26549108438f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9972,7 +9972,7 @@
         <x:v>AMD Radeon RX 6700 公式世代・仕様情報</x:v>
       </x:c>
       <x:c r="E239" s="121" t="str">
-        <x:v>https://www.amd.com/en/products/graphics/desktops/radeon.html</x:v>
+        <x:v>https://www.amd.com/en/products/graphics/desktops/radeon/6000-series/amd-radeon-rx-6700.html</x:v>
       </x:c>
       <x:c r="F239" s="125" t="n">
         <x:v>46218</x:v>
@@ -13844,27 +13844,72 @@
         <x:v>GPU Mega Page（最終更新2026-07-14）から取得。投稿サンプル更新により変動します。</x:v>
       </x:c>
     </x:row>
-    <x:row r="355">
-      <x:c r="A355"/>
-      <x:c r="B355"/>
-      <x:c r="C355"/>
-      <x:c r="D355" s="121"/>
-      <x:c r="E355" s="121"/>
-      <x:c r="F355" s="125"/>
-      <x:c r="G355" s="121"/>
-      <x:c r="H355" s="121"/>
-      <x:c r="I355" s="121"/>
-    </x:row>
-    <x:row r="356">
-      <x:c r="A356"/>
-      <x:c r="B356"/>
-      <x:c r="C356"/>
-      <x:c r="D356" s="121"/>
-      <x:c r="E356" s="121"/>
-      <x:c r="F356" s="125"/>
-      <x:c r="G356" s="121"/>
-      <x:c r="H356" s="121"/>
-      <x:c r="I356" s="121"/>
+    <x:row r="355" ht="42" customHeight="1">
+      <x:c r="A355" t="str">
+        <x:v>amd-radeon-rx-6500-xt-8gb-official</x:v>
+      </x:c>
+      <x:c r="B355" t="str">
+        <x:v>amd-radeon-rx-6500-xt-8gb</x:v>
+      </x:c>
+      <x:c r="C355" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D355" s="121" t="str">
+        <x:v>AMD Radeon RX 6500 XT 8GB 公式仕様情報</x:v>
+      </x:c>
+      <x:c r="E355" s="121" t="str">
+        <x:v>https://www.amd.com/en/products/graphics/desktops/radeon/6000-series/amd-radeon-rx-6500-xt.html</x:v>
+      </x:c>
+      <x:c r="F355" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G355" s="121" t="str">
+        <x:v>specs.architecture
+specs.generation
+specs.release_date
+specs.launch_period
+specs.vram_gb
+specs.memory_type
+specs.memory_bus_bits</x:v>
+      </x:c>
+      <x:c r="H355" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I355" s="121" t="str">
+        <x:v>AMD公式ページで8GB、RDNA 2、64-bit GDDR6、発売日を確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356" ht="42" customHeight="1">
+      <x:c r="A356" t="str">
+        <x:v>amd-radeon-rx-6500-xt-8gb-passmark</x:v>
+      </x:c>
+      <x:c r="B356" t="str">
+        <x:v>amd-radeon-rx-6500-xt-8gb</x:v>
+      </x:c>
+      <x:c r="C356" t="str">
+        <x:v>technical_database</x:v>
+      </x:c>
+      <x:c r="D356" s="121" t="str">
+        <x:v>Radeon RX 6500 XT PassMark benchmark（4GB/8GB共通集計）</x:v>
+      </x:c>
+      <x:c r="E356" s="121" t="str">
+        <x:v>https://www.videocardbenchmark.net/video_lookup.php?gpu=Radeon+RX+6500+XT&amp;id=4488</x:v>
+      </x:c>
+      <x:c r="F356" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G356" s="121" t="str">
+        <x:v>specs.passmark_g3d_mark
+specs.passmark_g2d_mark
+specs.benchmark_reported_tdp_w
+specs.passmark_checked_at</x:v>
+      </x:c>
+      <x:c r="H356" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I356" s="121" t="str">
+        <x:v>PassMarkはVRAM容量別に分離していないため共通スコアを参考値として記録。</x:v>
+      </x:c>
     </x:row>
     <x:row r="357">
       <x:c r="A357"/>
@@ -14076,7 +14121,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1738ba66d12747dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R517aef469ce84447"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14698,7 +14743,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R887f2297a1ac4b08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9a1e09d257e417d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15380,7 +15425,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cad639b3ab34d73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ecb08a4b6af43d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15789,7 +15834,7 @@
         <x:v>in</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>["A","B"]</x:v>
+        <x:v>["S","A","B"]</x:v>
       </x:c>
       <x:c r="F18" s="14" t="n">
         <x:v>30</x:v>
@@ -17339,7 +17384,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra88312a7eb58435a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re721ce02c8e84018"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17462,7 +17507,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcbc2775bc8b46b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R506d06735b39465b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17726,7 +17771,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cd4690b9f2e4f75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c99b6ddd7348f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24358,7 +24403,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5853d4ba4d448af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbc0cc467dbb4b93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25364,7 +25409,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R632568276b0f410b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9165a06c2daa4c39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25718,8 +25763,7 @@
         <x:v>AMD Radeon RX 6500 XT 4GB</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>Radeon RX 6500 XT 4GB
-Radeon RX 6500 XT</x:v>
+        <x:v>Radeon RX 6500 XT 4GB</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
         <x:v>research_required</x:v>
@@ -25780,19 +25824,19 @@
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>amd-radeon-rx-6600</x:v>
+        <x:v>amd-radeon-rx-6500-xt-8gb</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>Radeon RX 6600</x:v>
+        <x:v>Radeon RX 6500 XT 8GB</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>AMD Radeon RX 6600</x:v>
+        <x:v>AMD Radeon RX 6500 XT 8GB</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>Radeon RX 6600</x:v>
+        <x:v>Radeon RX 6500 XT 8GB</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
         <x:v>research_required</x:v>
@@ -25812,7 +25856,7 @@
         <x:v>ボードメーカー別の品質・保証・電源・寸法は未評価</x:v>
       </x:c>
       <x:c r="M7" s="14" t="str">
-        <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
+        <x:v>PassMarkは4GB/8GBを別集計していないため共通スコアを参考値として使用。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
         <x:v>RDNA 2</x:v>
@@ -25821,10 +25865,10 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P7" s="102" t="n">
-        <x:v>44482</x:v>
+        <x:v>44580</x:v>
       </x:c>
       <x:c r="Q7" s="12" t="str">
-        <x:v>2021-10-13</x:v>
+        <x:v>2022-01-19</x:v>
       </x:c>
       <x:c r="R7" s="12" t="str">
         <x:v>exact</x:v>
@@ -25836,16 +25880,16 @@
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U7" s="105" t="n">
-        <x:v>128</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="V7" s="105" t="n">
-        <x:v>15054</x:v>
+        <x:v>9622</x:v>
       </x:c>
       <x:c r="W7" s="105" t="n">
-        <x:v>896</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="X7" s="105" t="n">
-        <x:v>132</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="Y7" s="102" t="n">
         <x:v>46218</x:v>
@@ -25853,19 +25897,19 @@
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>amd-radeon-rx-6600-xt</x:v>
+        <x:v>amd-radeon-rx-6600</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>Radeon RX 6600 XT</x:v>
+        <x:v>Radeon RX 6600</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>AMD Radeon RX 6600 XT</x:v>
+        <x:v>AMD Radeon RX 6600</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>Radeon RX 6600 XT</x:v>
+        <x:v>Radeon RX 6600</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
         <x:v>research_required</x:v>
@@ -25894,10 +25938,10 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P8" s="102" t="n">
-        <x:v>44419</x:v>
+        <x:v>44482</x:v>
       </x:c>
       <x:c r="Q8" s="12" t="str">
-        <x:v>2021-08-11</x:v>
+        <x:v>2021-10-13</x:v>
       </x:c>
       <x:c r="R8" s="12" t="str">
         <x:v>exact</x:v>
@@ -25912,13 +25956,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V8" s="105" t="n">
-        <x:v>16440</x:v>
+        <x:v>15054</x:v>
       </x:c>
       <x:c r="W8" s="105" t="n">
-        <x:v>914</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="X8" s="105" t="n">
-        <x:v>160</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="Y8" s="102" t="n">
         <x:v>46218</x:v>
@@ -25926,19 +25970,19 @@
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>amd-radeon-rx-6650-xt</x:v>
+        <x:v>amd-radeon-rx-6600-xt</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>Radeon RX 6650 XT</x:v>
+        <x:v>Radeon RX 6600 XT</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>AMD Radeon RX 6650 XT</x:v>
+        <x:v>AMD Radeon RX 6600 XT</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>Radeon RX 6650 XT</x:v>
+        <x:v>Radeon RX 6600 XT</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
         <x:v>research_required</x:v>
@@ -25967,10 +26011,10 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P9" s="102" t="n">
-        <x:v>44691</x:v>
+        <x:v>44419</x:v>
       </x:c>
       <x:c r="Q9" s="12" t="str">
-        <x:v>2022-05-10</x:v>
+        <x:v>2021-08-11</x:v>
       </x:c>
       <x:c r="R9" s="12" t="str">
         <x:v>exact</x:v>
@@ -25985,13 +26029,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V9" s="105" t="n">
-        <x:v>17113</x:v>
+        <x:v>16440</x:v>
       </x:c>
       <x:c r="W9" s="105" t="n">
-        <x:v>926</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="X9" s="105" t="n">
-        <x:v>176</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="Y9" s="102" t="n">
         <x:v>46218</x:v>
@@ -25999,19 +26043,19 @@
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>amd-radeon-rx-6700</x:v>
+        <x:v>amd-radeon-rx-6650-xt</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>Radeon RX 6700</x:v>
+        <x:v>Radeon RX 6650 XT</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>AMD Radeon RX 6700</x:v>
+        <x:v>AMD Radeon RX 6650 XT</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>Radeon RX 6700</x:v>
+        <x:v>Radeon RX 6650 XT</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26039,30 +26083,32 @@
       <x:c r="O10" s="12" t="str">
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
-      <x:c r="P10" s="102"/>
+      <x:c r="P10" s="102" t="n">
+        <x:v>44691</x:v>
+      </x:c>
       <x:c r="Q10" s="12" t="str">
-        <x:v>Q2'22</x:v>
+        <x:v>2022-05-10</x:v>
       </x:c>
       <x:c r="R10" s="12" t="str">
-        <x:v>quarter</x:v>
+        <x:v>exact</x:v>
       </x:c>
       <x:c r="S10" s="104" t="n">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T10" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U10" s="105" t="n">
-        <x:v>160</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="V10" s="105" t="n">
-        <x:v>18929</x:v>
+        <x:v>17113</x:v>
       </x:c>
       <x:c r="W10" s="105" t="n">
-        <x:v>941</x:v>
+        <x:v>926</x:v>
       </x:c>
       <x:c r="X10" s="105" t="n">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="Y10" s="102" t="n">
         <x:v>46218</x:v>
@@ -26070,19 +26116,19 @@
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>amd-radeon-rx-6700-xt</x:v>
+        <x:v>amd-radeon-rx-6700</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>Radeon RX 6700 XT</x:v>
+        <x:v>Radeon RX 6700</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>AMD Radeon RX 6700 XT</x:v>
+        <x:v>AMD Radeon RX 6700</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>Radeon RX 6700 XT</x:v>
+        <x:v>Radeon RX 6700</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26111,31 +26157,31 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P11" s="102" t="n">
-        <x:v>44273</x:v>
+        <x:v>44356</x:v>
       </x:c>
       <x:c r="Q11" s="12" t="str">
-        <x:v>2021-03-18</x:v>
+        <x:v>2021-06-09</x:v>
       </x:c>
       <x:c r="R11" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S11" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T11" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U11" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="V11" s="105" t="n">
-        <x:v>19730</x:v>
+        <x:v>18929</x:v>
       </x:c>
       <x:c r="W11" s="105" t="n">
-        <x:v>954</x:v>
+        <x:v>941</x:v>
       </x:c>
       <x:c r="X11" s="105" t="n">
-        <x:v>230</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="Y11" s="102" t="n">
         <x:v>46218</x:v>
@@ -26143,19 +26189,19 @@
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>amd-radeon-rx-6750-xt</x:v>
+        <x:v>amd-radeon-rx-6700-xt</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>Radeon RX 6750 XT</x:v>
+        <x:v>Radeon RX 6700 XT</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>AMD Radeon RX 6750 XT</x:v>
+        <x:v>AMD Radeon RX 6700 XT</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>Radeon RX 6750 XT</x:v>
+        <x:v>Radeon RX 6700 XT</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26184,10 +26230,10 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P12" s="102" t="n">
-        <x:v>44691</x:v>
+        <x:v>44273</x:v>
       </x:c>
       <x:c r="Q12" s="12" t="str">
-        <x:v>2022-05-10</x:v>
+        <x:v>2021-03-18</x:v>
       </x:c>
       <x:c r="R12" s="12" t="str">
         <x:v>exact</x:v>
@@ -26202,13 +26248,13 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="V12" s="105" t="n">
-        <x:v>20711</x:v>
+        <x:v>19730</x:v>
       </x:c>
       <x:c r="W12" s="105" t="n">
-        <x:v>980</x:v>
+        <x:v>954</x:v>
       </x:c>
       <x:c r="X12" s="105" t="n">
-        <x:v>250</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="Y12" s="102" t="n">
         <x:v>46218</x:v>
@@ -26216,19 +26262,19 @@
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>amd-radeon-rx-6800</x:v>
+        <x:v>amd-radeon-rx-6750-xt</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>Radeon RX 6800</x:v>
+        <x:v>Radeon RX 6750 XT</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>AMD Radeon RX 6800</x:v>
+        <x:v>AMD Radeon RX 6750 XT</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>Radeon RX 6800</x:v>
+        <x:v>Radeon RX 6750 XT</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26257,28 +26303,28 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P13" s="102" t="n">
-        <x:v>44153</x:v>
+        <x:v>44691</x:v>
       </x:c>
       <x:c r="Q13" s="12" t="str">
-        <x:v>2020-11-18</x:v>
+        <x:v>2022-05-10</x:v>
       </x:c>
       <x:c r="R13" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S13" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T13" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U13" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V13" s="105" t="n">
-        <x:v>22071</x:v>
+        <x:v>20711</x:v>
       </x:c>
       <x:c r="W13" s="105" t="n">
-        <x:v>1000</x:v>
+        <x:v>980</x:v>
       </x:c>
       <x:c r="X13" s="105" t="n">
         <x:v>250</x:v>
@@ -26289,19 +26335,19 @@
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>amd-radeon-rx-6800-xt</x:v>
+        <x:v>amd-radeon-rx-6800</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>Radeon RX 6800 XT</x:v>
+        <x:v>Radeon RX 6800</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>AMD Radeon RX 6800 XT</x:v>
+        <x:v>AMD Radeon RX 6800</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>Radeon RX 6800 XT</x:v>
+        <x:v>Radeon RX 6800</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26348,13 +26394,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V14" s="105" t="n">
-        <x:v>25067</x:v>
+        <x:v>22071</x:v>
       </x:c>
       <x:c r="W14" s="105" t="n">
-        <x:v>1045</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="X14" s="105" t="n">
-        <x:v>300</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="Y14" s="102" t="n">
         <x:v>46218</x:v>
@@ -26362,19 +26408,19 @@
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>amd-radeon-rx-6900-xt</x:v>
+        <x:v>amd-radeon-rx-6800-xt</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>Radeon RX 6900 XT</x:v>
+        <x:v>Radeon RX 6800 XT</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>AMD Radeon RX 6900 XT</x:v>
+        <x:v>AMD Radeon RX 6800 XT</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>Radeon RX 6900 XT</x:v>
+        <x:v>Radeon RX 6800 XT</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26403,10 +26449,10 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P15" s="102" t="n">
-        <x:v>44173</x:v>
+        <x:v>44153</x:v>
       </x:c>
       <x:c r="Q15" s="12" t="str">
-        <x:v>2020-12-08</x:v>
+        <x:v>2020-11-18</x:v>
       </x:c>
       <x:c r="R15" s="12" t="str">
         <x:v>exact</x:v>
@@ -26421,10 +26467,10 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V15" s="105" t="n">
-        <x:v>26646</x:v>
+        <x:v>25067</x:v>
       </x:c>
       <x:c r="W15" s="105" t="n">
-        <x:v>1063</x:v>
+        <x:v>1045</x:v>
       </x:c>
       <x:c r="X15" s="105" t="n">
         <x:v>300</x:v>
@@ -26435,19 +26481,19 @@
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>amd-radeon-rx-6950-xt</x:v>
+        <x:v>amd-radeon-rx-6900-xt</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>Radeon RX 6950 XT</x:v>
+        <x:v>Radeon RX 6900 XT</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>AMD Radeon RX 6950 XT</x:v>
+        <x:v>AMD Radeon RX 6900 XT</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>Radeon RX 6950 XT</x:v>
+        <x:v>Radeon RX 6900 XT</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26476,10 +26522,10 @@
         <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P16" s="102" t="n">
-        <x:v>44691</x:v>
+        <x:v>44173</x:v>
       </x:c>
       <x:c r="Q16" s="12" t="str">
-        <x:v>2022-05-10</x:v>
+        <x:v>2020-12-08</x:v>
       </x:c>
       <x:c r="R16" s="12" t="str">
         <x:v>exact</x:v>
@@ -26494,13 +26540,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V16" s="105" t="n">
-        <x:v>28076</x:v>
+        <x:v>26646</x:v>
       </x:c>
       <x:c r="W16" s="105" t="n">
-        <x:v>1081</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="X16" s="105" t="n">
-        <x:v>335</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="Y16" s="102" t="n">
         <x:v>46218</x:v>
@@ -26508,19 +26554,19 @@
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>amd-radeon-rx-7600</x:v>
+        <x:v>amd-radeon-rx-6950-xt</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>Radeon RX 7600</x:v>
+        <x:v>Radeon RX 6950 XT</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>AMD Radeon RX 7600</x:v>
+        <x:v>AMD Radeon RX 6950 XT</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>Radeon RX 7600</x:v>
+        <x:v>Radeon RX 6950 XT</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26543,37 +26589,37 @@
         <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N17" s="12" t="str">
-        <x:v>RDNA 3</x:v>
+        <x:v>RDNA 2</x:v>
       </x:c>
       <x:c r="O17" s="12" t="str">
-        <x:v>Radeon RX 7000 Series</x:v>
+        <x:v>Radeon RX 6000 Series</x:v>
       </x:c>
       <x:c r="P17" s="102" t="n">
-        <x:v>45071</x:v>
+        <x:v>44691</x:v>
       </x:c>
       <x:c r="Q17" s="12" t="str">
-        <x:v>2023-05-25</x:v>
+        <x:v>2022-05-10</x:v>
       </x:c>
       <x:c r="R17" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S17" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T17" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U17" s="105" t="n">
-        <x:v>128</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V17" s="105" t="n">
-        <x:v>16463</x:v>
+        <x:v>28076</x:v>
       </x:c>
       <x:c r="W17" s="105" t="n">
-        <x:v>981</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="X17" s="105" t="n">
-        <x:v>165</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="Y17" s="102" t="n">
         <x:v>46218</x:v>
@@ -26581,19 +26627,19 @@
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>amd-radeon-rx-7600-xt</x:v>
+        <x:v>amd-radeon-rx-7600</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>Radeon RX 7600 XT</x:v>
+        <x:v>Radeon RX 7600</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>AMD Radeon RX 7600 XT</x:v>
+        <x:v>AMD Radeon RX 7600</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>Radeon RX 7600 XT</x:v>
+        <x:v>Radeon RX 7600</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26622,16 +26668,16 @@
         <x:v>Radeon RX 7000 Series</x:v>
       </x:c>
       <x:c r="P18" s="102" t="n">
-        <x:v>45315</x:v>
+        <x:v>45071</x:v>
       </x:c>
       <x:c r="Q18" s="12" t="str">
-        <x:v>2024-01-24</x:v>
+        <x:v>2023-05-25</x:v>
       </x:c>
       <x:c r="R18" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S18" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T18" s="12" t="str">
         <x:v>GDDR6</x:v>
@@ -26640,13 +26686,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V18" s="105" t="n">
-        <x:v>17329</x:v>
+        <x:v>16463</x:v>
       </x:c>
       <x:c r="W18" s="105" t="n">
-        <x:v>1027</x:v>
+        <x:v>981</x:v>
       </x:c>
       <x:c r="X18" s="105" t="n">
-        <x:v>190</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="Y18" s="102" t="n">
         <x:v>46218</x:v>
@@ -26654,19 +26700,19 @@
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>amd-radeon-rx-7700-xt</x:v>
+        <x:v>amd-radeon-rx-7600-xt</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>Radeon RX 7700 XT</x:v>
+        <x:v>Radeon RX 7600 XT</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>AMD Radeon RX 7700 XT</x:v>
+        <x:v>AMD Radeon RX 7600 XT</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>Radeon RX 7700 XT</x:v>
+        <x:v>Radeon RX 7600 XT</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26695,31 +26741,31 @@
         <x:v>Radeon RX 7000 Series</x:v>
       </x:c>
       <x:c r="P19" s="102" t="n">
-        <x:v>45175</x:v>
+        <x:v>45315</x:v>
       </x:c>
       <x:c r="Q19" s="12" t="str">
-        <x:v>2023-09-06</x:v>
+        <x:v>2024-01-24</x:v>
       </x:c>
       <x:c r="R19" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S19" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T19" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U19" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="V19" s="105" t="n">
-        <x:v>22692</x:v>
+        <x:v>17329</x:v>
       </x:c>
       <x:c r="W19" s="105" t="n">
-        <x:v>1158</x:v>
+        <x:v>1027</x:v>
       </x:c>
       <x:c r="X19" s="105" t="n">
-        <x:v>245</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="Y19" s="102" t="n">
         <x:v>46218</x:v>
@@ -26727,19 +26773,19 @@
     </x:row>
     <x:row r="20" ht="38" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>amd-radeon-rx-7800-xt</x:v>
+        <x:v>amd-radeon-rx-7700-xt</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>Radeon RX 7800 XT</x:v>
+        <x:v>Radeon RX 7700 XT</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>AMD Radeon RX 7800 XT</x:v>
+        <x:v>AMD Radeon RX 7700 XT</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>Radeon RX 7800 XT</x:v>
+        <x:v>Radeon RX 7700 XT</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26777,22 +26823,22 @@
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S20" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T20" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U20" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V20" s="105" t="n">
-        <x:v>24405</x:v>
+        <x:v>22692</x:v>
       </x:c>
       <x:c r="W20" s="105" t="n">
-        <x:v>1192</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="X20" s="105" t="n">
-        <x:v>263</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="Y20" s="102" t="n">
         <x:v>46218</x:v>
@@ -26800,19 +26846,19 @@
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>amd-radeon-rx-7900-gre</x:v>
+        <x:v>amd-radeon-rx-7800-xt</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C21" s="12" t="str">
-        <x:v>Radeon RX 7900 GRE</x:v>
+        <x:v>Radeon RX 7800 XT</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>AMD Radeon RX 7900 GRE</x:v>
+        <x:v>AMD Radeon RX 7800 XT</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>Radeon RX 7900 GRE</x:v>
+        <x:v>Radeon RX 7800 XT</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26841,10 +26887,10 @@
         <x:v>Radeon RX 7000 Series</x:v>
       </x:c>
       <x:c r="P21" s="102" t="n">
-        <x:v>45349</x:v>
+        <x:v>45175</x:v>
       </x:c>
       <x:c r="Q21" s="12" t="str">
-        <x:v>2024-02-27</x:v>
+        <x:v>2023-09-06</x:v>
       </x:c>
       <x:c r="R21" s="12" t="str">
         <x:v>exact</x:v>
@@ -26859,13 +26905,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V21" s="105" t="n">
-        <x:v>27457</x:v>
+        <x:v>24405</x:v>
       </x:c>
       <x:c r="W21" s="105" t="n">
-        <x:v>1209</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="X21" s="105" t="n">
-        <x:v>260</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="Y21" s="102" t="n">
         <x:v>46218</x:v>
@@ -26873,19 +26919,19 @@
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>amd-radeon-rx-7900-xt</x:v>
+        <x:v>amd-radeon-rx-7900-gre</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>Radeon RX 7900 XT</x:v>
+        <x:v>Radeon RX 7900 GRE</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>AMD Radeon RX 7900 XT</x:v>
+        <x:v>AMD Radeon RX 7900 GRE</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>Radeon RX 7900 XT</x:v>
+        <x:v>Radeon RX 7900 GRE</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26914,31 +26960,31 @@
         <x:v>Radeon RX 7000 Series</x:v>
       </x:c>
       <x:c r="P22" s="102" t="n">
-        <x:v>44908</x:v>
+        <x:v>45349</x:v>
       </x:c>
       <x:c r="Q22" s="12" t="str">
-        <x:v>2022-12-13</x:v>
+        <x:v>2024-02-27</x:v>
       </x:c>
       <x:c r="R22" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S22" s="104" t="n">
-        <x:v>20</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T22" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U22" s="105" t="n">
-        <x:v>320</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V22" s="105" t="n">
-        <x:v>29068</x:v>
+        <x:v>27457</x:v>
       </x:c>
       <x:c r="W22" s="105" t="n">
-        <x:v>1245</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="X22" s="105" t="n">
-        <x:v>315</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="Y22" s="102" t="n">
         <x:v>46218</x:v>
@@ -26946,19 +26992,19 @@
     </x:row>
     <x:row r="23" ht="38" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>amd-radeon-rx-7900-xtx</x:v>
+        <x:v>amd-radeon-rx-7900-xt</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>Radeon RX 7900 XTX</x:v>
+        <x:v>Radeon RX 7900 XT</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>AMD Radeon RX 7900 XTX</x:v>
+        <x:v>AMD Radeon RX 7900 XT</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>Radeon RX 7900 XTX</x:v>
+        <x:v>Radeon RX 7900 XT</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
         <x:v>research_required</x:v>
@@ -26996,22 +27042,22 @@
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S23" s="104" t="n">
-        <x:v>24</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="T23" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U23" s="105" t="n">
-        <x:v>384</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="V23" s="105" t="n">
-        <x:v>31430</x:v>
+        <x:v>29068</x:v>
       </x:c>
       <x:c r="W23" s="105" t="n">
-        <x:v>1288</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="X23" s="105" t="n">
-        <x:v>355</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="Y23" s="102" t="n">
         <x:v>46218</x:v>
@@ -27019,19 +27065,19 @@
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>amd-radeon-rx-9060</x:v>
+        <x:v>amd-radeon-rx-7900-xtx</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>Radeon RX 9060</x:v>
+        <x:v>Radeon RX 7900 XTX</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>AMD Radeon RX 9060</x:v>
+        <x:v>AMD Radeon RX 7900 XTX</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>Radeon RX 9060</x:v>
+        <x:v>Radeon RX 7900 XTX</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27054,35 +27100,37 @@
         <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N24" s="12" t="str">
-        <x:v>RDNA 4</x:v>
+        <x:v>RDNA 3</x:v>
       </x:c>
       <x:c r="O24" s="12" t="str">
-        <x:v>Radeon RX 9000 Series</x:v>
-      </x:c>
-      <x:c r="P24" s="102"/>
+        <x:v>Radeon RX 7000 Series</x:v>
+      </x:c>
+      <x:c r="P24" s="102" t="n">
+        <x:v>44908</x:v>
+      </x:c>
       <x:c r="Q24" s="12" t="str">
-        <x:v>Q3'25</x:v>
+        <x:v>2022-12-13</x:v>
       </x:c>
       <x:c r="R24" s="12" t="str">
-        <x:v>quarter</x:v>
+        <x:v>exact</x:v>
       </x:c>
       <x:c r="S24" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="T24" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U24" s="105" t="n">
-        <x:v>128</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="V24" s="105" t="n">
-        <x:v>17649</x:v>
+        <x:v>31430</x:v>
       </x:c>
       <x:c r="W24" s="105" t="n">
-        <x:v>999</x:v>
+        <x:v>1288</x:v>
       </x:c>
       <x:c r="X24" s="105" t="n">
-        <x:v>132</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="Y24" s="102" t="n">
         <x:v>46218</x:v>
@@ -27090,19 +27138,19 @@
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>amd-radeon-rx-9060-xt-8gb</x:v>
+        <x:v>amd-radeon-rx-9060</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>Radeon RX 9060 XT 8GB</x:v>
+        <x:v>Radeon RX 9060</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>AMD Radeon RX 9060 XT 8GB</x:v>
+        <x:v>AMD Radeon RX 9060</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>Radeon RX 9060 XT 8GB</x:v>
+        <x:v>Radeon RX 9060</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27130,14 +27178,12 @@
       <x:c r="O25" s="12" t="str">
         <x:v>Radeon RX 9000 Series</x:v>
       </x:c>
-      <x:c r="P25" s="102" t="n">
-        <x:v>45813</x:v>
-      </x:c>
+      <x:c r="P25" s="102"/>
       <x:c r="Q25" s="12" t="str">
-        <x:v>2025-06-05</x:v>
+        <x:v>Q3'25</x:v>
       </x:c>
       <x:c r="R25" s="12" t="str">
-        <x:v>exact</x:v>
+        <x:v>quarter</x:v>
       </x:c>
       <x:c r="S25" s="104" t="n">
         <x:v>8</x:v>
@@ -27149,13 +27195,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V25" s="105" t="n">
-        <x:v>19761</x:v>
+        <x:v>17649</x:v>
       </x:c>
       <x:c r="W25" s="105" t="n">
-        <x:v>1125</x:v>
+        <x:v>999</x:v>
       </x:c>
       <x:c r="X25" s="105" t="n">
-        <x:v>150</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="Y25" s="102" t="n">
         <x:v>46218</x:v>
@@ -27163,19 +27209,19 @@
     </x:row>
     <x:row r="26" ht="38" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>amd-radeon-rx-9060-xt-16gb</x:v>
+        <x:v>amd-radeon-rx-9060-xt-8gb</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>Radeon RX 9060 XT 16GB</x:v>
+        <x:v>Radeon RX 9060 XT 8GB</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>AMD Radeon RX 9060 XT 16GB</x:v>
+        <x:v>AMD Radeon RX 9060 XT 8GB</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>Radeon RX 9060 XT 16GB</x:v>
+        <x:v>Radeon RX 9060 XT 8GB</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27213,7 +27259,7 @@
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S26" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T26" s="12" t="str">
         <x:v>GDDR6</x:v>
@@ -27222,13 +27268,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V26" s="105" t="n">
-        <x:v>20081</x:v>
+        <x:v>19761</x:v>
       </x:c>
       <x:c r="W26" s="105" t="n">
-        <x:v>1171</x:v>
+        <x:v>1125</x:v>
       </x:c>
       <x:c r="X26" s="105" t="n">
-        <x:v>160</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="Y26" s="102" t="n">
         <x:v>46218</x:v>
@@ -27236,19 +27282,19 @@
     </x:row>
     <x:row r="27" ht="38" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>amd-radeon-rx-9070</x:v>
+        <x:v>amd-radeon-rx-9060-xt-16gb</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>Radeon RX 9070</x:v>
+        <x:v>Radeon RX 9060 XT 16GB</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>AMD Radeon RX 9070</x:v>
+        <x:v>AMD Radeon RX 9060 XT 16GB</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>Radeon RX 9070</x:v>
+        <x:v>Radeon RX 9060 XT 16GB</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27277,10 +27323,10 @@
         <x:v>Radeon RX 9000 Series</x:v>
       </x:c>
       <x:c r="P27" s="102" t="n">
-        <x:v>45722</x:v>
+        <x:v>45813</x:v>
       </x:c>
       <x:c r="Q27" s="12" t="str">
-        <x:v>2025-03-06</x:v>
+        <x:v>2025-06-05</x:v>
       </x:c>
       <x:c r="R27" s="12" t="str">
         <x:v>exact</x:v>
@@ -27292,16 +27338,16 @@
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U27" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="V27" s="105" t="n">
-        <x:v>25375</x:v>
+        <x:v>20081</x:v>
       </x:c>
       <x:c r="W27" s="105" t="n">
-        <x:v>1265</x:v>
+        <x:v>1171</x:v>
       </x:c>
       <x:c r="X27" s="105" t="n">
-        <x:v>220</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="Y27" s="102" t="n">
         <x:v>46218</x:v>
@@ -27309,19 +27355,19 @@
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>amd-radeon-rx-9070-gre</x:v>
+        <x:v>amd-radeon-rx-9070</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>Radeon RX 9070 GRE</x:v>
+        <x:v>Radeon RX 9070</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>AMD Radeon RX 9070 GRE</x:v>
+        <x:v>AMD Radeon RX 9070</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>Radeon RX 9070 GRE</x:v>
+        <x:v>Radeon RX 9070</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27350,28 +27396,28 @@
         <x:v>Radeon RX 9000 Series</x:v>
       </x:c>
       <x:c r="P28" s="102" t="n">
-        <x:v>46175</x:v>
+        <x:v>45722</x:v>
       </x:c>
       <x:c r="Q28" s="12" t="str">
-        <x:v>2026-06-02</x:v>
+        <x:v>2025-03-06</x:v>
       </x:c>
       <x:c r="R28" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S28" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T28" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U28" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V28" s="105" t="n">
-        <x:v>24257</x:v>
+        <x:v>25375</x:v>
       </x:c>
       <x:c r="W28" s="105" t="n">
-        <x:v>1198</x:v>
+        <x:v>1265</x:v>
       </x:c>
       <x:c r="X28" s="105" t="n">
         <x:v>220</x:v>
@@ -27382,19 +27428,19 @@
     </x:row>
     <x:row r="29" ht="38" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>amd-radeon-rx-9070-xt</x:v>
+        <x:v>amd-radeon-rx-9070-gre</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
         <x:v>AMD</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>Radeon RX 9070 XT</x:v>
+        <x:v>Radeon RX 9070 GRE</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>AMD Radeon RX 9070 XT</x:v>
+        <x:v>AMD Radeon RX 9070 GRE</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>Radeon RX 9070 XT</x:v>
+        <x:v>Radeon RX 9070 GRE</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27423,31 +27469,31 @@
         <x:v>Radeon RX 9000 Series</x:v>
       </x:c>
       <x:c r="P29" s="102" t="n">
-        <x:v>45722</x:v>
+        <x:v>46175</x:v>
       </x:c>
       <x:c r="Q29" s="12" t="str">
-        <x:v>2025-03-06</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="R29" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S29" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T29" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U29" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V29" s="105" t="n">
-        <x:v>26912</x:v>
+        <x:v>24257</x:v>
       </x:c>
       <x:c r="W29" s="105" t="n">
-        <x:v>1315</x:v>
+        <x:v>1198</x:v>
       </x:c>
       <x:c r="X29" s="105" t="n">
-        <x:v>304</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="Y29" s="102" t="n">
         <x:v>46218</x:v>
@@ -27455,20 +27501,19 @@
     </x:row>
     <x:row r="30" ht="38" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2060-6gb</x:v>
+        <x:v>amd-radeon-rx-9070-xt</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>NVIDIA</x:v>
+        <x:v>AMD</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>GeForce RTX 2060 6GB</x:v>
+        <x:v>Radeon RX 9070 XT</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2060 6GB</x:v>
+        <x:v>AMD Radeon RX 9070 XT</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>GeForce RTX 2060 6GB
-GeForce RTX 2060</x:v>
+        <x:v>Radeon RX 9070 XT</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27491,37 +27536,37 @@
         <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N30" s="12" t="str">
-        <x:v>Turing</x:v>
+        <x:v>RDNA 4</x:v>
       </x:c>
       <x:c r="O30" s="12" t="str">
-        <x:v>GeForce RTX 20 Series</x:v>
+        <x:v>Radeon RX 9000 Series</x:v>
       </x:c>
       <x:c r="P30" s="102" t="n">
-        <x:v>43480</x:v>
+        <x:v>45722</x:v>
       </x:c>
       <x:c r="Q30" s="12" t="str">
-        <x:v>2019-01-15</x:v>
+        <x:v>2025-03-06</x:v>
       </x:c>
       <x:c r="R30" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S30" s="104" t="n">
-        <x:v>6</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T30" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U30" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V30" s="105" t="n">
-        <x:v>14090</x:v>
+        <x:v>26912</x:v>
       </x:c>
       <x:c r="W30" s="105" t="n">
-        <x:v>744</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="X30" s="105" t="n">
-        <x:v>160</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="Y30" s="102" t="n">
         <x:v>46218</x:v>
@@ -27529,19 +27574,20 @@
     </x:row>
     <x:row r="31" ht="38" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2060-12gb</x:v>
+        <x:v>nvidia-geforce-rtx-2060-6gb</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>GeForce RTX 2060 12GB</x:v>
+        <x:v>GeForce RTX 2060 6GB</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2060 12GB</x:v>
+        <x:v>NVIDIA GeForce RTX 2060 6GB</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>GeForce RTX 2060 12GB</x:v>
+        <x:v>GeForce RTX 2060 6GB
+GeForce RTX 2060</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27570,16 +27616,16 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P31" s="102" t="n">
-        <x:v>44537</x:v>
+        <x:v>43480</x:v>
       </x:c>
       <x:c r="Q31" s="12" t="str">
-        <x:v>2021-12-07</x:v>
+        <x:v>2019-01-15</x:v>
       </x:c>
       <x:c r="R31" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S31" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="T31" s="12" t="str">
         <x:v>GDDR6</x:v>
@@ -27588,13 +27634,13 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="V31" s="105" t="n">
-        <x:v>15924</x:v>
+        <x:v>14090</x:v>
       </x:c>
       <x:c r="W31" s="105" t="n">
-        <x:v>851</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="X31" s="105" t="n">
-        <x:v>185</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="Y31" s="102" t="n">
         <x:v>46218</x:v>
@@ -27602,19 +27648,19 @@
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2060-super</x:v>
+        <x:v>nvidia-geforce-rtx-2060-12gb</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>GeForce RTX 2060 SUPER</x:v>
+        <x:v>GeForce RTX 2060 12GB</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2060 SUPER</x:v>
+        <x:v>NVIDIA GeForce RTX 2060 12GB</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>GeForce RTX 2060 SUPER</x:v>
+        <x:v>GeForce RTX 2060 12GB</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27643,31 +27689,31 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P32" s="102" t="n">
-        <x:v>43655</x:v>
+        <x:v>44537</x:v>
       </x:c>
       <x:c r="Q32" s="12" t="str">
-        <x:v>2019-07-09</x:v>
+        <x:v>2021-12-07</x:v>
       </x:c>
       <x:c r="R32" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S32" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T32" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U32" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V32" s="105" t="n">
-        <x:v>16469</x:v>
+        <x:v>15924</x:v>
       </x:c>
       <x:c r="W32" s="105" t="n">
-        <x:v>857</x:v>
+        <x:v>851</x:v>
       </x:c>
       <x:c r="X32" s="105" t="n">
-        <x:v>175</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="Y32" s="102" t="n">
         <x:v>46218</x:v>
@@ -27675,19 +27721,19 @@
     </x:row>
     <x:row r="33" ht="38" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2070</x:v>
+        <x:v>nvidia-geforce-rtx-2060-super</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>GeForce RTX 2070</x:v>
+        <x:v>GeForce RTX 2060 SUPER</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2070</x:v>
+        <x:v>NVIDIA GeForce RTX 2060 SUPER</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>GeForce RTX 2070</x:v>
+        <x:v>GeForce RTX 2060 SUPER</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27716,10 +27762,10 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P33" s="102" t="n">
-        <x:v>43390</x:v>
+        <x:v>43655</x:v>
       </x:c>
       <x:c r="Q33" s="12" t="str">
-        <x:v>2018-10-17</x:v>
+        <x:v>2019-07-09</x:v>
       </x:c>
       <x:c r="R33" s="12" t="str">
         <x:v>exact</x:v>
@@ -27734,10 +27780,10 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V33" s="105" t="n">
-        <x:v>16062</x:v>
+        <x:v>16469</x:v>
       </x:c>
       <x:c r="W33" s="105" t="n">
-        <x:v>816</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="X33" s="105" t="n">
         <x:v>175</x:v>
@@ -27748,19 +27794,19 @@
     </x:row>
     <x:row r="34" ht="38" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2070-super</x:v>
+        <x:v>nvidia-geforce-rtx-2070</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>GeForce RTX 2070 SUPER</x:v>
+        <x:v>GeForce RTX 2070</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2070 SUPER</x:v>
+        <x:v>NVIDIA GeForce RTX 2070</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>GeForce RTX 2070 SUPER</x:v>
+        <x:v>GeForce RTX 2070</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27789,10 +27835,10 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P34" s="102" t="n">
-        <x:v>43655</x:v>
+        <x:v>43390</x:v>
       </x:c>
       <x:c r="Q34" s="12" t="str">
-        <x:v>2019-07-09</x:v>
+        <x:v>2018-10-17</x:v>
       </x:c>
       <x:c r="R34" s="12" t="str">
         <x:v>exact</x:v>
@@ -27807,13 +27853,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V34" s="105" t="n">
-        <x:v>18127</x:v>
+        <x:v>16062</x:v>
       </x:c>
       <x:c r="W34" s="105" t="n">
-        <x:v>878</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="X34" s="105" t="n">
-        <x:v>215</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="Y34" s="102" t="n">
         <x:v>46218</x:v>
@@ -27821,19 +27867,19 @@
     </x:row>
     <x:row r="35" ht="38" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2080</x:v>
+        <x:v>nvidia-geforce-rtx-2070-super</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>GeForce RTX 2080</x:v>
+        <x:v>GeForce RTX 2070 SUPER</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2080</x:v>
+        <x:v>NVIDIA GeForce RTX 2070 SUPER</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>GeForce RTX 2080</x:v>
+        <x:v>GeForce RTX 2070 SUPER</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27862,10 +27908,10 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P35" s="102" t="n">
-        <x:v>43363</x:v>
+        <x:v>43655</x:v>
       </x:c>
       <x:c r="Q35" s="12" t="str">
-        <x:v>2018-09-20</x:v>
+        <x:v>2019-07-09</x:v>
       </x:c>
       <x:c r="R35" s="12" t="str">
         <x:v>exact</x:v>
@@ -27880,13 +27926,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V35" s="105" t="n">
-        <x:v>18567</x:v>
+        <x:v>18127</x:v>
       </x:c>
       <x:c r="W35" s="105" t="n">
-        <x:v>897</x:v>
+        <x:v>878</x:v>
       </x:c>
       <x:c r="X35" s="105" t="n">
-        <x:v>250</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="Y35" s="102" t="n">
         <x:v>46218</x:v>
@@ -27894,19 +27940,19 @@
     </x:row>
     <x:row r="36" ht="38" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2080-super</x:v>
+        <x:v>nvidia-geforce-rtx-2080</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>GeForce RTX 2080 SUPER</x:v>
+        <x:v>GeForce RTX 2080</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2080 SUPER</x:v>
+        <x:v>NVIDIA GeForce RTX 2080</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>GeForce RTX 2080 SUPER</x:v>
+        <x:v>GeForce RTX 2080</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
         <x:v>research_required</x:v>
@@ -27935,10 +27981,10 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P36" s="102" t="n">
-        <x:v>43669</x:v>
+        <x:v>43363</x:v>
       </x:c>
       <x:c r="Q36" s="12" t="str">
-        <x:v>2019-07-23</x:v>
+        <x:v>2018-09-20</x:v>
       </x:c>
       <x:c r="R36" s="12" t="str">
         <x:v>exact</x:v>
@@ -27953,10 +27999,10 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V36" s="105" t="n">
-        <x:v>19422</x:v>
+        <x:v>18567</x:v>
       </x:c>
       <x:c r="W36" s="105" t="n">
-        <x:v>918</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="X36" s="105" t="n">
         <x:v>250</x:v>
@@ -27967,19 +28013,19 @@
     </x:row>
     <x:row r="37" ht="38" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-2080-ti</x:v>
+        <x:v>nvidia-geforce-rtx-2080-super</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>GeForce RTX 2080 Ti</x:v>
+        <x:v>GeForce RTX 2080 SUPER</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 2080 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 2080 SUPER</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>GeForce RTX 2080 Ti</x:v>
+        <x:v>GeForce RTX 2080 SUPER</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28008,28 +28054,28 @@
         <x:v>GeForce RTX 20 Series</x:v>
       </x:c>
       <x:c r="P37" s="102" t="n">
-        <x:v>43370</x:v>
+        <x:v>43669</x:v>
       </x:c>
       <x:c r="Q37" s="12" t="str">
-        <x:v>2018-09-27</x:v>
+        <x:v>2019-07-23</x:v>
       </x:c>
       <x:c r="R37" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S37" s="104" t="n">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T37" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U37" s="105" t="n">
-        <x:v>352</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V37" s="105" t="n">
-        <x:v>21434</x:v>
+        <x:v>19422</x:v>
       </x:c>
       <x:c r="W37" s="105" t="n">
-        <x:v>925</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="X37" s="105" t="n">
         <x:v>250</x:v>
@@ -28040,19 +28086,19 @@
     </x:row>
     <x:row r="38" ht="38" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3050-6gb</x:v>
+        <x:v>nvidia-geforce-rtx-2080-ti</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>GeForce RTX 3050 6GB</x:v>
+        <x:v>GeForce RTX 2080 Ti</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3050 6GB</x:v>
+        <x:v>NVIDIA GeForce RTX 2080 Ti</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>GeForce RTX 3050 6GB</x:v>
+        <x:v>GeForce RTX 2080 Ti</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28075,35 +28121,37 @@
         <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N38" s="12" t="str">
-        <x:v>Ampere</x:v>
+        <x:v>Turing</x:v>
       </x:c>
       <x:c r="O38" s="12" t="str">
-        <x:v>GeForce RTX 30 Series</x:v>
-      </x:c>
-      <x:c r="P38" s="102"/>
+        <x:v>GeForce RTX 20 Series</x:v>
+      </x:c>
+      <x:c r="P38" s="102" t="n">
+        <x:v>43370</x:v>
+      </x:c>
       <x:c r="Q38" s="12" t="str">
-        <x:v>2024-02</x:v>
+        <x:v>2018-09-27</x:v>
       </x:c>
       <x:c r="R38" s="12" t="str">
-        <x:v>month</x:v>
+        <x:v>exact</x:v>
       </x:c>
       <x:c r="S38" s="104" t="n">
-        <x:v>6</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="T38" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U38" s="105" t="n">
-        <x:v>96</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="V38" s="105" t="n">
-        <x:v>10743</x:v>
+        <x:v>21434</x:v>
       </x:c>
       <x:c r="W38" s="105" t="n">
-        <x:v>882</x:v>
+        <x:v>925</x:v>
       </x:c>
       <x:c r="X38" s="105" t="n">
-        <x:v>70</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="Y38" s="102" t="n">
         <x:v>46218</x:v>
@@ -28111,19 +28159,19 @@
     </x:row>
     <x:row r="39" ht="38" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3050-8gb</x:v>
+        <x:v>nvidia-geforce-rtx-3050-6gb</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>GeForce RTX 3050 8GB</x:v>
+        <x:v>GeForce RTX 3050 6GB</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3050 8GB</x:v>
+        <x:v>NVIDIA GeForce RTX 3050 6GB</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>GeForce RTX 3050 8GB</x:v>
+        <x:v>GeForce RTX 3050 6GB</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28151,32 +28199,30 @@
       <x:c r="O39" s="12" t="str">
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
-      <x:c r="P39" s="102" t="n">
-        <x:v>44588</x:v>
-      </x:c>
+      <x:c r="P39" s="102"/>
       <x:c r="Q39" s="12" t="str">
-        <x:v>2022-01-27</x:v>
+        <x:v>2024-02</x:v>
       </x:c>
       <x:c r="R39" s="12" t="str">
-        <x:v>exact</x:v>
+        <x:v>month</x:v>
       </x:c>
       <x:c r="S39" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="T39" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U39" s="105" t="n">
-        <x:v>128</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="V39" s="105" t="n">
-        <x:v>12485</x:v>
+        <x:v>10743</x:v>
       </x:c>
       <x:c r="W39" s="105" t="n">
-        <x:v>918</x:v>
+        <x:v>882</x:v>
       </x:c>
       <x:c r="X39" s="105" t="n">
-        <x:v>130</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="Y39" s="102" t="n">
         <x:v>46218</x:v>
@@ -28184,19 +28230,19 @@
     </x:row>
     <x:row r="40" ht="38" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3060-8gb</x:v>
+        <x:v>nvidia-geforce-rtx-3050-8gb</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str">
-        <x:v>GeForce RTX 3060 8GB</x:v>
+        <x:v>GeForce RTX 3050 8GB</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3060 8GB</x:v>
+        <x:v>NVIDIA GeForce RTX 3050 8GB</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>GeForce RTX 3060 8GB</x:v>
+        <x:v>GeForce RTX 3050 8GB</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28224,12 +28270,14 @@
       <x:c r="O40" s="12" t="str">
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
-      <x:c r="P40" s="102"/>
+      <x:c r="P40" s="102" t="n">
+        <x:v>44588</x:v>
+      </x:c>
       <x:c r="Q40" s="12" t="str">
-        <x:v>Q4'22</x:v>
+        <x:v>2022-01-27</x:v>
       </x:c>
       <x:c r="R40" s="12" t="str">
-        <x:v>quarter</x:v>
+        <x:v>exact</x:v>
       </x:c>
       <x:c r="S40" s="104" t="n">
         <x:v>8</x:v>
@@ -28241,13 +28289,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V40" s="105" t="n">
-        <x:v>15203</x:v>
+        <x:v>12485</x:v>
       </x:c>
       <x:c r="W40" s="105" t="n">
-        <x:v>974</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="X40" s="105" t="n">
-        <x:v>170</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="Y40" s="102" t="n">
         <x:v>46218</x:v>
@@ -28255,19 +28303,19 @@
     </x:row>
     <x:row r="41" ht="38" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3060-12gb</x:v>
+        <x:v>nvidia-geforce-rtx-3060-8gb</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str">
-        <x:v>GeForce RTX 3060 12GB</x:v>
+        <x:v>GeForce RTX 3060 8GB</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3060 12GB</x:v>
+        <x:v>NVIDIA GeForce RTX 3060 8GB</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>GeForce RTX 3060 12GB</x:v>
+        <x:v>GeForce RTX 3060 8GB</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28295,29 +28343,27 @@
       <x:c r="O41" s="12" t="str">
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
-      <x:c r="P41" s="102" t="n">
-        <x:v>44252</x:v>
-      </x:c>
+      <x:c r="P41" s="102"/>
       <x:c r="Q41" s="12" t="str">
-        <x:v>2021-02-25</x:v>
+        <x:v>Q4'22</x:v>
       </x:c>
       <x:c r="R41" s="12" t="str">
-        <x:v>exact</x:v>
+        <x:v>quarter</x:v>
       </x:c>
       <x:c r="S41" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T41" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U41" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="V41" s="105" t="n">
-        <x:v>16716</x:v>
+        <x:v>15203</x:v>
       </x:c>
       <x:c r="W41" s="105" t="n">
-        <x:v>965</x:v>
+        <x:v>974</x:v>
       </x:c>
       <x:c r="X41" s="105" t="n">
         <x:v>170</x:v>
@@ -28328,19 +28374,19 @@
     </x:row>
     <x:row r="42" ht="38" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3060-ti</x:v>
+        <x:v>nvidia-geforce-rtx-3060-12gb</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str">
-        <x:v>GeForce RTX 3060 Ti</x:v>
+        <x:v>GeForce RTX 3060 12GB</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3060 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 3060 12GB</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>GeForce RTX 3060 Ti</x:v>
+        <x:v>GeForce RTX 3060 12GB</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28369,31 +28415,31 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P42" s="102" t="n">
-        <x:v>44167</x:v>
+        <x:v>44252</x:v>
       </x:c>
       <x:c r="Q42" s="12" t="str">
-        <x:v>2020-12-02</x:v>
+        <x:v>2021-02-25</x:v>
       </x:c>
       <x:c r="R42" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S42" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T42" s="12" t="str">
         <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U42" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V42" s="105" t="n">
-        <x:v>20240</x:v>
+        <x:v>16716</x:v>
       </x:c>
       <x:c r="W42" s="105" t="n">
-        <x:v>989</x:v>
+        <x:v>965</x:v>
       </x:c>
       <x:c r="X42" s="105" t="n">
-        <x:v>200</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="Y42" s="102" t="n">
         <x:v>46218</x:v>
@@ -28401,19 +28447,19 @@
     </x:row>
     <x:row r="43" ht="38" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3070</x:v>
+        <x:v>nvidia-geforce-rtx-3060-ti</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
-        <x:v>GeForce RTX 3070</x:v>
+        <x:v>GeForce RTX 3060 Ti</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3070</x:v>
+        <x:v>NVIDIA GeForce RTX 3060 Ti</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>GeForce RTX 3070</x:v>
+        <x:v>GeForce RTX 3060 Ti</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28442,10 +28488,10 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P43" s="102" t="n">
-        <x:v>44133</x:v>
+        <x:v>44167</x:v>
       </x:c>
       <x:c r="Q43" s="12" t="str">
-        <x:v>2020-10-29</x:v>
+        <x:v>2020-12-02</x:v>
       </x:c>
       <x:c r="R43" s="12" t="str">
         <x:v>exact</x:v>
@@ -28460,13 +28506,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V43" s="105" t="n">
-        <x:v>22095</x:v>
+        <x:v>20240</x:v>
       </x:c>
       <x:c r="W43" s="105" t="n">
-        <x:v>1005</x:v>
+        <x:v>989</x:v>
       </x:c>
       <x:c r="X43" s="105" t="n">
-        <x:v>220</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="Y43" s="102" t="n">
         <x:v>46218</x:v>
@@ -28474,19 +28520,19 @@
     </x:row>
     <x:row r="44" ht="38" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3070-ti</x:v>
+        <x:v>nvidia-geforce-rtx-3070</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
-        <x:v>GeForce RTX 3070 Ti</x:v>
+        <x:v>GeForce RTX 3070</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3070 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 3070</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>GeForce RTX 3070 Ti</x:v>
+        <x:v>GeForce RTX 3070</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28515,10 +28561,10 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P44" s="102" t="n">
-        <x:v>44357</x:v>
+        <x:v>44133</x:v>
       </x:c>
       <x:c r="Q44" s="12" t="str">
-        <x:v>2021-06-10</x:v>
+        <x:v>2020-10-29</x:v>
       </x:c>
       <x:c r="R44" s="12" t="str">
         <x:v>exact</x:v>
@@ -28527,19 +28573,19 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="T44" s="12" t="str">
-        <x:v>GDDR6X</x:v>
+        <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U44" s="105" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="V44" s="105" t="n">
-        <x:v>23196</x:v>
+        <x:v>22095</x:v>
       </x:c>
       <x:c r="W44" s="105" t="n">
-        <x:v>1058</x:v>
+        <x:v>1005</x:v>
       </x:c>
       <x:c r="X44" s="105" t="n">
-        <x:v>290</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="Y44" s="102" t="n">
         <x:v>46218</x:v>
@@ -28547,19 +28593,19 @@
     </x:row>
     <x:row r="45" ht="38" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3080</x:v>
+        <x:v>nvidia-geforce-rtx-3070-ti</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str">
-        <x:v>GeForce RTX 3080</x:v>
+        <x:v>GeForce RTX 3070 Ti</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3080</x:v>
+        <x:v>NVIDIA GeForce RTX 3070 Ti</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>GeForce RTX 3080</x:v>
+        <x:v>GeForce RTX 3070 Ti</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28588,31 +28634,31 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P45" s="102" t="n">
-        <x:v>44091</x:v>
+        <x:v>44357</x:v>
       </x:c>
       <x:c r="Q45" s="12" t="str">
-        <x:v>2020-09-17</x:v>
+        <x:v>2021-06-10</x:v>
       </x:c>
       <x:c r="R45" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S45" s="104" t="n">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T45" s="12" t="str">
         <x:v>GDDR6X</x:v>
       </x:c>
       <x:c r="U45" s="105" t="n">
-        <x:v>320</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V45" s="105" t="n">
-        <x:v>25001</x:v>
+        <x:v>23196</x:v>
       </x:c>
       <x:c r="W45" s="105" t="n">
-        <x:v>1062</x:v>
+        <x:v>1058</x:v>
       </x:c>
       <x:c r="X45" s="105" t="n">
-        <x:v>320</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="Y45" s="102" t="n">
         <x:v>46218</x:v>
@@ -28620,19 +28666,19 @@
     </x:row>
     <x:row r="46" ht="38" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3080-12gb</x:v>
+        <x:v>nvidia-geforce-rtx-3080</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
-        <x:v>GeForce RTX 3080 12GB</x:v>
+        <x:v>GeForce RTX 3080</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3080 12GB</x:v>
+        <x:v>NVIDIA GeForce RTX 3080</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>GeForce RTX 3080 12GB</x:v>
+        <x:v>GeForce RTX 3080</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28661,31 +28707,31 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P46" s="102" t="n">
-        <x:v>44572</x:v>
+        <x:v>44091</x:v>
       </x:c>
       <x:c r="Q46" s="12" t="str">
-        <x:v>2022-01-11</x:v>
+        <x:v>2020-09-17</x:v>
       </x:c>
       <x:c r="R46" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S46" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T46" s="12" t="str">
         <x:v>GDDR6X</x:v>
       </x:c>
       <x:c r="U46" s="105" t="n">
-        <x:v>384</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="V46" s="105" t="n">
-        <x:v>26559</x:v>
+        <x:v>25001</x:v>
       </x:c>
       <x:c r="W46" s="105" t="n">
-        <x:v>1095</x:v>
+        <x:v>1062</x:v>
       </x:c>
       <x:c r="X46" s="105" t="n">
-        <x:v>350</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="Y46" s="102" t="n">
         <x:v>46218</x:v>
@@ -28693,19 +28739,19 @@
     </x:row>
     <x:row r="47" ht="38" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3080-ti</x:v>
+        <x:v>nvidia-geforce-rtx-3080-12gb</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str">
-        <x:v>GeForce RTX 3080 Ti</x:v>
+        <x:v>GeForce RTX 3080 12GB</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3080 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 3080 12GB</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>GeForce RTX 3080 Ti</x:v>
+        <x:v>GeForce RTX 3080 12GB</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28734,10 +28780,10 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P47" s="102" t="n">
-        <x:v>44350</x:v>
+        <x:v>44572</x:v>
       </x:c>
       <x:c r="Q47" s="12" t="str">
-        <x:v>2021-06-03</x:v>
+        <x:v>2022-01-11</x:v>
       </x:c>
       <x:c r="R47" s="12" t="str">
         <x:v>exact</x:v>
@@ -28752,7 +28798,7 @@
         <x:v>384</x:v>
       </x:c>
       <x:c r="V47" s="105" t="n">
-        <x:v>26750</x:v>
+        <x:v>26559</x:v>
       </x:c>
       <x:c r="W47" s="105" t="n">
         <x:v>1095</x:v>
@@ -28766,19 +28812,19 @@
     </x:row>
     <x:row r="48" ht="38" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3090</x:v>
+        <x:v>nvidia-geforce-rtx-3080-ti</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
-        <x:v>GeForce RTX 3090</x:v>
+        <x:v>GeForce RTX 3080 Ti</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3090</x:v>
+        <x:v>NVIDIA GeForce RTX 3080 Ti</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>GeForce RTX 3090</x:v>
+        <x:v>GeForce RTX 3080 Ti</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28807,16 +28853,16 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P48" s="102" t="n">
-        <x:v>44098</x:v>
+        <x:v>44350</x:v>
       </x:c>
       <x:c r="Q48" s="12" t="str">
-        <x:v>2020-09-24</x:v>
+        <x:v>2021-06-03</x:v>
       </x:c>
       <x:c r="R48" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S48" s="104" t="n">
-        <x:v>24</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T48" s="12" t="str">
         <x:v>GDDR6X</x:v>
@@ -28825,10 +28871,10 @@
         <x:v>384</x:v>
       </x:c>
       <x:c r="V48" s="105" t="n">
-        <x:v>26518</x:v>
+        <x:v>26750</x:v>
       </x:c>
       <x:c r="W48" s="105" t="n">
-        <x:v>1069</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="X48" s="105" t="n">
         <x:v>350</x:v>
@@ -28839,19 +28885,19 @@
     </x:row>
     <x:row r="49" ht="38" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-3090-ti</x:v>
+        <x:v>nvidia-geforce-rtx-3090</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
-        <x:v>GeForce RTX 3090 Ti</x:v>
+        <x:v>GeForce RTX 3090</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 3090 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 3090</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>GeForce RTX 3090 Ti</x:v>
+        <x:v>GeForce RTX 3090</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28880,10 +28926,10 @@
         <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P49" s="102" t="n">
-        <x:v>44649</x:v>
+        <x:v>44098</x:v>
       </x:c>
       <x:c r="Q49" s="12" t="str">
-        <x:v>2022-03-29</x:v>
+        <x:v>2020-09-24</x:v>
       </x:c>
       <x:c r="R49" s="12" t="str">
         <x:v>exact</x:v>
@@ -28898,13 +28944,13 @@
         <x:v>384</x:v>
       </x:c>
       <x:c r="V49" s="105" t="n">
-        <x:v>29272</x:v>
+        <x:v>26518</x:v>
       </x:c>
       <x:c r="W49" s="105" t="n">
-        <x:v>1226</x:v>
+        <x:v>1069</x:v>
       </x:c>
       <x:c r="X49" s="105" t="n">
-        <x:v>450</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="Y49" s="102" t="n">
         <x:v>46218</x:v>
@@ -28912,19 +28958,19 @@
     </x:row>
     <x:row r="50" ht="38" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4060</x:v>
+        <x:v>nvidia-geforce-rtx-3090-ti</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
-        <x:v>GeForce RTX 4060</x:v>
+        <x:v>GeForce RTX 3090 Ti</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4060</x:v>
+        <x:v>NVIDIA GeForce RTX 3090 Ti</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>GeForce RTX 4060</x:v>
+        <x:v>GeForce RTX 3090 Ti</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
         <x:v>research_required</x:v>
@@ -28947,37 +28993,37 @@
         <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N50" s="12" t="str">
-        <x:v>Ada Lovelace</x:v>
+        <x:v>Ampere</x:v>
       </x:c>
       <x:c r="O50" s="12" t="str">
-        <x:v>GeForce RTX 40 Series</x:v>
+        <x:v>GeForce RTX 30 Series</x:v>
       </x:c>
       <x:c r="P50" s="102" t="n">
-        <x:v>45106</x:v>
+        <x:v>44649</x:v>
       </x:c>
       <x:c r="Q50" s="12" t="str">
-        <x:v>2023-06-29</x:v>
+        <x:v>2022-03-29</x:v>
       </x:c>
       <x:c r="R50" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S50" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="T50" s="12" t="str">
-        <x:v>GDDR6</x:v>
+        <x:v>GDDR6X</x:v>
       </x:c>
       <x:c r="U50" s="105" t="n">
-        <x:v>128</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="V50" s="105" t="n">
-        <x:v>19494</x:v>
+        <x:v>29272</x:v>
       </x:c>
       <x:c r="W50" s="105" t="n">
-        <x:v>1037</x:v>
+        <x:v>1226</x:v>
       </x:c>
       <x:c r="X50" s="105" t="n">
-        <x:v>115</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="Y50" s="102" t="n">
         <x:v>46218</x:v>
@@ -28985,20 +29031,19 @@
     </x:row>
     <x:row r="51" ht="38" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4060-ti-8gb</x:v>
+        <x:v>nvidia-geforce-rtx-4060</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C51" s="12" t="str">
-        <x:v>GeForce RTX 4060 Ti 8GB</x:v>
+        <x:v>GeForce RTX 4060</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4060 Ti 8GB</x:v>
+        <x:v>NVIDIA GeForce RTX 4060</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>GeForce RTX 4060 Ti 8GB
-GeForce RTX 4060 Ti</x:v>
+        <x:v>GeForce RTX 4060</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29027,10 +29072,10 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P51" s="102" t="n">
-        <x:v>45070</x:v>
+        <x:v>45106</x:v>
       </x:c>
       <x:c r="Q51" s="12" t="str">
-        <x:v>2023-05-24</x:v>
+        <x:v>2023-06-29</x:v>
       </x:c>
       <x:c r="R51" s="12" t="str">
         <x:v>exact</x:v>
@@ -29045,13 +29090,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V51" s="105" t="n">
-        <x:v>22603</x:v>
+        <x:v>19494</x:v>
       </x:c>
       <x:c r="W51" s="105" t="n">
-        <x:v>1095</x:v>
+        <x:v>1037</x:v>
       </x:c>
       <x:c r="X51" s="105" t="n">
-        <x:v>160</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="Y51" s="102" t="n">
         <x:v>46218</x:v>
@@ -29059,19 +29104,20 @@
     </x:row>
     <x:row r="52" ht="38" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4060-ti-16gb</x:v>
+        <x:v>nvidia-geforce-rtx-4060-ti-8gb</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
-        <x:v>GeForce RTX 4060 Ti 16GB</x:v>
+        <x:v>GeForce RTX 4060 Ti 8GB</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4060 Ti 16GB</x:v>
+        <x:v>NVIDIA GeForce RTX 4060 Ti 8GB</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>GeForce RTX 4060 Ti 16GB</x:v>
+        <x:v>GeForce RTX 4060 Ti 8GB
+GeForce RTX 4060 Ti</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29100,16 +29146,16 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P52" s="102" t="n">
-        <x:v>45125</x:v>
+        <x:v>45070</x:v>
       </x:c>
       <x:c r="Q52" s="12" t="str">
-        <x:v>2023-07-18</x:v>
+        <x:v>2023-05-24</x:v>
       </x:c>
       <x:c r="R52" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S52" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T52" s="12" t="str">
         <x:v>GDDR6</x:v>
@@ -29118,13 +29164,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V52" s="105" t="n">
-        <x:v>22592</x:v>
+        <x:v>22603</x:v>
       </x:c>
       <x:c r="W52" s="105" t="n">
-        <x:v>1079</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="X52" s="105" t="n">
-        <x:v>165</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="Y52" s="102" t="n">
         <x:v>46218</x:v>
@@ -29132,19 +29178,19 @@
     </x:row>
     <x:row r="53" ht="38" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4070</x:v>
+        <x:v>nvidia-geforce-rtx-4060-ti-16gb</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
-        <x:v>GeForce RTX 4070</x:v>
+        <x:v>GeForce RTX 4060 Ti 16GB</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4070</x:v>
+        <x:v>NVIDIA GeForce RTX 4060 Ti 16GB</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>GeForce RTX 4070</x:v>
+        <x:v>GeForce RTX 4060 Ti 16GB</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29173,31 +29219,31 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P53" s="102" t="n">
-        <x:v>45029</x:v>
+        <x:v>45125</x:v>
       </x:c>
       <x:c r="Q53" s="12" t="str">
-        <x:v>2023-04-13</x:v>
+        <x:v>2023-07-18</x:v>
       </x:c>
       <x:c r="R53" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S53" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T53" s="12" t="str">
-        <x:v>GDDR6X</x:v>
+        <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U53" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="V53" s="105" t="n">
-        <x:v>26880</x:v>
+        <x:v>22592</x:v>
       </x:c>
       <x:c r="W53" s="105" t="n">
-        <x:v>1167</x:v>
+        <x:v>1079</x:v>
       </x:c>
       <x:c r="X53" s="105" t="n">
-        <x:v>200</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="Y53" s="102" t="n">
         <x:v>46218</x:v>
@@ -29205,19 +29251,19 @@
     </x:row>
     <x:row r="54" ht="38" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4070-super</x:v>
+        <x:v>nvidia-geforce-rtx-4070</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C54" s="12" t="str">
-        <x:v>GeForce RTX 4070 SUPER</x:v>
+        <x:v>GeForce RTX 4070</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4070 SUPER</x:v>
+        <x:v>NVIDIA GeForce RTX 4070</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>GeForce RTX 4070 SUPER</x:v>
+        <x:v>GeForce RTX 4070</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29246,10 +29292,10 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P54" s="102" t="n">
-        <x:v>45308</x:v>
+        <x:v>45029</x:v>
       </x:c>
       <x:c r="Q54" s="12" t="str">
-        <x:v>2024-01-17</x:v>
+        <x:v>2023-04-13</x:v>
       </x:c>
       <x:c r="R54" s="12" t="str">
         <x:v>exact</x:v>
@@ -29264,13 +29310,13 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="V54" s="105" t="n">
-        <x:v>29944</x:v>
+        <x:v>26880</x:v>
       </x:c>
       <x:c r="W54" s="105" t="n">
-        <x:v>1192</x:v>
+        <x:v>1167</x:v>
       </x:c>
       <x:c r="X54" s="105" t="n">
-        <x:v>220</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="Y54" s="102" t="n">
         <x:v>46218</x:v>
@@ -29278,19 +29324,19 @@
     </x:row>
     <x:row r="55" ht="38" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4070-ti</x:v>
+        <x:v>nvidia-geforce-rtx-4070-super</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>GeForce RTX 4070 Ti</x:v>
+        <x:v>GeForce RTX 4070 SUPER</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4070 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 4070 SUPER</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>GeForce RTX 4070 Ti</x:v>
+        <x:v>GeForce RTX 4070 SUPER</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29319,10 +29365,10 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P55" s="102" t="n">
-        <x:v>44931</x:v>
+        <x:v>45308</x:v>
       </x:c>
       <x:c r="Q55" s="12" t="str">
-        <x:v>2023-01-05</x:v>
+        <x:v>2024-01-17</x:v>
       </x:c>
       <x:c r="R55" s="12" t="str">
         <x:v>exact</x:v>
@@ -29337,13 +29383,13 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="V55" s="105" t="n">
-        <x:v>31540</x:v>
+        <x:v>29944</x:v>
       </x:c>
       <x:c r="W55" s="105" t="n">
-        <x:v>1209</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="X55" s="105" t="n">
-        <x:v>285</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="Y55" s="102" t="n">
         <x:v>46218</x:v>
@@ -29351,19 +29397,19 @@
     </x:row>
     <x:row r="56" ht="38" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4070-ti-super</x:v>
+        <x:v>nvidia-geforce-rtx-4070-ti</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>GeForce RTX 4070 Ti SUPER</x:v>
+        <x:v>GeForce RTX 4070 Ti</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4070 Ti SUPER</x:v>
+        <x:v>NVIDIA GeForce RTX 4070 Ti</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>GeForce RTX 4070 Ti SUPER</x:v>
+        <x:v>GeForce RTX 4070 Ti</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29392,28 +29438,28 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P56" s="102" t="n">
-        <x:v>45315</x:v>
+        <x:v>44931</x:v>
       </x:c>
       <x:c r="Q56" s="12" t="str">
-        <x:v>2024-01-24</x:v>
+        <x:v>2023-01-05</x:v>
       </x:c>
       <x:c r="R56" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S56" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T56" s="12" t="str">
         <x:v>GDDR6X</x:v>
       </x:c>
       <x:c r="U56" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V56" s="105" t="n">
-        <x:v>31851</x:v>
+        <x:v>31540</x:v>
       </x:c>
       <x:c r="W56" s="105" t="n">
-        <x:v>1246</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="X56" s="105" t="n">
         <x:v>285</x:v>
@@ -29424,19 +29470,19 @@
     </x:row>
     <x:row r="57" ht="38" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4080</x:v>
+        <x:v>nvidia-geforce-rtx-4070-ti-super</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C57" s="12" t="str">
-        <x:v>GeForce RTX 4080</x:v>
+        <x:v>GeForce RTX 4070 Ti SUPER</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4080</x:v>
+        <x:v>NVIDIA GeForce RTX 4070 Ti SUPER</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>GeForce RTX 4080</x:v>
+        <x:v>GeForce RTX 4070 Ti SUPER</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29465,10 +29511,10 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P57" s="102" t="n">
-        <x:v>44881</x:v>
+        <x:v>45315</x:v>
       </x:c>
       <x:c r="Q57" s="12" t="str">
-        <x:v>2022-11-16</x:v>
+        <x:v>2024-01-24</x:v>
       </x:c>
       <x:c r="R57" s="12" t="str">
         <x:v>exact</x:v>
@@ -29483,13 +29529,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V57" s="105" t="n">
-        <x:v>34447</x:v>
+        <x:v>31851</x:v>
       </x:c>
       <x:c r="W57" s="105" t="n">
-        <x:v>1250</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="X57" s="105" t="n">
-        <x:v>320</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="Y57" s="102" t="n">
         <x:v>46218</x:v>
@@ -29497,19 +29543,19 @@
     </x:row>
     <x:row r="58" ht="38" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4080-super</x:v>
+        <x:v>nvidia-geforce-rtx-4080</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
-        <x:v>GeForce RTX 4080 SUPER</x:v>
+        <x:v>GeForce RTX 4080</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4080 SUPER</x:v>
+        <x:v>NVIDIA GeForce RTX 4080</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>GeForce RTX 4080 SUPER</x:v>
+        <x:v>GeForce RTX 4080</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29538,10 +29584,10 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P58" s="102" t="n">
-        <x:v>45322</x:v>
+        <x:v>44881</x:v>
       </x:c>
       <x:c r="Q58" s="12" t="str">
-        <x:v>2024-01-31</x:v>
+        <x:v>2022-11-16</x:v>
       </x:c>
       <x:c r="R58" s="12" t="str">
         <x:v>exact</x:v>
@@ -29556,10 +29602,10 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V58" s="105" t="n">
-        <x:v>34237</x:v>
+        <x:v>34447</x:v>
       </x:c>
       <x:c r="W58" s="105" t="n">
-        <x:v>1279</x:v>
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="X58" s="105" t="n">
         <x:v>320</x:v>
@@ -29570,19 +29616,19 @@
     </x:row>
     <x:row r="59" ht="38" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-4090</x:v>
+        <x:v>nvidia-geforce-rtx-4080-super</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
-        <x:v>GeForce RTX 4090</x:v>
+        <x:v>GeForce RTX 4080 SUPER</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 4090</x:v>
+        <x:v>NVIDIA GeForce RTX 4080 SUPER</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>GeForce RTX 4090</x:v>
+        <x:v>GeForce RTX 4080 SUPER</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29611,31 +29657,31 @@
         <x:v>GeForce RTX 40 Series</x:v>
       </x:c>
       <x:c r="P59" s="102" t="n">
-        <x:v>44846</x:v>
+        <x:v>45322</x:v>
       </x:c>
       <x:c r="Q59" s="12" t="str">
-        <x:v>2022-10-12</x:v>
+        <x:v>2024-01-31</x:v>
       </x:c>
       <x:c r="R59" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S59" s="104" t="n">
-        <x:v>24</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T59" s="12" t="str">
         <x:v>GDDR6X</x:v>
       </x:c>
       <x:c r="U59" s="105" t="n">
-        <x:v>384</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V59" s="105" t="n">
-        <x:v>38054</x:v>
+        <x:v>34237</x:v>
       </x:c>
       <x:c r="W59" s="105" t="n">
-        <x:v>1303</x:v>
+        <x:v>1279</x:v>
       </x:c>
       <x:c r="X59" s="105" t="n">
-        <x:v>450</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="Y59" s="102" t="n">
         <x:v>46218</x:v>
@@ -29643,19 +29689,19 @@
     </x:row>
     <x:row r="60" ht="38" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5050</x:v>
+        <x:v>nvidia-geforce-rtx-4090</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
-        <x:v>GeForce RTX 5050</x:v>
+        <x:v>GeForce RTX 4090</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5050</x:v>
+        <x:v>NVIDIA GeForce RTX 4090</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>GeForce RTX 5050</x:v>
+        <x:v>GeForce RTX 4090</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29678,35 +29724,37 @@
         <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
       </x:c>
       <x:c r="N60" s="12" t="str">
-        <x:v>Blackwell</x:v>
+        <x:v>Ada Lovelace</x:v>
       </x:c>
       <x:c r="O60" s="12" t="str">
-        <x:v>GeForce RTX 50 Series</x:v>
-      </x:c>
-      <x:c r="P60" s="102"/>
+        <x:v>GeForce RTX 40 Series</x:v>
+      </x:c>
+      <x:c r="P60" s="102" t="n">
+        <x:v>44846</x:v>
+      </x:c>
       <x:c r="Q60" s="12" t="str">
-        <x:v>2025-07</x:v>
+        <x:v>2022-10-12</x:v>
       </x:c>
       <x:c r="R60" s="12" t="str">
-        <x:v>month</x:v>
+        <x:v>exact</x:v>
       </x:c>
       <x:c r="S60" s="104" t="n">
-        <x:v>8</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="T60" s="12" t="str">
-        <x:v>GDDR6</x:v>
+        <x:v>GDDR6X</x:v>
       </x:c>
       <x:c r="U60" s="105" t="n">
-        <x:v>128</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="V60" s="105" t="n">
-        <x:v>16954</x:v>
+        <x:v>38054</x:v>
       </x:c>
       <x:c r="W60" s="105" t="n">
-        <x:v>1070</x:v>
+        <x:v>1303</x:v>
       </x:c>
       <x:c r="X60" s="105" t="n">
-        <x:v>130</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="Y60" s="102" t="n">
         <x:v>46218</x:v>
@@ -29714,19 +29762,19 @@
     </x:row>
     <x:row r="61" ht="38" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5060</x:v>
+        <x:v>nvidia-geforce-rtx-5050</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C61" s="12" t="str">
-        <x:v>GeForce RTX 5060</x:v>
+        <x:v>GeForce RTX 5050</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5060</x:v>
+        <x:v>NVIDIA GeForce RTX 5050</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>GeForce RTX 5060</x:v>
+        <x:v>GeForce RTX 5050</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29754,32 +29802,30 @@
       <x:c r="O61" s="12" t="str">
         <x:v>GeForce RTX 50 Series</x:v>
       </x:c>
-      <x:c r="P61" s="102" t="n">
-        <x:v>45796</x:v>
-      </x:c>
+      <x:c r="P61" s="102"/>
       <x:c r="Q61" s="12" t="str">
-        <x:v>2025-05-19</x:v>
+        <x:v>2025-07</x:v>
       </x:c>
       <x:c r="R61" s="12" t="str">
-        <x:v>exact</x:v>
+        <x:v>month</x:v>
       </x:c>
       <x:c r="S61" s="104" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="T61" s="12" t="str">
-        <x:v>GDDR7</x:v>
+        <x:v>GDDR6</x:v>
       </x:c>
       <x:c r="U61" s="105" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="V61" s="105" t="n">
-        <x:v>20692</x:v>
+        <x:v>16954</x:v>
       </x:c>
       <x:c r="W61" s="105" t="n">
-        <x:v>1150</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="X61" s="105" t="n">
-        <x:v>170</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="Y61" s="102" t="n">
         <x:v>46218</x:v>
@@ -29787,19 +29833,19 @@
     </x:row>
     <x:row r="62" ht="38" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5060-ti-8gb</x:v>
+        <x:v>nvidia-geforce-rtx-5060</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>GeForce RTX 5060 Ti 8GB</x:v>
+        <x:v>GeForce RTX 5060</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5060 Ti 8GB</x:v>
+        <x:v>NVIDIA GeForce RTX 5060</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
-        <x:v>GeForce RTX 5060 Ti 8GB</x:v>
+        <x:v>GeForce RTX 5060</x:v>
       </x:c>
       <x:c r="F62" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29828,10 +29874,10 @@
         <x:v>GeForce RTX 50 Series</x:v>
       </x:c>
       <x:c r="P62" s="102" t="n">
-        <x:v>45763</x:v>
+        <x:v>45796</x:v>
       </x:c>
       <x:c r="Q62" s="12" t="str">
-        <x:v>2025-04-16</x:v>
+        <x:v>2025-05-19</x:v>
       </x:c>
       <x:c r="R62" s="12" t="str">
         <x:v>exact</x:v>
@@ -29846,13 +29892,13 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V62" s="105" t="n">
-        <x:v>22067</x:v>
+        <x:v>20692</x:v>
       </x:c>
       <x:c r="W62" s="105" t="n">
-        <x:v>1175</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="X62" s="105" t="n">
-        <x:v>180</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="Y62" s="102" t="n">
         <x:v>46218</x:v>
@@ -29860,19 +29906,19 @@
     </x:row>
     <x:row r="63" ht="38" customHeight="1">
       <x:c r="A63" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5060-ti-16gb</x:v>
+        <x:v>nvidia-geforce-rtx-5060-ti-8gb</x:v>
       </x:c>
       <x:c r="B63" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C63" s="12" t="str">
-        <x:v>GeForce RTX 5060 Ti 16GB</x:v>
+        <x:v>GeForce RTX 5060 Ti 8GB</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5060 Ti 16GB</x:v>
+        <x:v>NVIDIA GeForce RTX 5060 Ti 8GB</x:v>
       </x:c>
       <x:c r="E63" s="12" t="str">
-        <x:v>GeForce RTX 5060 Ti 16GB</x:v>
+        <x:v>GeForce RTX 5060 Ti 8GB</x:v>
       </x:c>
       <x:c r="F63" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29910,7 +29956,7 @@
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S63" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T63" s="12" t="str">
         <x:v>GDDR7</x:v>
@@ -29919,10 +29965,10 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="V63" s="105" t="n">
-        <x:v>22626</x:v>
+        <x:v>22067</x:v>
       </x:c>
       <x:c r="W63" s="105" t="n">
-        <x:v>1207</x:v>
+        <x:v>1175</x:v>
       </x:c>
       <x:c r="X63" s="105" t="n">
         <x:v>180</x:v>
@@ -29933,19 +29979,19 @@
     </x:row>
     <x:row r="64" ht="38" customHeight="1">
       <x:c r="A64" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5070</x:v>
+        <x:v>nvidia-geforce-rtx-5060-ti-16gb</x:v>
       </x:c>
       <x:c r="B64" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
-        <x:v>GeForce RTX 5070</x:v>
+        <x:v>GeForce RTX 5060 Ti 16GB</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5070</x:v>
+        <x:v>NVIDIA GeForce RTX 5060 Ti 16GB</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>GeForce RTX 5070</x:v>
+        <x:v>GeForce RTX 5060 Ti 16GB</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
         <x:v>research_required</x:v>
@@ -29974,31 +30020,31 @@
         <x:v>GeForce RTX 50 Series</x:v>
       </x:c>
       <x:c r="P64" s="102" t="n">
-        <x:v>45721</x:v>
+        <x:v>45763</x:v>
       </x:c>
       <x:c r="Q64" s="12" t="str">
-        <x:v>2025-03-05</x:v>
+        <x:v>2025-04-16</x:v>
       </x:c>
       <x:c r="R64" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S64" s="104" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T64" s="12" t="str">
         <x:v>GDDR7</x:v>
       </x:c>
       <x:c r="U64" s="105" t="n">
-        <x:v>192</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="V64" s="105" t="n">
-        <x:v>28684</x:v>
+        <x:v>22626</x:v>
       </x:c>
       <x:c r="W64" s="105" t="n">
-        <x:v>1294</x:v>
+        <x:v>1207</x:v>
       </x:c>
       <x:c r="X64" s="105" t="n">
-        <x:v>250</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="Y64" s="102" t="n">
         <x:v>46218</x:v>
@@ -30006,19 +30052,19 @@
     </x:row>
     <x:row r="65" ht="38" customHeight="1">
       <x:c r="A65" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5070-ti</x:v>
+        <x:v>nvidia-geforce-rtx-5070</x:v>
       </x:c>
       <x:c r="B65" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C65" s="12" t="str">
-        <x:v>GeForce RTX 5070 Ti</x:v>
+        <x:v>GeForce RTX 5070</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5070 Ti</x:v>
+        <x:v>NVIDIA GeForce RTX 5070</x:v>
       </x:c>
       <x:c r="E65" s="12" t="str">
-        <x:v>GeForce RTX 5070 Ti</x:v>
+        <x:v>GeForce RTX 5070</x:v>
       </x:c>
       <x:c r="F65" s="12" t="str">
         <x:v>research_required</x:v>
@@ -30047,31 +30093,31 @@
         <x:v>GeForce RTX 50 Series</x:v>
       </x:c>
       <x:c r="P65" s="102" t="n">
-        <x:v>45708</x:v>
+        <x:v>45721</x:v>
       </x:c>
       <x:c r="Q65" s="12" t="str">
-        <x:v>2025-02-20</x:v>
+        <x:v>2025-03-05</x:v>
       </x:c>
       <x:c r="R65" s="12" t="str">
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S65" s="104" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="T65" s="12" t="str">
         <x:v>GDDR7</x:v>
       </x:c>
       <x:c r="U65" s="105" t="n">
-        <x:v>256</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="V65" s="105" t="n">
-        <x:v>32367</x:v>
+        <x:v>28684</x:v>
       </x:c>
       <x:c r="W65" s="105" t="n">
-        <x:v>1326</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="X65" s="105" t="n">
-        <x:v>300</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="Y65" s="102" t="n">
         <x:v>46218</x:v>
@@ -30079,19 +30125,19 @@
     </x:row>
     <x:row r="66" ht="38" customHeight="1">
       <x:c r="A66" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5080</x:v>
+        <x:v>nvidia-geforce-rtx-5070-ti</x:v>
       </x:c>
       <x:c r="B66" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C66" s="12" t="str">
-        <x:v>GeForce RTX 5080</x:v>
+        <x:v>GeForce RTX 5070 Ti</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5080</x:v>
+        <x:v>NVIDIA GeForce RTX 5070 Ti</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
-        <x:v>GeForce RTX 5080</x:v>
+        <x:v>GeForce RTX 5070 Ti</x:v>
       </x:c>
       <x:c r="F66" s="12" t="str">
         <x:v>research_required</x:v>
@@ -30120,10 +30166,10 @@
         <x:v>GeForce RTX 50 Series</x:v>
       </x:c>
       <x:c r="P66" s="102" t="n">
-        <x:v>45687</x:v>
+        <x:v>45708</x:v>
       </x:c>
       <x:c r="Q66" s="12" t="str">
-        <x:v>2025-01-30</x:v>
+        <x:v>2025-02-20</x:v>
       </x:c>
       <x:c r="R66" s="12" t="str">
         <x:v>exact</x:v>
@@ -30138,13 +30184,13 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="V66" s="105" t="n">
-        <x:v>35656</x:v>
+        <x:v>32367</x:v>
       </x:c>
       <x:c r="W66" s="105" t="n">
-        <x:v>1402</x:v>
+        <x:v>1326</x:v>
       </x:c>
       <x:c r="X66" s="105" t="n">
-        <x:v>360</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="Y66" s="102" t="n">
         <x:v>46218</x:v>
@@ -30152,19 +30198,19 @@
     </x:row>
     <x:row r="67" ht="38" customHeight="1">
       <x:c r="A67" s="12" t="str">
-        <x:v>nvidia-geforce-rtx-5090</x:v>
+        <x:v>nvidia-geforce-rtx-5080</x:v>
       </x:c>
       <x:c r="B67" s="12" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="C67" s="12" t="str">
-        <x:v>GeForce RTX 5090</x:v>
+        <x:v>GeForce RTX 5080</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>NVIDIA GeForce RTX 5090</x:v>
+        <x:v>NVIDIA GeForce RTX 5080</x:v>
       </x:c>
       <x:c r="E67" s="12" t="str">
-        <x:v>GeForce RTX 5090</x:v>
+        <x:v>GeForce RTX 5080</x:v>
       </x:c>
       <x:c r="F67" s="12" t="str">
         <x:v>research_required</x:v>
@@ -30202,53 +30248,99 @@
         <x:v>exact</x:v>
       </x:c>
       <x:c r="S67" s="104" t="n">
-        <x:v>32</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="T67" s="12" t="str">
         <x:v>GDDR7</x:v>
       </x:c>
       <x:c r="U67" s="105" t="n">
-        <x:v>512</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="V67" s="105" t="n">
-        <x:v>38970</x:v>
+        <x:v>35656</x:v>
       </x:c>
       <x:c r="W67" s="105" t="n">
-        <x:v>1411</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="X67" s="105" t="n">
-        <x:v>575</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="Y67" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
     </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="12"/>
-      <x:c r="B68" s="12"/>
-      <x:c r="C68" s="12"/>
-      <x:c r="D68" s="12"/>
-      <x:c r="E68" s="12"/>
-      <x:c r="F68" s="12"/>
-      <x:c r="G68" s="12"/>
-      <x:c r="H68" s="102"/>
-      <x:c r="I68" s="14"/>
+    <x:row r="68" ht="38" customHeight="1">
+      <x:c r="A68" s="12" t="str">
+        <x:v>nvidia-geforce-rtx-5090</x:v>
+      </x:c>
+      <x:c r="B68" s="12" t="str">
+        <x:v>NVIDIA</x:v>
+      </x:c>
+      <x:c r="C68" s="12" t="str">
+        <x:v>GeForce RTX 5090</x:v>
+      </x:c>
+      <x:c r="D68" s="12" t="str">
+        <x:v>NVIDIA GeForce RTX 5090</x:v>
+      </x:c>
+      <x:c r="E68" s="12" t="str">
+        <x:v>GeForce RTX 5090</x:v>
+      </x:c>
+      <x:c r="F68" s="12" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="G68" s="12" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="H68" s="102" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="I68" s="14" t="str">
+        <x:v>GPUチップ性能比較用の基準レコード。実製品の冷却・騒音・寸法・保証はGPUシートのボードSKUで別評価します。</x:v>
+      </x:c>
       <x:c r="J68" s="14"/>
       <x:c r="K68" s="14"/>
-      <x:c r="L68" s="14"/>
-      <x:c r="M68" s="14"/>
-      <x:c r="N68" s="12"/>
-      <x:c r="O68" s="12"/>
-      <x:c r="P68" s="102"/>
-      <x:c r="Q68" s="12"/>
-      <x:c r="R68" s="12"/>
-      <x:c r="S68" s="104"/>
-      <x:c r="T68" s="12"/>
-      <x:c r="U68" s="105"/>
-      <x:c r="V68" s="105"/>
-      <x:c r="W68" s="105"/>
-      <x:c r="X68" s="105"/>
-      <x:c r="Y68" s="102"/>
+      <x:c r="L68" s="14" t="str">
+        <x:v>ボードメーカー別の品質・保証・電源・寸法は未評価</x:v>
+      </x:c>
+      <x:c r="M68" s="14" t="str">
+        <x:v>PassMark値は2026-07-15確認時点。販売商品への自動承認には使用せず、個別ボードSKUを別途登録してください。</x:v>
+      </x:c>
+      <x:c r="N68" s="12" t="str">
+        <x:v>Blackwell</x:v>
+      </x:c>
+      <x:c r="O68" s="12" t="str">
+        <x:v>GeForce RTX 50 Series</x:v>
+      </x:c>
+      <x:c r="P68" s="102" t="n">
+        <x:v>45687</x:v>
+      </x:c>
+      <x:c r="Q68" s="12" t="str">
+        <x:v>2025-01-30</x:v>
+      </x:c>
+      <x:c r="R68" s="12" t="str">
+        <x:v>exact</x:v>
+      </x:c>
+      <x:c r="S68" s="104" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T68" s="12" t="str">
+        <x:v>GDDR7</x:v>
+      </x:c>
+      <x:c r="U68" s="105" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="V68" s="105" t="n">
+        <x:v>38970</x:v>
+      </x:c>
+      <x:c r="W68" s="105" t="n">
+        <x:v>1411</x:v>
+      </x:c>
+      <x:c r="X68" s="105" t="n">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="Y68" s="102" t="n">
+        <x:v>46218</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="12"/>
@@ -30768,16 +30860,30 @@
     <x:mergeCell ref="A1:Y1"/>
     <x:mergeCell ref="A2:Y2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="V5:W67">
+  <x:conditionalFormatting sqref="V5:V87">
     <x:cfRule type="dataBar" priority="1">
       <x:dataBar>
         <x:cfvo type="min"/>
         <x:cfvo type="max"/>
-        <x:color rgb="FF8064A2"/>
+        <x:color rgb="FFA855F7"/>
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{58B05D94-C265-D22A-9AA4-204FA01C3CBA}</x14:id>
+        </x:ext>
+      </x:extLst>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="W5:W87">
+    <x:cfRule type="dataBar" priority="2">
+      <x:dataBar>
+        <x:cfvo type="min"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FF8B5CF6"/>
+      </x:dataBar>
+      <x:extLst>
+        <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{93A4E389-95CD-84F5-1798-C041AB50329E}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -30795,7 +30901,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a4bd449bcf24c48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8c76e70cf774e95"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -30805,10 +30911,20 @@
             <x14:dataBar gradient="1">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
-              <x14:fillColor rgb="FF8064A2"/>
+              <x14:fillColor rgb="FFA855F7"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>V5:W67</xm:sqref>
+          <xm:sqref>V5:V87</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting>
+          <x14:cfRule type="dataBar" priority="2" id="{93A4E389-95CD-84F5-1798-C041AB50329E}">
+            <x14:dataBar gradient="1">
+              <x14:cfvo type="min"/>
+              <x14:cfvo type="max"/>
+              <x14:fillColor rgb="FF8B5CF6"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>W5:W87</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </x:ext>
@@ -30905,7 +31021,7 @@
       </x:c>
       <x:c r="B6" s="129" t="n">
         <x:f>COUNTA('GPUChips'!$A$5:$A$500)</x:f>
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C6" s="129" t="n">
         <x:f>COUNTIF('GPUChips'!$F$5:$F$500,"approved")+COUNTIF('GPUChips'!$F$5:$F$500,"preferred")</x:f>
@@ -30913,7 +31029,7 @@
       </x:c>
       <x:c r="D6" s="129" t="n">
         <x:f>COUNTIF('GPUChips'!$F$5:$F$500,"research_required")</x:f>
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -44132,7 +44248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d339dde30054c22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaabbb4581b545aa"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -45242,25 +45358,25 @@
     <x:dataValidation type="list" sqref="K5:K24">
       <x:formula1>"unrated,C,B,A,S"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="V5:V24">
-      <x:formula1>'Lists'!$P$5:$P$8</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="X5:X24">
-      <x:formula1>'Lists'!$R$5:$R$9</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="Y5:Y24">
-      <x:formula1>'Lists'!$Q$5:$Q$9</x:formula1>
-    </x:dataValidation>
     <x:dataValidation type="list" sqref="R5:R24">
       <x:formula1>'GPUChips'!$A$5:$A$500</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="W5:X24">
+    <x:dataValidation type="list" sqref="AD5:AD24">
+      <x:formula1>'Lists'!$R$5:$R$9</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AE5:AE24">
+      <x:formula1>'Lists'!$Q$5:$Q$9</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="W5:X24">
       <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AA5:AA24">
+      <x:formula1>'Lists'!$P$5:$P$8</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b6af0a39b5a44a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07f84f3f9f514877"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46052,7 +46168,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e2bb9bcf0ee4bb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R012ff84d6dfe4ee3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46931,7 +47047,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9867a169ffe4a38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7ee230b1a24923"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47764,7 +47880,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R471e08fd03124319"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62d95a28f4014403"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -48643,7 +48759,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fff36a2ab1446e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2152620cd1ef480e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49548,7 +49664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd95d743236144001"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f62067fc137430b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add memory catalog with default SPD rates
</commit_message>
<xml_diff>
--- a/catalog/quality_catalog.xlsx
+++ b/catalog/quality_catalog.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R09c47f1f21614974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search" sheetId="2" r:id="R97835d0666cf4df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="3" r:id="Ra362d31abacf4598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="4" r:id="Rd89dc71bee4c43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="5" r:id="R0a50948d92124688"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="6" r:id="R6c96d6ff06ba4fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PSU" sheetId="7" r:id="R7e3b40c22657474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motherboard" sheetId="8" r:id="R86bac745f273485e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitor" sheetId="9" r:id="Ra67db51a50674f95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifiers" sheetId="10" r:id="R617d0ab61d524d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="11" r:id="R913c5df0f03b4637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="12" r:id="R7d5a66584dda4e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="13" r:id="R5e10acd8fdd24f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="14" r:id="R402a3a2cc7df4190"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" r:id="R836bde92f0fe4283"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SheetDefinitions" sheetId="16" r:id="Rfc5d49b8c49b419d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDefinitions" sheetId="17" r:id="R944dc2fe72c04b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" r:id="R080cf0bc2c4a4ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPUChips" sheetId="19" r:id="Rb69935859f914bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R95ca3fde305240ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search" sheetId="2" r:id="R780e913fc8b74466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="3" r:id="R7cdacb4615d24ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="4" r:id="R1e0e771df4594734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="5" r:id="Rc2dcaa3030974c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="6" r:id="R20f3ed3eef104bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PSU" sheetId="7" r:id="Rfbeaead9b171492b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motherboard" sheetId="8" r:id="R5f9f0e3ac686463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitor" sheetId="9" r:id="R9e4b1a5905dc4b1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifiers" sheetId="10" r:id="Re543e4f5d47d40ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="11" r:id="R6c6488849fda439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="12" r:id="Rd9eb67d5f9fe4c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="13" r:id="Re004581f24bb49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="14" r:id="R88f3f05bdb3e4c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" r:id="R21e63ea10f7345ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SheetDefinitions" sheetId="16" r:id="R3434ea178c4f41be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDefinitions" sheetId="17" r:id="Rdfb362e5c1cd415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" r:id="R1e871404da94470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPUChips" sheetId="19" r:id="R5581e7ed0f534955"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -187,6 +187,11 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="7">
     <x:border/>
@@ -248,7 +253,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="131">
+  <x:cellXfs count="137">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -554,6 +559,18 @@
     <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1066,9 +1083,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="MemoryCatalog" displayName="MemoryCatalog" ref="A4:AA24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:AA24"/>
-  <x:tableColumns count="27">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="MemoryCatalog" displayName="MemoryCatalog" ref="A4:AB24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="28">
     <x:tableColumn id="1" name="product_id"/>
     <x:tableColumn id="2" name="brand"/>
     <x:tableColumn id="3" name="model"/>
@@ -1096,6 +1112,7 @@
     <x:tableColumn id="25" name="warranty_class"/>
     <x:tableColumn id="26" name="voltage_v"/>
     <x:tableColumn id="27" name="chip_type"/>
+    <x:tableColumn id="28" name="default_data_rate_mt_s"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2044,7 +2061,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81bd26549108438f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3c06410a2074764"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13911,181 +13928,618 @@
         <x:v>PassMarkはVRAM容量別に分離していないため共通スコアを参考値として記録。</x:v>
       </x:c>
     </x:row>
-    <x:row r="357">
-      <x:c r="A357"/>
-      <x:c r="B357"/>
-      <x:c r="C357"/>
-      <x:c r="D357" s="121"/>
-      <x:c r="E357" s="121"/>
-      <x:c r="F357" s="125"/>
-      <x:c r="G357" s="121"/>
-      <x:c r="H357" s="121"/>
-      <x:c r="I357" s="121"/>
-    </x:row>
-    <x:row r="358">
-      <x:c r="A358"/>
-      <x:c r="B358"/>
-      <x:c r="C358"/>
-      <x:c r="D358" s="121"/>
-      <x:c r="E358" s="121"/>
-      <x:c r="F358" s="125"/>
-      <x:c r="G358" s="121"/>
-      <x:c r="H358" s="121"/>
-      <x:c r="I358" s="121"/>
-    </x:row>
-    <x:row r="359">
-      <x:c r="A359"/>
-      <x:c r="B359"/>
-      <x:c r="C359"/>
-      <x:c r="D359" s="121"/>
-      <x:c r="E359" s="121"/>
-      <x:c r="F359" s="125"/>
-      <x:c r="G359" s="121"/>
-      <x:c r="H359" s="121"/>
-      <x:c r="I359" s="121"/>
-    </x:row>
-    <x:row r="360">
-      <x:c r="A360"/>
-      <x:c r="B360"/>
-      <x:c r="C360"/>
-      <x:c r="D360" s="121"/>
-      <x:c r="E360" s="121"/>
-      <x:c r="F360" s="125"/>
-      <x:c r="G360" s="121"/>
-      <x:c r="H360" s="121"/>
-      <x:c r="I360" s="121"/>
-    </x:row>
-    <x:row r="361">
-      <x:c r="A361"/>
-      <x:c r="B361"/>
-      <x:c r="C361"/>
-      <x:c r="D361" s="121"/>
-      <x:c r="E361" s="121"/>
-      <x:c r="F361" s="125"/>
-      <x:c r="G361" s="121"/>
-      <x:c r="H361" s="121"/>
-      <x:c r="I361" s="121"/>
-    </x:row>
-    <x:row r="362">
-      <x:c r="A362"/>
-      <x:c r="B362"/>
-      <x:c r="C362"/>
-      <x:c r="D362" s="121"/>
-      <x:c r="E362" s="121"/>
-      <x:c r="F362" s="125"/>
-      <x:c r="G362" s="121"/>
-      <x:c r="H362" s="121"/>
-      <x:c r="I362" s="121"/>
-    </x:row>
-    <x:row r="363">
-      <x:c r="A363"/>
-      <x:c r="B363"/>
-      <x:c r="C363"/>
-      <x:c r="D363" s="121"/>
-      <x:c r="E363" s="121"/>
-      <x:c r="F363" s="125"/>
-      <x:c r="G363" s="121"/>
-      <x:c r="H363" s="121"/>
-      <x:c r="I363" s="121"/>
-    </x:row>
-    <x:row r="364">
-      <x:c r="A364"/>
-      <x:c r="B364"/>
-      <x:c r="C364"/>
-      <x:c r="D364" s="121"/>
-      <x:c r="E364" s="121"/>
-      <x:c r="F364" s="125"/>
-      <x:c r="G364" s="121"/>
-      <x:c r="H364" s="121"/>
-      <x:c r="I364" s="121"/>
-    </x:row>
-    <x:row r="365">
-      <x:c r="A365"/>
-      <x:c r="B365"/>
-      <x:c r="C365"/>
-      <x:c r="D365" s="121"/>
-      <x:c r="E365" s="121"/>
-      <x:c r="F365" s="125"/>
-      <x:c r="G365" s="121"/>
-      <x:c r="H365" s="121"/>
-      <x:c r="I365" s="121"/>
-    </x:row>
-    <x:row r="366">
-      <x:c r="A366"/>
-      <x:c r="B366"/>
-      <x:c r="C366"/>
-      <x:c r="D366" s="121"/>
-      <x:c r="E366" s="121"/>
-      <x:c r="F366" s="125"/>
-      <x:c r="G366" s="121"/>
-      <x:c r="H366" s="121"/>
-      <x:c r="I366" s="121"/>
-    </x:row>
-    <x:row r="367">
-      <x:c r="A367"/>
-      <x:c r="B367"/>
-      <x:c r="C367"/>
-      <x:c r="D367" s="121"/>
-      <x:c r="E367" s="121"/>
-      <x:c r="F367" s="125"/>
-      <x:c r="G367" s="121"/>
-      <x:c r="H367" s="121"/>
-      <x:c r="I367" s="121"/>
-    </x:row>
-    <x:row r="368">
-      <x:c r="A368"/>
-      <x:c r="B368"/>
-      <x:c r="C368"/>
-      <x:c r="D368" s="121"/>
-      <x:c r="E368" s="121"/>
-      <x:c r="F368" s="125"/>
-      <x:c r="G368" s="121"/>
-      <x:c r="H368" s="121"/>
-      <x:c r="I368" s="121"/>
-    </x:row>
-    <x:row r="369">
-      <x:c r="A369"/>
-      <x:c r="B369"/>
-      <x:c r="C369"/>
-      <x:c r="D369" s="121"/>
-      <x:c r="E369" s="121"/>
-      <x:c r="F369" s="125"/>
-      <x:c r="G369" s="121"/>
-      <x:c r="H369" s="121"/>
-      <x:c r="I369" s="121"/>
-    </x:row>
-    <x:row r="370">
-      <x:c r="A370"/>
-      <x:c r="B370"/>
-      <x:c r="C370"/>
-      <x:c r="D370" s="121"/>
-      <x:c r="E370" s="121"/>
-      <x:c r="F370" s="125"/>
-      <x:c r="G370" s="121"/>
-      <x:c r="H370" s="121"/>
-      <x:c r="I370" s="121"/>
-    </x:row>
-    <x:row r="371">
-      <x:c r="A371"/>
-      <x:c r="B371"/>
-      <x:c r="C371"/>
-      <x:c r="D371" s="121"/>
-      <x:c r="E371" s="121"/>
-      <x:c r="F371" s="125"/>
-      <x:c r="G371" s="121"/>
-      <x:c r="H371" s="121"/>
-      <x:c r="I371" s="121"/>
-    </x:row>
-    <x:row r="372">
-      <x:c r="A372"/>
-      <x:c r="B372"/>
-      <x:c r="C372"/>
-      <x:c r="D372" s="121"/>
-      <x:c r="E372" s="121"/>
-      <x:c r="F372" s="125"/>
-      <x:c r="G372" s="121"/>
-      <x:c r="H372" s="121"/>
-      <x:c r="I372" s="121"/>
+    <x:row r="357" ht="42" customHeight="1">
+      <x:c r="A357" t="str">
+        <x:v>memory-corsair-cmk32gx5m2b6000z30-official</x:v>
+      </x:c>
+      <x:c r="B357" t="str">
+        <x:v>memory-corsair-cmk32gx5m2b6000z30</x:v>
+      </x:c>
+      <x:c r="C357" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D357" s="121" t="str">
+        <x:v>Corsair VENGEANCE DDR5 CMK32GX5M2B6000Z30 公式仕様</x:v>
+      </x:c>
+      <x:c r="E357" s="121" t="str">
+        <x:v>https://www.corsair.com/us/en/p/memory/cmk32gx5m2b6000z30/vengeance-32gb-2x16gb-ddr5-dram-6000mt-s-cl30-amd-expo-memory-black-cmk32gx5m2b6000z30</x:v>
+      </x:c>
+      <x:c r="F357" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G357" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H357" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I357" s="121" t="str">
+        <x:v>32GB (2×16GB)、6000MT/s、30-36-36-76、1.40V、EXPO/XMP、限定永久保証を確認。 標準SPD/JEDEC速度は4800MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358" ht="42" customHeight="1">
+      <x:c r="A358" t="str">
+        <x:v>memory-corsair-cmk64gx5m2b6000z30-official</x:v>
+      </x:c>
+      <x:c r="B358" t="str">
+        <x:v>memory-corsair-cmk64gx5m2b6000z30</x:v>
+      </x:c>
+      <x:c r="C358" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D358" s="121" t="str">
+        <x:v>Corsair VENGEANCE DDR5 CMK64GX5M2B6000Z30 公式仕様</x:v>
+      </x:c>
+      <x:c r="E358" s="121" t="str">
+        <x:v>https://www.corsair.com/ww/en/p/memory/CMK64GX5M2B6000Z30/vengeance-64gb-2x32gb-ddr5-dram-6000mt-s-cl30-amd-expo-%26-intel-xmp-memory-kit-cmk64gx5m2b6000z30</x:v>
+      </x:c>
+      <x:c r="F358" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G358" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H358" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I358" s="121" t="str">
+        <x:v>64GB (2×32GB)、6000MT/s、30-36-36-76、1.40V、EXPO/XMP、限定永久保証を確認。 標準SPD/JEDEC速度は4800MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359" ht="42" customHeight="1">
+      <x:c r="A359" t="str">
+        <x:v>memory-corsair-cmk32gx4m2e3200c16-official</x:v>
+      </x:c>
+      <x:c r="B359" t="str">
+        <x:v>memory-corsair-cmk32gx4m2e3200c16</x:v>
+      </x:c>
+      <x:c r="C359" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D359" s="121" t="str">
+        <x:v>Corsair VENGEANCE LPX CMK32GX4M2E3200C16 公式仕様</x:v>
+      </x:c>
+      <x:c r="E359" s="121" t="str">
+        <x:v>https://www.corsair.com/us/en/p/memory/cmk32gx4m2e3200c16/vengeance-lpx-32gb-2-x-16gb-ddr4-dram-3200mhz-c16-memory-kit-black-cmk32gx4m2e3200c16</x:v>
+      </x:c>
+      <x:c r="F359" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G359" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H359" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I359" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR4-3200 CL16、1.35V、XMP 2.0、限定永久保証を確認。 標準SPD/JEDEC速度は2133MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360" ht="42" customHeight="1">
+      <x:c r="A360" t="str">
+        <x:v>memory-corsair-cmk64gx4m2e3200c16-official</x:v>
+      </x:c>
+      <x:c r="B360" t="str">
+        <x:v>memory-corsair-cmk64gx4m2e3200c16</x:v>
+      </x:c>
+      <x:c r="C360" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D360" s="121" t="str">
+        <x:v>Corsair VENGEANCE LPX CMK64GX4M2E3200C16 公式仕様</x:v>
+      </x:c>
+      <x:c r="E360" s="121" t="str">
+        <x:v>https://www.corsair.com/us/en/p/memory/cmk64gx4m2e3200c16/vengeancea-lpx-64gb-2-x-32gb-ddr4-dram-3200mhz-c16-memory-kit-black-cmk64gx4m2e3200c16</x:v>
+      </x:c>
+      <x:c r="F360" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G360" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H360" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I360" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR4-3200、16-20-20-38、1.35V、XMP 2.0、限定永久保証を確認。 標準SPD/JEDEC速度は2133MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361" ht="42" customHeight="1">
+      <x:c r="A361" t="str">
+        <x:v>memory-gskill-f5-6000j3038f16gx2-fx5-official</x:v>
+      </x:c>
+      <x:c r="B361" t="str">
+        <x:v>memory-gskill-f5-6000j3038f16gx2-fx5</x:v>
+      </x:c>
+      <x:c r="C361" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D361" s="121" t="str">
+        <x:v>G.SKILL F5-6000J3038F16GX2-FX5 EXPO自己認証レポート</x:v>
+      </x:c>
+      <x:c r="E361" s="121" t="str">
+        <x:v>https://www.gskill.com/_upload/files/F5-6000J3038F16GX2-FX5.pdf</x:v>
+      </x:c>
+      <x:c r="F361" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G361" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.chip_type
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H361" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I361" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR5-6000、30-38-38-96、1.35V、EXPO、Module Rev.1.0のSK hynix構成を確認。 標準SPD/JEDEC速度は4800MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="42" customHeight="1">
+      <x:c r="A362" t="str">
+        <x:v>memory-gskill-f5-6000j3040g32gx2-fx5-official</x:v>
+      </x:c>
+      <x:c r="B362" t="str">
+        <x:v>memory-gskill-f5-6000j3040g32gx2-fx5</x:v>
+      </x:c>
+      <x:c r="C362" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D362" s="121" t="str">
+        <x:v>G.SKILL F5-6000J3040G32GX2-FX5 公式仕様</x:v>
+      </x:c>
+      <x:c r="E362" s="121" t="str">
+        <x:v>https://www.gskill.com/cn/specification/204/398/1691400033/F5-6000J3040G32GX2-FX5-Specification</x:v>
+      </x:c>
+      <x:c r="F362" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G362" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H362" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I362" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR5-6000、30-40-40-96、1.40V、EXPO/XMP、限定永久保証を確認。 標準SPD/JEDEC速度は4800MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363" ht="42" customHeight="1">
+      <x:c r="A363" t="str">
+        <x:v>memory-gskill-f4-3600c16d-32gvkc-official</x:v>
+      </x:c>
+      <x:c r="B363" t="str">
+        <x:v>memory-gskill-f4-3600c16d-32gvkc</x:v>
+      </x:c>
+      <x:c r="C363" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D363" s="121" t="str">
+        <x:v>G.SKILL F4-3600C16D-32GVKC 公式仕様</x:v>
+      </x:c>
+      <x:c r="E363" s="121" t="str">
+        <x:v>https://www.gskill.com/specification/165/184/1562831784/F4-3600C16D-32GVKC-Specification</x:v>
+      </x:c>
+      <x:c r="F363" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G363" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H363" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I363" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR4-3600、16-19-19-39、1.35V、XMP 2.0、限定永久保証を確認。 標準SPD/JEDEC速度は2133MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="42" customHeight="1">
+      <x:c r="A364" t="str">
+        <x:v>memory-gskill-f4-3600c18d-64gvk-official</x:v>
+      </x:c>
+      <x:c r="B364" t="str">
+        <x:v>memory-gskill-f4-3600c18d-64gvk</x:v>
+      </x:c>
+      <x:c r="C364" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D364" s="121" t="str">
+        <x:v>G.SKILL F4-3600C18D-64GVK 公式仕様</x:v>
+      </x:c>
+      <x:c r="E364" s="121" t="str">
+        <x:v>https://www.gskill.com/cn/specification/204/218/1571734306/F4-3600C18D-64GVK-Specification</x:v>
+      </x:c>
+      <x:c r="F364" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G364" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H364" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I364" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR4-3600、18-22-22-42、1.35V、XMP 2.0、限定永久保証を確認。 標準SPD/JEDEC速度は2666MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365" ht="42" customHeight="1">
+      <x:c r="A365" t="str">
+        <x:v>memory-kingston-kf560c30bbek2-32-official</x:v>
+      </x:c>
+      <x:c r="B365" t="str">
+        <x:v>memory-kingston-kf560c30bbek2-32</x:v>
+      </x:c>
+      <x:c r="C365" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D365" s="121" t="str">
+        <x:v>Kingston KF560C30BBEK2-32 公式データシート</x:v>
+      </x:c>
+      <x:c r="E365" s="121" t="str">
+        <x:v>https://www.kingston.com/datasheets/KF560C30BBEK2-32.pdf</x:v>
+      </x:c>
+      <x:c r="F365" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G365" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.module_height_mm
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H365" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I365" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR5-6000 CL30-36-36、1.40V、EXPO/XMP、高さ34.9mm、1Rx8を確認。 標準SPD/JEDEC速度は4800MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366" ht="42" customHeight="1">
+      <x:c r="A366" t="str">
+        <x:v>memory-kingston-kf560c30bbek2-64-official</x:v>
+      </x:c>
+      <x:c r="B366" t="str">
+        <x:v>memory-kingston-kf560c30bbek2-64</x:v>
+      </x:c>
+      <x:c r="C366" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D366" s="121" t="str">
+        <x:v>Kingston KF560C30BBEK2-64 公式データシート</x:v>
+      </x:c>
+      <x:c r="E366" s="121" t="str">
+        <x:v>https://www.kingston.com/datasheets/KF560C30BBEK2-64.pdf</x:v>
+      </x:c>
+      <x:c r="F366" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G366" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.module_height_mm
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H366" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I366" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR5-6000 CL30-36-36、1.40V、EXPO/XMP、高さ34.9mm、2Rx8を確認。 標準SPD/JEDEC速度は4800MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367" ht="42" customHeight="1">
+      <x:c r="A367" t="str">
+        <x:v>memory-kingston-kf432c16bbk2-32-official</x:v>
+      </x:c>
+      <x:c r="B367" t="str">
+        <x:v>memory-kingston-kf432c16bbk2-32</x:v>
+      </x:c>
+      <x:c r="C367" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D367" s="121" t="str">
+        <x:v>Kingston KF432C16BBK2/32 公式データシート</x:v>
+      </x:c>
+      <x:c r="E367" s="121" t="str">
+        <x:v>https://www.kingston.com/dataSheets/KF432C16BBK2_32.pdf</x:v>
+      </x:c>
+      <x:c r="F367" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G367" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.module_height_mm
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H367" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I367" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR4-3200 CL16-20-20、1.35V、XMP 2.0、高さ34mm、1Rx8を確認。 標準SPD/JEDEC速度は2400MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368" ht="42" customHeight="1">
+      <x:c r="A368" t="str">
+        <x:v>memory-kingston-kf432c16bbk2-64-official</x:v>
+      </x:c>
+      <x:c r="B368" t="str">
+        <x:v>memory-kingston-kf432c16bbk2-64</x:v>
+      </x:c>
+      <x:c r="C368" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D368" s="121" t="str">
+        <x:v>Kingston KF432C16BBK2/64 公式データシート</x:v>
+      </x:c>
+      <x:c r="E368" s="121" t="str">
+        <x:v>https://www.kingston.com/datasheets/KF432C16BBK2_64.pdf</x:v>
+      </x:c>
+      <x:c r="F368" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G368" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.module_height_mm
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H368" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I368" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR4-3200 CL16-20-20、1.35V、XMP 2.0、高さ34mm、2Rx8を確認。 標準SPD/JEDEC速度は2400MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369" ht="42" customHeight="1">
+      <x:c r="A369" t="str">
+        <x:v>memory-crucial-cp2k16g60c36u5b-official</x:v>
+      </x:c>
+      <x:c r="B369" t="str">
+        <x:v>memory-crucial-cp2k16g60c36u5b</x:v>
+      </x:c>
+      <x:c r="C369" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D369" s="121" t="str">
+        <x:v>Crucial Pro CP2K16G60C36U5B 公式仕様</x:v>
+      </x:c>
+      <x:c r="E369" s="121" t="str">
+        <x:v>https://eu.crucial.com/memory/ddr5/cp2k16g60c36u5b/ct24919604</x:v>
+      </x:c>
+      <x:c r="F369" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G369" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H369" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I369" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR5-6000 CL36-38-38-80、1.35V、XMP/EXPO、限定永久保証を確認。 標準SPD/JEDEC速度は5600MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370" ht="42" customHeight="1">
+      <x:c r="A370" t="str">
+        <x:v>memory-crucial-cp2k32g60c40u5b-official</x:v>
+      </x:c>
+      <x:c r="B370" t="str">
+        <x:v>memory-crucial-cp2k32g60c40u5b</x:v>
+      </x:c>
+      <x:c r="C370" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D370" s="121" t="str">
+        <x:v>Crucial Pro CP2K32G60C40U5B 公式仕様</x:v>
+      </x:c>
+      <x:c r="E370" s="121" t="str">
+        <x:v>https://uk.crucial.com/memory/ddr5/cp2k32g60c40u5b</x:v>
+      </x:c>
+      <x:c r="F370" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G370" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H370" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I370" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR5-6000 CL40、1.35V、XMP/EXPO、限定永久保証を確認。 標準SPD/JEDEC速度は5600MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371" ht="42" customHeight="1">
+      <x:c r="A371" t="str">
+        <x:v>memory-crucial-cp2k16g4dfra32a-official</x:v>
+      </x:c>
+      <x:c r="B371" t="str">
+        <x:v>memory-crucial-cp2k16g4dfra32a</x:v>
+      </x:c>
+      <x:c r="C371" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D371" s="121" t="str">
+        <x:v>Crucial Pro CP2K16G4DFRA32A 公式仕様</x:v>
+      </x:c>
+      <x:c r="E371" s="121" t="str">
+        <x:v>https://www.crucial.com/memory/ddr4/cp2k16g4dfra32a/ct24204185</x:v>
+      </x:c>
+      <x:c r="F371" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G371" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H371" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I371" s="121" t="str">
+        <x:v>32GB (2×16GB)、DDR4-3200 CL22、1.20V、XMP 2.0、限定永久保証を確認。 標準SPD/JEDEC速度は3200MT/s。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372" ht="42" customHeight="1">
+      <x:c r="A372" t="str">
+        <x:v>memory-crucial-cp2k32g4dfra32a-official</x:v>
+      </x:c>
+      <x:c r="B372" t="str">
+        <x:v>memory-crucial-cp2k32g4dfra32a</x:v>
+      </x:c>
+      <x:c r="C372" t="str">
+        <x:v>manufacturer</x:v>
+      </x:c>
+      <x:c r="D372" s="121" t="str">
+        <x:v>Crucial Pro CP2K32G4DFRA32A 公式仕様</x:v>
+      </x:c>
+      <x:c r="E372" s="121" t="str">
+        <x:v>https://uk.crucial.com/memory/ddr4/cp2k32g4dfra32a</x:v>
+      </x:c>
+      <x:c r="F372" s="125" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="G372" s="121" t="str">
+        <x:v>identifiers.part_numbers
+specs.warranty_class
+specs.memory_type
+specs.total_capacity_gb
+specs.module_count
+specs.data_rate_mt_s
+specs.expo
+specs.cas_latency
+specs.voltage_v
+specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="H372" s="121" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I372" s="121" t="str">
+        <x:v>64GB (2×32GB)、DDR4-3200 CL22、1.20V、XMP 2.0、限定永久保証を確認。 標準SPD/JEDEC速度は3200MT/s。</x:v>
+      </x:c>
     </x:row>
     <x:row r="373">
       <x:c r="A373"/>
@@ -14121,7 +14575,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R517aef469ce84447"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R194a70fe949242bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14743,7 +15197,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9a1e09d257e417d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8797f06f165a43e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15425,7 +15879,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ecb08a4b6af43d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570d16fe6aae4abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17384,7 +17838,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re721ce02c8e84018"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75947ef1a5e34911"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17507,7 +17961,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R506d06735b39465b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24a713a07d71432a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17771,7 +18225,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c99b6ddd7348f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e9bd6e53ead40b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20627,7 +21081,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F113" s="121" t="str">
-        <x:v>データレート</x:v>
+        <x:v>XMP/EXPO等のOCプロファイル適用時の公称データレート</x:v>
       </x:c>
       <x:c r="G113" t="str">
         <x:v>MT/s</x:v>
@@ -24165,16 +24619,32 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="250">
-      <x:c r="A250"/>
-      <x:c r="B250"/>
-      <x:c r="C250"/>
-      <x:c r="D250"/>
-      <x:c r="E250"/>
-      <x:c r="F250" s="121"/>
-      <x:c r="G250"/>
+    <x:row r="250" ht="34" customHeight="1">
+      <x:c r="A250" t="str">
+        <x:v>Memory</x:v>
+      </x:c>
+      <x:c r="B250" t="str">
+        <x:v>default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="C250" t="str">
+        <x:v>specs.default_data_rate_mt_s</x:v>
+      </x:c>
+      <x:c r="D250" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="E250" s="9" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F250" s="121" t="str">
+        <x:v>OCプロファイル未適用時の標準SPD/JEDECデータレート</x:v>
+      </x:c>
+      <x:c r="G250" t="str">
+        <x:v>MT/s</x:v>
+      </x:c>
       <x:c r="H250"/>
-      <x:c r="I250"/>
+      <x:c r="I250" s="9" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="251">
       <x:c r="A251"/>
@@ -24403,7 +24873,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbc0cc467dbb4b93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R874710e8260b410f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25409,7 +25879,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9165a06c2daa4c39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b8a072bedd54914"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30901,7 +31371,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8c76e70cf774e95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f67cd6b597e411b"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -31055,7 +31525,7 @@
       </x:c>
       <x:c r="B8" s="129" t="n">
         <x:f>COUNTA('Memory'!$A$5:$A$500)</x:f>
-        <x:v>0</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C8" s="129" t="n">
         <x:f>COUNTIF('Memory'!$J$5:$J$500,"approved")+COUNTIF('Memory'!$J$5:$J$500,"preferred")</x:f>
@@ -31063,7 +31533,7 @@
       </x:c>
       <x:c r="D8" s="129" t="n">
         <x:f>COUNTIF('Memory'!$J$5:$J$500,"research_required")</x:f>
-        <x:v>0</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -44248,7 +44718,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaabbb4581b545aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4962af88a8144ade"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -45376,7 +45846,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07f84f3f9f514877"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1439b99680d41ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45412,6 +45882,7 @@
     <x:col min="25" max="25" width="14" hidden="0" customWidth="1"/>
     <x:col min="26" max="26" width="14" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="14" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -45447,7 +45918,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>メモリ容量、速度、レイテンシ、EXPO、寸法と保証を管理。新製品は最初の空行へ入力してください。列追加時はFieldDefinitionsにも1行追加します。</x:v>
+        <x:v>メモリ容量、XMP/EXPO公称速度、標準SPD/JEDEC速度、レイテンシ、寸法と保証を管理。新製品は最初の空行へ入力してください。列追加時はFieldDefinitionsにも1行追加します。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -45558,470 +46029,1306 @@
       <x:c r="AA4" s="21" t="str">
         <x:v>chip_type</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="22"/>
-      <x:c r="B5" s="14"/>
-      <x:c r="C5" s="14"/>
-      <x:c r="D5" s="14"/>
+      <x:c r="AB4" s="135" t="str">
+        <x:v>default_data_rate_mt_s</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52" customHeight="1">
+      <x:c r="A5" s="22" t="str">
+        <x:v>memory-corsair-cmk32gx5m2b6000z30</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>Corsair</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>CMK32GX5M2B6000Z30</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Corsair VENGEANCE DDR5-6000 32GB (16GB×2) CL30 AMD EXPO</x:v>
+      </x:c>
       <x:c r="E5" s="22"/>
       <x:c r="F5" s="22"/>
-      <x:c r="G5" s="22"/>
+      <x:c r="G5" s="22" t="str">
+        <x:v>CMK32GX5M2B6000Z30</x:v>
+      </x:c>
       <x:c r="H5" s="22"/>
-      <x:c r="I5" s="14"/>
-      <x:c r="J5" s="14"/>
-      <x:c r="K5" s="14"/>
-      <x:c r="L5" s="23"/>
-      <x:c r="M5" s="14"/>
-      <x:c r="N5" s="14"/>
-      <x:c r="O5" s="14"/>
-      <x:c r="P5" s="14"/>
-      <x:c r="Q5" s="14"/>
-      <x:c r="R5" s="14"/>
-      <x:c r="S5" s="25"/>
-      <x:c r="T5" s="24"/>
-      <x:c r="U5" s="24"/>
-      <x:c r="V5" s="14"/>
-      <x:c r="W5" s="25"/>
+      <x:c r="I5" s="14" t="str">
+        <x:v>VENGEANCE DDR5 32GB 6000 CL30 EXPO</x:v>
+      </x:c>
+      <x:c r="J5" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K5" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L5" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M5" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N5" s="14" t="str">
+        <x:v>DDR5-6000 CL30
+AMD EXPO・Intel XMP対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O5" s="14" t="str">
+        <x:v>定格動作にはプロファイル有効化と対応プラットフォームが必要
+公式商品ページでモジュール高さを数値確認できず</x:v>
+      </x:c>
+      <x:c r="P5" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q5" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R5" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S5" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T5" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U5" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V5" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W5" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="X5" s="25"/>
-      <x:c r="Y5" s="14"/>
-      <x:c r="Z5" s="25"/>
+      <x:c r="Y5" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z5" s="25" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
       <x:c r="AA5" s="14"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="22"/>
-      <x:c r="B6" s="14"/>
-      <x:c r="C6" s="14"/>
-      <x:c r="D6" s="14"/>
+      <x:c r="AB5" s="136" t="n">
+        <x:v>4800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
+      <x:c r="A6" s="22" t="str">
+        <x:v>memory-corsair-cmk64gx5m2b6000z30</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>Corsair</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>CMK64GX5M2B6000Z30</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>Corsair VENGEANCE DDR5-6000 64GB (32GB×2) CL30 AMD EXPO</x:v>
+      </x:c>
       <x:c r="E6" s="22"/>
       <x:c r="F6" s="22"/>
-      <x:c r="G6" s="22"/>
+      <x:c r="G6" s="22" t="str">
+        <x:v>CMK64GX5M2B6000Z30</x:v>
+      </x:c>
       <x:c r="H6" s="22"/>
-      <x:c r="I6" s="14"/>
-      <x:c r="J6" s="14"/>
-      <x:c r="K6" s="14"/>
-      <x:c r="L6" s="23"/>
-      <x:c r="M6" s="14"/>
-      <x:c r="N6" s="14"/>
-      <x:c r="O6" s="14"/>
-      <x:c r="P6" s="14"/>
-      <x:c r="Q6" s="14"/>
-      <x:c r="R6" s="14"/>
-      <x:c r="S6" s="25"/>
-      <x:c r="T6" s="24"/>
-      <x:c r="U6" s="24"/>
-      <x:c r="V6" s="14"/>
-      <x:c r="W6" s="25"/>
+      <x:c r="I6" s="14" t="str">
+        <x:v>VENGEANCE DDR5 64GB 6000 CL30 EXPO</x:v>
+      </x:c>
+      <x:c r="J6" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K6" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L6" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M6" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N6" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR5-6000 CL30
+AMD EXPO・Intel XMP対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O6" s="14" t="str">
+        <x:v>32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける
+公式商品ページでモジュール高さを数値確認できず</x:v>
+      </x:c>
+      <x:c r="P6" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q6" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R6" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S6" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T6" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U6" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V6" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W6" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="X6" s="25"/>
-      <x:c r="Y6" s="14"/>
-      <x:c r="Z6" s="25"/>
+      <x:c r="Y6" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z6" s="25" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
       <x:c r="AA6" s="14"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="22"/>
-      <x:c r="B7" s="14"/>
-      <x:c r="C7" s="14"/>
-      <x:c r="D7" s="14"/>
+      <x:c r="AB6" s="136" t="n">
+        <x:v>4800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
+      <x:c r="A7" s="22" t="str">
+        <x:v>memory-corsair-cmk32gx4m2e3200c16</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>Corsair</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>CMK32GX4M2E3200C16</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>Corsair VENGEANCE LPX DDR4-3200 32GB (16GB×2) CL16</x:v>
+      </x:c>
       <x:c r="E7" s="22"/>
       <x:c r="F7" s="22"/>
-      <x:c r="G7" s="22"/>
+      <x:c r="G7" s="22" t="str">
+        <x:v>CMK32GX4M2E3200C16</x:v>
+      </x:c>
       <x:c r="H7" s="22"/>
-      <x:c r="I7" s="14"/>
-      <x:c r="J7" s="14"/>
-      <x:c r="K7" s="14"/>
-      <x:c r="L7" s="23"/>
-      <x:c r="M7" s="14"/>
-      <x:c r="N7" s="14"/>
-      <x:c r="O7" s="14"/>
-      <x:c r="P7" s="14"/>
-      <x:c r="Q7" s="14"/>
-      <x:c r="R7" s="14"/>
-      <x:c r="S7" s="25"/>
-      <x:c r="T7" s="24"/>
-      <x:c r="U7" s="24"/>
-      <x:c r="V7" s="14"/>
-      <x:c r="W7" s="25"/>
+      <x:c r="I7" s="14" t="str">
+        <x:v>VENGEANCE LPX 32GB 3200 C16</x:v>
+      </x:c>
+      <x:c r="J7" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K7" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L7" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M7" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N7" s="14" t="str">
+        <x:v>DDR4-3200 CL16
+Intel XMP 2.0対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O7" s="14" t="str">
+        <x:v>AMD EXPO非対応
+公式商品ページでモジュール高さを数値確認できず</x:v>
+      </x:c>
+      <x:c r="P7" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q7" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R7" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S7" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T7" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U7" s="24" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="V7" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W7" s="25" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="X7" s="25"/>
-      <x:c r="Y7" s="14"/>
-      <x:c r="Z7" s="25"/>
+      <x:c r="Y7" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z7" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA7" s="14"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="22"/>
-      <x:c r="B8" s="14"/>
-      <x:c r="C8" s="14"/>
-      <x:c r="D8" s="14"/>
+      <x:c r="AB7" s="136" t="n">
+        <x:v>2133</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
+      <x:c r="A8" s="22" t="str">
+        <x:v>memory-corsair-cmk64gx4m2e3200c16</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>Corsair</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>CMK64GX4M2E3200C16</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>Corsair VENGEANCE LPX DDR4-3200 64GB (32GB×2) CL16</x:v>
+      </x:c>
       <x:c r="E8" s="22"/>
       <x:c r="F8" s="22"/>
-      <x:c r="G8" s="22"/>
+      <x:c r="G8" s="22" t="str">
+        <x:v>CMK64GX4M2E3200C16</x:v>
+      </x:c>
       <x:c r="H8" s="22"/>
-      <x:c r="I8" s="14"/>
-      <x:c r="J8" s="14"/>
-      <x:c r="K8" s="14"/>
-      <x:c r="L8" s="23"/>
-      <x:c r="M8" s="14"/>
-      <x:c r="N8" s="14"/>
-      <x:c r="O8" s="14"/>
-      <x:c r="P8" s="14"/>
-      <x:c r="Q8" s="14"/>
-      <x:c r="R8" s="14"/>
-      <x:c r="S8" s="25"/>
-      <x:c r="T8" s="24"/>
-      <x:c r="U8" s="24"/>
-      <x:c r="V8" s="14"/>
-      <x:c r="W8" s="25"/>
+      <x:c r="I8" s="14" t="str">
+        <x:v>VENGEANCE LPX 64GB 3200 C16</x:v>
+      </x:c>
+      <x:c r="J8" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K8" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L8" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M8" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N8" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR4-3200 CL16
+Intel XMP 2.0対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O8" s="14" t="str">
+        <x:v>AMD EXPO非対応
+32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける</x:v>
+      </x:c>
+      <x:c r="P8" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q8" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R8" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S8" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T8" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U8" s="24" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="V8" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W8" s="25" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="X8" s="25"/>
-      <x:c r="Y8" s="14"/>
-      <x:c r="Z8" s="25"/>
+      <x:c r="Y8" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z8" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA8" s="14"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="22"/>
-      <x:c r="B9" s="14"/>
-      <x:c r="C9" s="14"/>
-      <x:c r="D9" s="14"/>
+      <x:c r="AB8" s="136" t="n">
+        <x:v>2133</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="22" t="str">
+        <x:v>memory-gskill-f5-6000j3038f16gx2-fx5</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>G.SKILL</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>F5-6000J3038F16GX2-FX5</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>G.SKILL Flare X5 DDR5-6000 32GB (16GB×2) CL30</x:v>
+      </x:c>
       <x:c r="E9" s="22"/>
       <x:c r="F9" s="22"/>
-      <x:c r="G9" s="22"/>
+      <x:c r="G9" s="22" t="str">
+        <x:v>F5-6000J3038F16GX2-FX5</x:v>
+      </x:c>
       <x:c r="H9" s="22"/>
-      <x:c r="I9" s="14"/>
-      <x:c r="J9" s="14"/>
-      <x:c r="K9" s="14"/>
-      <x:c r="L9" s="23"/>
-      <x:c r="M9" s="14"/>
-      <x:c r="N9" s="14"/>
-      <x:c r="O9" s="14"/>
-      <x:c r="P9" s="14"/>
-      <x:c r="Q9" s="14"/>
-      <x:c r="R9" s="14"/>
-      <x:c r="S9" s="25"/>
-      <x:c r="T9" s="24"/>
-      <x:c r="U9" s="24"/>
-      <x:c r="V9" s="14"/>
-      <x:c r="W9" s="25"/>
+      <x:c r="I9" s="14" t="str">
+        <x:v>Flare X5 32GB DDR5-6000 CL30</x:v>
+      </x:c>
+      <x:c r="J9" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K9" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L9" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M9" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N9" s="14" t="str">
+        <x:v>DDR5-6000 CL30-38-38-96
+AMD EXPO対応
+公式EXPO自己認証レポートあり
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O9" s="14" t="str">
+        <x:v>定格動作はマザーボード・CPUの互換性に依存
+メモリキットの混在不可</x:v>
+      </x:c>
+      <x:c r="P9" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q9" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。
+SK hynix表記は公式EXPOレポートのModule Revision 1.0に対する情報で、将来の部品変更を保証しません。</x:v>
+      </x:c>
+      <x:c r="R9" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S9" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T9" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U9" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V9" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W9" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="X9" s="25"/>
-      <x:c r="Y9" s="14"/>
-      <x:c r="Z9" s="25"/>
-      <x:c r="AA9" s="14"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="22"/>
-      <x:c r="B10" s="14"/>
-      <x:c r="C10" s="14"/>
-      <x:c r="D10" s="14"/>
+      <x:c r="Y9" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z9" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="AA9" s="14" t="str">
+        <x:v>SK hynix (EXPO report rev.1.0)</x:v>
+      </x:c>
+      <x:c r="AB9" s="136" t="n">
+        <x:v>4800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="22" t="str">
+        <x:v>memory-gskill-f5-6000j3040g32gx2-fx5</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>G.SKILL</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>F5-6000J3040G32GX2-FX5</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>G.SKILL Flare X5 DDR5-6000 64GB (32GB×2) CL30</x:v>
+      </x:c>
       <x:c r="E10" s="22"/>
       <x:c r="F10" s="22"/>
-      <x:c r="G10" s="22"/>
+      <x:c r="G10" s="22" t="str">
+        <x:v>F5-6000J3040G32GX2-FX5</x:v>
+      </x:c>
       <x:c r="H10" s="22"/>
-      <x:c r="I10" s="14"/>
-      <x:c r="J10" s="14"/>
-      <x:c r="K10" s="14"/>
-      <x:c r="L10" s="23"/>
-      <x:c r="M10" s="14"/>
-      <x:c r="N10" s="14"/>
-      <x:c r="O10" s="14"/>
-      <x:c r="P10" s="14"/>
-      <x:c r="Q10" s="14"/>
-      <x:c r="R10" s="14"/>
-      <x:c r="S10" s="25"/>
-      <x:c r="T10" s="24"/>
-      <x:c r="U10" s="24"/>
-      <x:c r="V10" s="14"/>
-      <x:c r="W10" s="25"/>
+      <x:c r="I10" s="14" t="str">
+        <x:v>Flare X5 64GB DDR5-6000 CL30</x:v>
+      </x:c>
+      <x:c r="J10" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K10" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L10" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M10" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N10" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR5-6000 CL30-40-40-96
+AMD EXPO・Intel XMP 3.0対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O10" s="14" t="str">
+        <x:v>32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける
+メモリキットの混在不可</x:v>
+      </x:c>
+      <x:c r="P10" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q10" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R10" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S10" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T10" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U10" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V10" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W10" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="X10" s="25"/>
-      <x:c r="Y10" s="14"/>
-      <x:c r="Z10" s="25"/>
+      <x:c r="Y10" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z10" s="25" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
       <x:c r="AA10" s="14"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="22"/>
-      <x:c r="B11" s="14"/>
-      <x:c r="C11" s="14"/>
-      <x:c r="D11" s="14"/>
+      <x:c r="AB10" s="136" t="n">
+        <x:v>4800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="52" customHeight="1">
+      <x:c r="A11" s="22" t="str">
+        <x:v>memory-gskill-f4-3600c16d-32gvkc</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>G.SKILL</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>F4-3600C16D-32GVKC</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>G.SKILL Ripjaws V DDR4-3600 32GB (16GB×2) CL16</x:v>
+      </x:c>
       <x:c r="E11" s="22"/>
       <x:c r="F11" s="22"/>
-      <x:c r="G11" s="22"/>
+      <x:c r="G11" s="22" t="str">
+        <x:v>F4-3600C16D-32GVKC</x:v>
+      </x:c>
       <x:c r="H11" s="22"/>
-      <x:c r="I11" s="14"/>
-      <x:c r="J11" s="14"/>
-      <x:c r="K11" s="14"/>
-      <x:c r="L11" s="23"/>
-      <x:c r="M11" s="14"/>
-      <x:c r="N11" s="14"/>
-      <x:c r="O11" s="14"/>
-      <x:c r="P11" s="14"/>
-      <x:c r="Q11" s="14"/>
-      <x:c r="R11" s="14"/>
-      <x:c r="S11" s="25"/>
-      <x:c r="T11" s="24"/>
-      <x:c r="U11" s="24"/>
-      <x:c r="V11" s="14"/>
-      <x:c r="W11" s="25"/>
+      <x:c r="I11" s="14" t="str">
+        <x:v>Ripjaws V 32GB DDR4-3600 CL16</x:v>
+      </x:c>
+      <x:c r="J11" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K11" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L11" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M11" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N11" s="14" t="str">
+        <x:v>DDR4-3600 CL16-19-19-39
+Intel XMP 2.0対応
+公式QVLあり
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O11" s="14" t="str">
+        <x:v>AMD EXPO非対応
+定格動作はQVL・CPU IMC・BIOSに依存
+メモリキットの混在不可</x:v>
+      </x:c>
+      <x:c r="P11" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q11" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R11" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S11" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T11" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U11" s="24" t="n">
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="V11" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W11" s="25" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="X11" s="25"/>
-      <x:c r="Y11" s="14"/>
-      <x:c r="Z11" s="25"/>
+      <x:c r="Y11" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z11" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA11" s="14"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="22"/>
-      <x:c r="B12" s="14"/>
-      <x:c r="C12" s="14"/>
-      <x:c r="D12" s="14"/>
+      <x:c r="AB11" s="136" t="n">
+        <x:v>2133</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="52" customHeight="1">
+      <x:c r="A12" s="22" t="str">
+        <x:v>memory-gskill-f4-3600c18d-64gvk</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>G.SKILL</x:v>
+      </x:c>
+      <x:c r="C12" s="14" t="str">
+        <x:v>F4-3600C18D-64GVK</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>G.SKILL Ripjaws V DDR4-3600 64GB (32GB×2) CL18</x:v>
+      </x:c>
       <x:c r="E12" s="22"/>
       <x:c r="F12" s="22"/>
-      <x:c r="G12" s="22"/>
+      <x:c r="G12" s="22" t="str">
+        <x:v>F4-3600C18D-64GVK</x:v>
+      </x:c>
       <x:c r="H12" s="22"/>
-      <x:c r="I12" s="14"/>
-      <x:c r="J12" s="14"/>
-      <x:c r="K12" s="14"/>
-      <x:c r="L12" s="23"/>
-      <x:c r="M12" s="14"/>
-      <x:c r="N12" s="14"/>
-      <x:c r="O12" s="14"/>
-      <x:c r="P12" s="14"/>
-      <x:c r="Q12" s="14"/>
-      <x:c r="R12" s="14"/>
-      <x:c r="S12" s="25"/>
-      <x:c r="T12" s="24"/>
-      <x:c r="U12" s="24"/>
-      <x:c r="V12" s="14"/>
-      <x:c r="W12" s="25"/>
+      <x:c r="I12" s="14" t="str">
+        <x:v>Ripjaws V 64GB DDR4-3600 CL18</x:v>
+      </x:c>
+      <x:c r="J12" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K12" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L12" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M12" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N12" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR4-3600 CL18-22-22-42
+Intel XMP 2.0対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O12" s="14" t="str">
+        <x:v>AMD EXPO非対応
+32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける
+メモリキットの混在不可</x:v>
+      </x:c>
+      <x:c r="P12" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q12" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R12" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S12" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T12" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U12" s="24" t="n">
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="V12" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W12" s="25" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="X12" s="25"/>
-      <x:c r="Y12" s="14"/>
-      <x:c r="Z12" s="25"/>
+      <x:c r="Y12" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z12" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA12" s="14"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="22"/>
-      <x:c r="B13" s="14"/>
-      <x:c r="C13" s="14"/>
-      <x:c r="D13" s="14"/>
+      <x:c r="AB12" s="136" t="n">
+        <x:v>2666</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="52" customHeight="1">
+      <x:c r="A13" s="22" t="str">
+        <x:v>memory-kingston-kf560c30bbek2-32</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>Kingston</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>KF560C30BBEK2-32</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Kingston FURY Beast DDR5-6000 32GB (16GB×2) CL30 EXPO</x:v>
+      </x:c>
       <x:c r="E13" s="22"/>
       <x:c r="F13" s="22"/>
-      <x:c r="G13" s="22"/>
+      <x:c r="G13" s="22" t="str">
+        <x:v>KF560C30BBEK2-32</x:v>
+      </x:c>
       <x:c r="H13" s="22"/>
-      <x:c r="I13" s="14"/>
-      <x:c r="J13" s="14"/>
-      <x:c r="K13" s="14"/>
-      <x:c r="L13" s="23"/>
-      <x:c r="M13" s="14"/>
-      <x:c r="N13" s="14"/>
-      <x:c r="O13" s="14"/>
-      <x:c r="P13" s="14"/>
-      <x:c r="Q13" s="14"/>
-      <x:c r="R13" s="14"/>
-      <x:c r="S13" s="25"/>
-      <x:c r="T13" s="24"/>
-      <x:c r="U13" s="24"/>
-      <x:c r="V13" s="14"/>
-      <x:c r="W13" s="25"/>
-      <x:c r="X13" s="25"/>
-      <x:c r="Y13" s="14"/>
-      <x:c r="Z13" s="25"/>
+      <x:c r="I13" s="14" t="str">
+        <x:v>FURY Beast 32GB DDR5-6000 CL30 EXPO</x:v>
+      </x:c>
+      <x:c r="J13" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K13" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L13" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M13" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N13" s="14" t="str">
+        <x:v>DDR5-6000 CL30-36-36
+AMD EXPO 1.1・Intel XMP 3.0対応
+高さ34.9mm
+製品寿命保証</x:v>
+      </x:c>
+      <x:c r="O13" s="14" t="str">
+        <x:v>定格動作にはプロファイル有効化と対応プラットフォームが必要</x:v>
+      </x:c>
+      <x:c r="P13" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q13" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。
+公式データシートの当該リビジョンでは1Rx8。</x:v>
+      </x:c>
+      <x:c r="R13" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S13" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T13" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U13" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V13" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W13" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="X13" s="25" t="n">
+        <x:v>34.9</x:v>
+      </x:c>
+      <x:c r="Y13" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z13" s="25" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
       <x:c r="AA13" s="14"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="22"/>
-      <x:c r="B14" s="14"/>
-      <x:c r="C14" s="14"/>
-      <x:c r="D14" s="14"/>
+      <x:c r="AB13" s="136" t="n">
+        <x:v>4800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="52" customHeight="1">
+      <x:c r="A14" s="22" t="str">
+        <x:v>memory-kingston-kf560c30bbek2-64</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>Kingston</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>KF560C30BBEK2-64</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Kingston FURY Beast DDR5-6000 64GB (32GB×2) CL30 EXPO</x:v>
+      </x:c>
       <x:c r="E14" s="22"/>
       <x:c r="F14" s="22"/>
-      <x:c r="G14" s="22"/>
+      <x:c r="G14" s="22" t="str">
+        <x:v>KF560C30BBEK2-64</x:v>
+      </x:c>
       <x:c r="H14" s="22"/>
-      <x:c r="I14" s="14"/>
-      <x:c r="J14" s="14"/>
-      <x:c r="K14" s="14"/>
-      <x:c r="L14" s="23"/>
-      <x:c r="M14" s="14"/>
-      <x:c r="N14" s="14"/>
-      <x:c r="O14" s="14"/>
-      <x:c r="P14" s="14"/>
-      <x:c r="Q14" s="14"/>
-      <x:c r="R14" s="14"/>
-      <x:c r="S14" s="25"/>
-      <x:c r="T14" s="24"/>
-      <x:c r="U14" s="24"/>
-      <x:c r="V14" s="14"/>
-      <x:c r="W14" s="25"/>
-      <x:c r="X14" s="25"/>
-      <x:c r="Y14" s="14"/>
-      <x:c r="Z14" s="25"/>
+      <x:c r="I14" s="14" t="str">
+        <x:v>FURY Beast 64GB DDR5-6000 CL30 EXPO</x:v>
+      </x:c>
+      <x:c r="J14" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K14" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L14" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M14" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N14" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR5-6000 CL30-36-36
+AMD EXPO 1.1・Intel XMP 3.0対応
+高さ34.9mm
+製品寿命保証</x:v>
+      </x:c>
+      <x:c r="O14" s="14" t="str">
+        <x:v>32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける</x:v>
+      </x:c>
+      <x:c r="P14" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q14" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。
+公式データシートの当該リビジョンでは2Rx8。</x:v>
+      </x:c>
+      <x:c r="R14" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S14" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T14" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U14" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V14" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W14" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="X14" s="25" t="n">
+        <x:v>34.9</x:v>
+      </x:c>
+      <x:c r="Y14" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z14" s="25" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
       <x:c r="AA14" s="14"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="22"/>
-      <x:c r="B15" s="14"/>
-      <x:c r="C15" s="14"/>
-      <x:c r="D15" s="14"/>
+      <x:c r="AB14" s="136" t="n">
+        <x:v>4800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="52" customHeight="1">
+      <x:c r="A15" s="22" t="str">
+        <x:v>memory-kingston-kf432c16bbk2-32</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>Kingston</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>KF432C16BBK2/32</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Kingston FURY Beast DDR4-3200 32GB (16GB×2) CL16</x:v>
+      </x:c>
       <x:c r="E15" s="22"/>
       <x:c r="F15" s="22"/>
-      <x:c r="G15" s="22"/>
+      <x:c r="G15" s="22" t="str">
+        <x:v>KF432C16BBK2/32</x:v>
+      </x:c>
       <x:c r="H15" s="22"/>
-      <x:c r="I15" s="14"/>
-      <x:c r="J15" s="14"/>
-      <x:c r="K15" s="14"/>
-      <x:c r="L15" s="23"/>
-      <x:c r="M15" s="14"/>
-      <x:c r="N15" s="14"/>
-      <x:c r="O15" s="14"/>
-      <x:c r="P15" s="14"/>
-      <x:c r="Q15" s="14"/>
-      <x:c r="R15" s="14"/>
-      <x:c r="S15" s="25"/>
-      <x:c r="T15" s="24"/>
-      <x:c r="U15" s="24"/>
-      <x:c r="V15" s="14"/>
-      <x:c r="W15" s="25"/>
-      <x:c r="X15" s="25"/>
-      <x:c r="Y15" s="14"/>
-      <x:c r="Z15" s="25"/>
+      <x:c r="I15" s="14" t="str">
+        <x:v>FURY Beast 32GB DDR4-3200 CL16</x:v>
+      </x:c>
+      <x:c r="J15" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K15" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L15" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M15" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N15" s="14" t="str">
+        <x:v>DDR4-3200 CL16-20-20
+Intel XMP 2.0対応
+高さ34mm
+製品寿命保証</x:v>
+      </x:c>
+      <x:c r="O15" s="14" t="str">
+        <x:v>AMD EXPO非対応
+定格動作はマザーボード・CPUの互換性に依存</x:v>
+      </x:c>
+      <x:c r="P15" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q15" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。
+公式データシートの当該リビジョンでは1Rx8。</x:v>
+      </x:c>
+      <x:c r="R15" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S15" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T15" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U15" s="24" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="V15" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W15" s="25" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="X15" s="25" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="Y15" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z15" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA15" s="14"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="22"/>
-      <x:c r="B16" s="14"/>
-      <x:c r="C16" s="14"/>
-      <x:c r="D16" s="14"/>
+      <x:c r="AB15" s="136" t="n">
+        <x:v>2400</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="52" customHeight="1">
+      <x:c r="A16" s="22" t="str">
+        <x:v>memory-kingston-kf432c16bbk2-64</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>Kingston</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>KF432C16BBK2/64</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Kingston FURY Beast DDR4-3200 64GB (32GB×2) CL16</x:v>
+      </x:c>
       <x:c r="E16" s="22"/>
       <x:c r="F16" s="22"/>
-      <x:c r="G16" s="22"/>
+      <x:c r="G16" s="22" t="str">
+        <x:v>KF432C16BBK2/64</x:v>
+      </x:c>
       <x:c r="H16" s="22"/>
-      <x:c r="I16" s="14"/>
-      <x:c r="J16" s="14"/>
-      <x:c r="K16" s="14"/>
-      <x:c r="L16" s="23"/>
-      <x:c r="M16" s="14"/>
-      <x:c r="N16" s="14"/>
-      <x:c r="O16" s="14"/>
-      <x:c r="P16" s="14"/>
-      <x:c r="Q16" s="14"/>
-      <x:c r="R16" s="14"/>
-      <x:c r="S16" s="25"/>
-      <x:c r="T16" s="24"/>
-      <x:c r="U16" s="24"/>
-      <x:c r="V16" s="14"/>
-      <x:c r="W16" s="25"/>
-      <x:c r="X16" s="25"/>
-      <x:c r="Y16" s="14"/>
-      <x:c r="Z16" s="25"/>
+      <x:c r="I16" s="14" t="str">
+        <x:v>FURY Beast 64GB DDR4-3200 CL16</x:v>
+      </x:c>
+      <x:c r="J16" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K16" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L16" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M16" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N16" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR4-3200 CL16-20-20
+Intel XMP 2.0対応
+高さ34mm
+製品寿命保証</x:v>
+      </x:c>
+      <x:c r="O16" s="14" t="str">
+        <x:v>AMD EXPO非対応
+32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける</x:v>
+      </x:c>
+      <x:c r="P16" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q16" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。
+公式データシートの当該リビジョンでは2Rx8。</x:v>
+      </x:c>
+      <x:c r="R16" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S16" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T16" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U16" s="24" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="V16" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W16" s="25" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="X16" s="25" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="Y16" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z16" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA16" s="14"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="22"/>
-      <x:c r="B17" s="14"/>
-      <x:c r="C17" s="14"/>
-      <x:c r="D17" s="14"/>
+      <x:c r="AB16" s="136" t="n">
+        <x:v>2400</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="52" customHeight="1">
+      <x:c r="A17" s="22" t="str">
+        <x:v>memory-crucial-cp2k16g60c36u5b</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>Crucial</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>CP2K16G60C36U5B</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Crucial Pro OC DDR5-6000 32GB (16GB×2) CL36</x:v>
+      </x:c>
       <x:c r="E17" s="22"/>
       <x:c r="F17" s="22"/>
-      <x:c r="G17" s="22"/>
+      <x:c r="G17" s="22" t="str">
+        <x:v>CP2K16G60C36U5B</x:v>
+      </x:c>
       <x:c r="H17" s="22"/>
-      <x:c r="I17" s="14"/>
-      <x:c r="J17" s="14"/>
-      <x:c r="K17" s="14"/>
-      <x:c r="L17" s="23"/>
-      <x:c r="M17" s="14"/>
-      <x:c r="N17" s="14"/>
-      <x:c r="O17" s="14"/>
-      <x:c r="P17" s="14"/>
-      <x:c r="Q17" s="14"/>
-      <x:c r="R17" s="14"/>
-      <x:c r="S17" s="25"/>
-      <x:c r="T17" s="24"/>
-      <x:c r="U17" s="24"/>
-      <x:c r="V17" s="14"/>
-      <x:c r="W17" s="25"/>
+      <x:c r="I17" s="14" t="str">
+        <x:v>Crucial Pro Overclocking 32GB DDR5-6000 CL36</x:v>
+      </x:c>
+      <x:c r="J17" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K17" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L17" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M17" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N17" s="14" t="str">
+        <x:v>DDR5-6000 CL36-38-38-80
+Intel XMP 3.0・AMD EXPO対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O17" s="14" t="str">
+        <x:v>CL36のため既存AM5 CL32以下優先条件では加点対象外
+公式商品ページでモジュール高さを数値確認できず</x:v>
+      </x:c>
+      <x:c r="P17" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q17" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R17" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S17" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T17" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U17" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V17" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W17" s="25" t="n">
+        <x:v>36</x:v>
+      </x:c>
       <x:c r="X17" s="25"/>
-      <x:c r="Y17" s="14"/>
-      <x:c r="Z17" s="25"/>
+      <x:c r="Y17" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z17" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA17" s="14"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="22"/>
-      <x:c r="B18" s="14"/>
-      <x:c r="C18" s="14"/>
-      <x:c r="D18" s="14"/>
+      <x:c r="AB17" s="136" t="n">
+        <x:v>5600</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="52" customHeight="1">
+      <x:c r="A18" s="22" t="str">
+        <x:v>memory-crucial-cp2k32g60c40u5b</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>Crucial</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>CP2K32G60C40U5B</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>Crucial Pro OC DDR5-6000 64GB (32GB×2) CL40</x:v>
+      </x:c>
       <x:c r="E18" s="22"/>
       <x:c r="F18" s="22"/>
-      <x:c r="G18" s="22"/>
+      <x:c r="G18" s="22" t="str">
+        <x:v>CP2K32G60C40U5B</x:v>
+      </x:c>
       <x:c r="H18" s="22"/>
-      <x:c r="I18" s="14"/>
-      <x:c r="J18" s="14"/>
-      <x:c r="K18" s="14"/>
-      <x:c r="L18" s="23"/>
-      <x:c r="M18" s="14"/>
-      <x:c r="N18" s="14"/>
-      <x:c r="O18" s="14"/>
-      <x:c r="P18" s="14"/>
-      <x:c r="Q18" s="14"/>
-      <x:c r="R18" s="14"/>
-      <x:c r="S18" s="25"/>
-      <x:c r="T18" s="24"/>
-      <x:c r="U18" s="24"/>
-      <x:c r="V18" s="14"/>
-      <x:c r="W18" s="25"/>
+      <x:c r="I18" s="14" t="str">
+        <x:v>Crucial Pro Overclocking 64GB DDR5-6000 CL40</x:v>
+      </x:c>
+      <x:c r="J18" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K18" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L18" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M18" s="14" t="str">
+        <x:v>公式仕様を確認したDDR5デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N18" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR5-6000 CL40
+Intel XMP 3.0・AMD EXPO対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O18" s="14" t="str">
+        <x:v>CL40のため既存AM5 CL32以下優先条件では加点対象外
+32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける</x:v>
+      </x:c>
+      <x:c r="P18" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q18" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R18" s="14" t="str">
+        <x:v>DDR5</x:v>
+      </x:c>
+      <x:c r="S18" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T18" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U18" s="24" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="V18" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W18" s="25" t="n">
+        <x:v>40</x:v>
+      </x:c>
       <x:c r="X18" s="25"/>
-      <x:c r="Y18" s="14"/>
-      <x:c r="Z18" s="25"/>
+      <x:c r="Y18" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z18" s="25" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
       <x:c r="AA18" s="14"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="22"/>
-      <x:c r="B19" s="14"/>
-      <x:c r="C19" s="14"/>
-      <x:c r="D19" s="14"/>
+      <x:c r="AB18" s="136" t="n">
+        <x:v>5600</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="52" customHeight="1">
+      <x:c r="A19" s="22" t="str">
+        <x:v>memory-crucial-cp2k16g4dfra32a</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>Crucial</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>CP2K16G4DFRA32A</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Crucial Pro DDR4-3200 32GB (16GB×2) CL22</x:v>
+      </x:c>
       <x:c r="E19" s="22"/>
       <x:c r="F19" s="22"/>
-      <x:c r="G19" s="22"/>
+      <x:c r="G19" s="22" t="str">
+        <x:v>CP2K16G4DFRA32A</x:v>
+      </x:c>
       <x:c r="H19" s="22"/>
-      <x:c r="I19" s="14"/>
-      <x:c r="J19" s="14"/>
-      <x:c r="K19" s="14"/>
-      <x:c r="L19" s="23"/>
-      <x:c r="M19" s="14"/>
-      <x:c r="N19" s="14"/>
-      <x:c r="O19" s="14"/>
-      <x:c r="P19" s="14"/>
-      <x:c r="Q19" s="14"/>
-      <x:c r="R19" s="14"/>
-      <x:c r="S19" s="25"/>
-      <x:c r="T19" s="24"/>
-      <x:c r="U19" s="24"/>
-      <x:c r="V19" s="14"/>
-      <x:c r="W19" s="25"/>
+      <x:c r="I19" s="14" t="str">
+        <x:v>Crucial Pro 32GB DDR4-3200</x:v>
+      </x:c>
+      <x:c r="J19" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L19" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M19" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N19" s="14" t="str">
+        <x:v>DDR4-3200 CL22
+JEDEC定格1.2V
+Intel XMP 2.0対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O19" s="14" t="str">
+        <x:v>AMD EXPO非対応
+CL16製品よりレイテンシが大きい
+公式商品ページでモジュール高さを数値確認できず</x:v>
+      </x:c>
+      <x:c r="P19" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q19" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R19" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S19" s="25" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="T19" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U19" s="24" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="V19" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W19" s="25" t="n">
+        <x:v>22</x:v>
+      </x:c>
       <x:c r="X19" s="25"/>
-      <x:c r="Y19" s="14"/>
-      <x:c r="Z19" s="25"/>
+      <x:c r="Y19" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z19" s="25" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
       <x:c r="AA19" s="14"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="22"/>
-      <x:c r="B20" s="14"/>
-      <x:c r="C20" s="14"/>
-      <x:c r="D20" s="14"/>
+      <x:c r="AB19" s="136" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52" customHeight="1">
+      <x:c r="A20" s="22" t="str">
+        <x:v>memory-crucial-cp2k32g4dfra32a</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Crucial</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>CP2K32G4DFRA32A</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>Crucial Pro DDR4-3200 64GB (32GB×2) CL22</x:v>
+      </x:c>
       <x:c r="E20" s="22"/>
       <x:c r="F20" s="22"/>
-      <x:c r="G20" s="22"/>
+      <x:c r="G20" s="22" t="str">
+        <x:v>CP2K32G4DFRA32A</x:v>
+      </x:c>
       <x:c r="H20" s="22"/>
-      <x:c r="I20" s="14"/>
-      <x:c r="J20" s="14"/>
-      <x:c r="K20" s="14"/>
-      <x:c r="L20" s="23"/>
-      <x:c r="M20" s="14"/>
-      <x:c r="N20" s="14"/>
-      <x:c r="O20" s="14"/>
-      <x:c r="P20" s="14"/>
-      <x:c r="Q20" s="14"/>
-      <x:c r="R20" s="14"/>
-      <x:c r="S20" s="25"/>
-      <x:c r="T20" s="24"/>
-      <x:c r="U20" s="24"/>
-      <x:c r="V20" s="14"/>
-      <x:c r="W20" s="25"/>
+      <x:c r="I20" s="14" t="str">
+        <x:v>Crucial Pro 64GB DDR4-3200</x:v>
+      </x:c>
+      <x:c r="J20" s="14" t="str">
+        <x:v>research_required</x:v>
+      </x:c>
+      <x:c r="K20" s="14" t="str">
+        <x:v>unrated</x:v>
+      </x:c>
+      <x:c r="L20" s="23" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="M20" s="14" t="str">
+        <x:v>公式仕様を確認したDDR4デュアルチャネルキット。国内流通SKU、独立レビュー、QVL確認前の調査中レコードです。</x:v>
+      </x:c>
+      <x:c r="N20" s="14" t="str">
+        <x:v>64GBを2枚で構成
+DDR4-3200 CL22
+JEDEC定格1.2V
+Intel XMP 2.0対応
+限定永久保証</x:v>
+      </x:c>
+      <x:c r="O20" s="14" t="str">
+        <x:v>AMD EXPO非対応
+CL16製品よりレイテンシが大きい
+32GBモジュール2枚の定格動作はCPU IMCとBIOSの影響を受ける</x:v>
+      </x:c>
+      <x:c r="P20" s="14" t="str">
+        <x:v>XMP/EXPO定格はCPU IMC・マザーボード・BIOS依存。DRAM IC・ランク・基板リビジョンは購入時期で変わる可能性があります。</x:v>
+      </x:c>
+      <x:c r="Q20" s="14" t="str">
+        <x:v>ASIN・JAN・国内保証窓口は未確定。購入前に完全型番、マザーボードQVL、CPUの対応速度、クーラーとの干渉、販売店の保証条件を確認してください。</x:v>
+      </x:c>
+      <x:c r="R20" s="14" t="str">
+        <x:v>DDR4</x:v>
+      </x:c>
+      <x:c r="S20" s="25" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="T20" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="U20" s="24" t="n">
+        <x:v>3200</x:v>
+      </x:c>
+      <x:c r="V20" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W20" s="25" t="n">
+        <x:v>22</x:v>
+      </x:c>
       <x:c r="X20" s="25"/>
-      <x:c r="Y20" s="14"/>
-      <x:c r="Z20" s="25"/>
+      <x:c r="Y20" s="14" t="str">
+        <x:v>limited_lifetime</x:v>
+      </x:c>
+      <x:c r="Z20" s="25" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
       <x:c r="AA20" s="14"/>
+      <x:c r="AB20" s="136" t="n">
+        <x:v>3200</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="22"/>
@@ -46051,6 +47358,7 @@
       <x:c r="Y21" s="14"/>
       <x:c r="Z21" s="25"/>
       <x:c r="AA21" s="14"/>
+      <x:c r="AB21" s="136"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="22"/>
@@ -46080,6 +47388,7 @@
       <x:c r="Y22" s="14"/>
       <x:c r="Z22" s="25"/>
       <x:c r="AA22" s="14"/>
+      <x:c r="AB22" s="136"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22"/>
@@ -46109,6 +47418,7 @@
       <x:c r="Y23" s="14"/>
       <x:c r="Z23" s="25"/>
       <x:c r="AA23" s="14"/>
+      <x:c r="AB23" s="136"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="22"/>
@@ -46138,6 +47448,7 @@
       <x:c r="Y24" s="14"/>
       <x:c r="Z24" s="25"/>
       <x:c r="AA24" s="14"/>
+      <x:c r="AB24" s="136"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -46168,7 +47479,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R012ff84d6dfe4ee3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf219b6e74bce404c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47047,7 +48358,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7ee230b1a24923"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R536991f5925048da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47880,7 +49191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62d95a28f4014403"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R793b1e3dbd44428a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -48759,7 +50070,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2152620cd1ef480e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5747c7d55d54c33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49664,7 +50975,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f62067fc137430b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9a4fd68dd0d4e08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add GPU performance comparison view
</commit_message>
<xml_diff>
--- a/catalog/quality_catalog.xlsx
+++ b/catalog/quality_catalog.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rdb47fdf3e506452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search" sheetId="2" r:id="Rcae53701eef14f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="3" r:id="R13bb1ac7d66c45ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="4" r:id="R605ccadd928b4d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPUChips" sheetId="19" r:id="R1e285574938743fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="5" r:id="R8483731e3a5e47d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="6" r:id="Re80fecb7801c48f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PSU" sheetId="7" r:id="R2d563cc61efe4f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motherboard" sheetId="8" r:id="Rf1a890badbe744ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitor" sheetId="9" r:id="R594f07d50edf476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifiers" sheetId="10" r:id="R0d26252080f2491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="11" r:id="Rb7856801d6d943dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="12" r:id="Rf577cd256eb84b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="13" r:id="Rf19f5fe339c24956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="14" r:id="R85f2b556a98145c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" r:id="R22ee9d55f7614a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SheetDefinitions" sheetId="16" r:id="R197623603af24e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDefinitions" sheetId="17" r:id="Rab74da8ada294c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" r:id="R95f718ec2e954b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rb99fcd473a8d48d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search" sheetId="2" r:id="R3c4ac796611047f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPU" sheetId="3" r:id="R93b1f4a9bc804230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU" sheetId="4" r:id="R30fdda71ec824336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPUChips" sheetId="19" r:id="R8cb0c0ac56034f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory" sheetId="5" r:id="R43edea59c6be4c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SSD" sheetId="6" r:id="Ra576b379588f47af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PSU" sheetId="7" r:id="Rb4303eb037e441d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motherboard" sheetId="8" r:id="R00cfb859e29e4e6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitor" sheetId="9" r:id="Rec92970838ba4ab8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifiers" sheetId="10" r:id="R2401696b1daa4a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="11" r:id="R1e4861393aeb442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="12" r:id="R7d2dd907a64f4de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="13" r:id="R1631937def274920"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="14" r:id="R395ba227b6c8409e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="15" r:id="R6954a39527974299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SheetDefinitions" sheetId="16" r:id="R237716bc1d964b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldDefinitions" sheetId="17" r:id="Raafca534760c4280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="18" r:id="R72c2be2ccd9e40ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39,7 +39,7 @@
     <x:numFmt numFmtId="204" formatCode="0"/>
     <x:numFmt numFmtId="205" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -94,8 +94,25 @@
       <x:color rgb="FF1F1F1F"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF4B275F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF274E13"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -192,6 +209,46 @@
         <x:fgColor rgb="FF2F75B5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4B275F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4DFEC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF8064A2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF008C95"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="7">
     <x:border/>
@@ -253,7 +310,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="138">
+  <x:cellXfs count="176">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -572,6 +629,92 @@
     </x:xf>
     <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2523,7 +2666,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b1c29721d88406f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4e2abb0b158421a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2967,7 +3110,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7318fc65705b4aa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf208c6fceee48cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17175,7 +17318,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ec6c9b012948cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770d75b572ee49d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17797,7 +17940,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2aefac450bc4dad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112019efb7254290"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18479,7 +18622,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cfc7b912eca4681"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf220824bb03347fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20438,7 +20581,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf1db422ac8a4757"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rced61d7ab3c64647"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20561,7 +20704,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87e5854388fb41e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d014df068f4405b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20825,7 +20968,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ed2e6f366614c6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53a9531cbb4f4fc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27473,7 +27616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88f4cddea4d249cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f59e998085f4d9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27518,6 +27661,8 @@
     <x:col min="34" max="34" width="18" hidden="0" customWidth="1"/>
     <x:col min="35" max="35" width="18" hidden="0" customWidth="1"/>
     <x:col min="36" max="36" width="18" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="20" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -27709,6 +27854,12 @@
       <x:c r="AJ4" s="8" t="str">
         <x:v>PanelType</x:v>
       </x:c>
+      <x:c r="AK4" s="172" t="str">
+        <x:v>GPUPerformanceClass</x:v>
+      </x:c>
+      <x:c r="AL4" s="172" t="str">
+        <x:v>MinRelativeIndex</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -27819,6 +27970,12 @@
       <x:c r="AJ5" t="str">
         <x:v>IPS</x:v>
       </x:c>
+      <x:c r="AK5" s="174" t="str">
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AL5" s="175" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
@@ -27929,6 +28086,12 @@
       <x:c r="AJ6" t="str">
         <x:v>Fast IPS</x:v>
       </x:c>
+      <x:c r="AK6" s="174" t="str">
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AL6" s="175" t="n">
+        <x:v>75</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -28032,6 +28195,12 @@
       </x:c>
       <x:c r="AJ7" t="str">
         <x:v>Nano IPS</x:v>
+      </x:c>
+      <x:c r="AK7" s="174" t="str">
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AL7" s="175" t="n">
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -28130,6 +28299,12 @@
       </x:c>
       <x:c r="AJ8" t="str">
         <x:v>VA</x:v>
+      </x:c>
+      <x:c r="AK8" s="174" t="str">
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AL8" s="175" t="n">
+        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -28210,6 +28385,12 @@
       </x:c>
       <x:c r="AJ9" t="str">
         <x:v>TN</x:v>
+      </x:c>
+      <x:c r="AK9" s="174" t="str">
+        <x:v>フラッグシップ</x:v>
+      </x:c>
+      <x:c r="AL9" s="175" t="n">
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -28487,7 +28668,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raca187b0b0604b38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e23a9ece59845f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41808,7 +41989,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20ef99cbd1a4f7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ee33f610bb4c58"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -48286,7 +48467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69597ed2e8e54c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R532c7f9ecc894e12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -48320,6 +48501,10 @@
     <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="15" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="20" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="13" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="17" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -48398,10 +48583,16 @@
       <x:c r="Y1" s="108" t="str">
         <x:v>GPUチップ 性能カタログ</x:v>
       </x:c>
+      <x:c r="Z1" s="141" t="str">
+        <x:v>GPU性能 比較ビュー（自動計算）</x:v>
+      </x:c>
+      <x:c r="AA1" s="141"/>
+      <x:c r="AB1" s="141"/>
+      <x:c r="AC1" s="141"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="111" t="str">
-        <x:v>Radeon RX 6000以降とGeForce RTXシリーズのデスクトップ向け基準データです。価格商品ではなく、ボードSKUから参照する性能・VRAM情報として使用します。</x:v>
+        <x:v>Radeon RX 6000以降とGeForce RTXシリーズのデスクトップ向け基準データです。PassMark生値に加え、右側の自動計算ビューで相対性能・順位・性能帯・G3D/Wを比較できます。価格商品ではなく、ボードSKUから参照する性能・VRAM情報として使用します。</x:v>
       </x:c>
       <x:c r="B2" s="111" t="str">
         <x:v>Radeon RX 6000以降とGeForce RTXシリーズのデスクトップ向け基準データです。価格商品ではなく、ボードSKUから参照する性能・VRAM情報として使用します。</x:v>
@@ -48475,6 +48666,22 @@
       <x:c r="Y2" s="111" t="str">
         <x:v>Radeon RX 6000以降とGeForce RTXシリーズのデスクトップ向け基準データです。価格商品ではなく、ボードSKUから参照する性能・VRAM情報として使用します。</x:v>
       </x:c>
+      <x:c r="Z2" s="145" t="str">
+        <x:v>PassMark G3Dから算出。実ゲームFPS・レイトレーシング性能ではありません。性能帯しきい値はListsで変更できます。</x:v>
+      </x:c>
+      <x:c r="AA2" s="145"/>
+      <x:c r="AB2" s="145"/>
+      <x:c r="AC2" s="145"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="Z3" s="149" t="str">
+        <x:v>基準GPU ID</x:v>
+      </x:c>
+      <x:c r="AA3" s="153" t="str">
+        <x:v>nvidia-geforce-rtx-4060</x:v>
+      </x:c>
+      <x:c r="AB3" s="153"/>
+      <x:c r="AC3" s="153"/>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="116" t="str">
@@ -48551,6 +48758,18 @@
       </x:c>
       <x:c r="Y4" s="116" t="str">
         <x:v>passmark_checked_at</x:v>
+      </x:c>
+      <x:c r="Z4" s="158" t="str">
+        <x:v>performance_index_rtx4060_100</x:v>
+      </x:c>
+      <x:c r="AA4" s="158" t="str">
+        <x:v>performance_rank</x:v>
+      </x:c>
+      <x:c r="AB4" s="158" t="str">
+        <x:v>performance_class</x:v>
+      </x:c>
+      <x:c r="AC4" s="158" t="str">
+        <x:v>passmark_g3d_per_watt</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
@@ -48625,6 +48844,22 @@
       <x:c r="Y5" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z5" s="164" t="n">
+        <x:f>IF(A5="","",ROUND(V5/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>39.7</x:v>
+      </x:c>
+      <x:c r="AA5" s="166" t="n">
+        <x:f>IF(V5="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V5)+1)</x:f>
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="AB5" s="162" t="str">
+        <x:f>IF(Z5="","",IF(Z5&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z5&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z5&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z5&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AC5" s="164" t="n">
+        <x:f>IF(OR(V5="",X5="",X5=0),"",ROUND(V5/X5,1))</x:f>
+        <x:v>146.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -48698,6 +48933,22 @@
       <x:c r="Y6" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z6" s="165" t="n">
+        <x:f>IF(A6="","",ROUND(V6/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>49.4</x:v>
+      </x:c>
+      <x:c r="AA6" s="167" t="n">
+        <x:f>IF(V6="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V6)+1)</x:f>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="AB6" s="163" t="str">
+        <x:f>IF(Z6="","",IF(Z6&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z6&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z6&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z6&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AC6" s="165" t="n">
+        <x:f>IF(OR(V6="",X6="",X6=0),"",ROUND(V6/X6,1))</x:f>
+        <x:v>89.9</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -48771,6 +49022,22 @@
       <x:c r="Y7" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z7" s="164" t="n">
+        <x:f>IF(A7="","",ROUND(V7/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>49.4</x:v>
+      </x:c>
+      <x:c r="AA7" s="166" t="n">
+        <x:f>IF(V7="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V7)+1)</x:f>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="AB7" s="162" t="str">
+        <x:f>IF(Z7="","",IF(Z7&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z7&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z7&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z7&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AC7" s="164" t="n">
+        <x:f>IF(OR(V7="",X7="",X7=0),"",ROUND(V7/X7,1))</x:f>
+        <x:v>89.9</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -48844,6 +49111,22 @@
       <x:c r="Y8" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z8" s="165" t="n">
+        <x:f>IF(A8="","",ROUND(V8/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>77.2</x:v>
+      </x:c>
+      <x:c r="AA8" s="167" t="n">
+        <x:f>IF(V8="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V8)+1)</x:f>
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="AB8" s="163" t="str">
+        <x:f>IF(Z8="","",IF(Z8&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z8&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z8&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z8&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC8" s="165" t="n">
+        <x:f>IF(OR(V8="",X8="",X8=0),"",ROUND(V8/X8,1))</x:f>
+        <x:v>114</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -48917,6 +49200,22 @@
       <x:c r="Y9" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z9" s="164" t="n">
+        <x:f>IF(A9="","",ROUND(V9/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>84.3</x:v>
+      </x:c>
+      <x:c r="AA9" s="166" t="n">
+        <x:f>IF(V9="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V9)+1)</x:f>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="AB9" s="162" t="str">
+        <x:f>IF(Z9="","",IF(Z9&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z9&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z9&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z9&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC9" s="164" t="n">
+        <x:f>IF(OR(V9="",X9="",X9=0),"",ROUND(V9/X9,1))</x:f>
+        <x:v>102.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -48990,6 +49289,22 @@
       <x:c r="Y10" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z10" s="165" t="n">
+        <x:f>IF(A10="","",ROUND(V10/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>87.8</x:v>
+      </x:c>
+      <x:c r="AA10" s="167" t="n">
+        <x:f>IF(V10="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V10)+1)</x:f>
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="AB10" s="163" t="str">
+        <x:f>IF(Z10="","",IF(Z10&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z10&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z10&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z10&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC10" s="165" t="n">
+        <x:f>IF(OR(V10="",X10="",X10=0),"",ROUND(V10/X10,1))</x:f>
+        <x:v>97.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -49063,6 +49378,22 @@
       <x:c r="Y11" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z11" s="164" t="n">
+        <x:f>IF(A11="","",ROUND(V11/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>97.1</x:v>
+      </x:c>
+      <x:c r="AA11" s="166" t="n">
+        <x:f>IF(V11="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V11)+1)</x:f>
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="AB11" s="162" t="str">
+        <x:f>IF(Z11="","",IF(Z11&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z11&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z11&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z11&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC11" s="164" t="n">
+        <x:f>IF(OR(V11="",X11="",X11=0),"",ROUND(V11/X11,1))</x:f>
+        <x:v>108.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -49136,6 +49467,22 @@
       <x:c r="Y12" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z12" s="165" t="n">
+        <x:f>IF(A12="","",ROUND(V12/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>101.2</x:v>
+      </x:c>
+      <x:c r="AA12" s="167" t="n">
+        <x:f>IF(V12="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V12)+1)</x:f>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="AB12" s="163" t="str">
+        <x:f>IF(Z12="","",IF(Z12&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z12&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z12&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z12&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC12" s="165" t="n">
+        <x:f>IF(OR(V12="",X12="",X12=0),"",ROUND(V12/X12,1))</x:f>
+        <x:v>85.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" s="12" t="str">
@@ -49209,6 +49556,22 @@
       <x:c r="Y13" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z13" s="164" t="n">
+        <x:f>IF(A13="","",ROUND(V13/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>106.2</x:v>
+      </x:c>
+      <x:c r="AA13" s="166" t="n">
+        <x:f>IF(V13="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V13)+1)</x:f>
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="AB13" s="162" t="str">
+        <x:f>IF(Z13="","",IF(Z13&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z13&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z13&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z13&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC13" s="164" t="n">
+        <x:f>IF(OR(V13="",X13="",X13=0),"",ROUND(V13/X13,1))</x:f>
+        <x:v>82.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -49282,6 +49645,22 @@
       <x:c r="Y14" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z14" s="165" t="n">
+        <x:f>IF(A14="","",ROUND(V14/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>113.2</x:v>
+      </x:c>
+      <x:c r="AA14" s="167" t="n">
+        <x:f>IF(V14="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V14)+1)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="AB14" s="163" t="str">
+        <x:f>IF(Z14="","",IF(Z14&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z14&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z14&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z14&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC14" s="165" t="n">
+        <x:f>IF(OR(V14="",X14="",X14=0),"",ROUND(V14/X14,1))</x:f>
+        <x:v>88.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -49355,6 +49734,22 @@
       <x:c r="Y15" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z15" s="164" t="n">
+        <x:f>IF(A15="","",ROUND(V15/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>128.6</x:v>
+      </x:c>
+      <x:c r="AA15" s="166" t="n">
+        <x:f>IF(V15="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V15)+1)</x:f>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="AB15" s="162" t="str">
+        <x:f>IF(Z15="","",IF(Z15&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z15&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z15&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z15&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC15" s="164" t="n">
+        <x:f>IF(OR(V15="",X15="",X15=0),"",ROUND(V15/X15,1))</x:f>
+        <x:v>83.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
       <x:c r="A16" s="12" t="str">
@@ -49428,6 +49823,22 @@
       <x:c r="Y16" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z16" s="165" t="n">
+        <x:f>IF(A16="","",ROUND(V16/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>136.7</x:v>
+      </x:c>
+      <x:c r="AA16" s="167" t="n">
+        <x:f>IF(V16="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V16)+1)</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="AB16" s="163" t="str">
+        <x:f>IF(Z16="","",IF(Z16&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z16&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z16&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z16&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC16" s="165" t="n">
+        <x:f>IF(OR(V16="",X16="",X16=0),"",ROUND(V16/X16,1))</x:f>
+        <x:v>88.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
       <x:c r="A17" s="12" t="str">
@@ -49501,6 +49912,22 @@
       <x:c r="Y17" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z17" s="164" t="n">
+        <x:f>IF(A17="","",ROUND(V17/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="AA17" s="166" t="n">
+        <x:f>IF(V17="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V17)+1)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="AB17" s="162" t="str">
+        <x:f>IF(Z17="","",IF(Z17&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z17&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z17&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z17&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC17" s="164" t="n">
+        <x:f>IF(OR(V17="",X17="",X17=0),"",ROUND(V17/X17,1))</x:f>
+        <x:v>83.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
       <x:c r="A18" s="12" t="str">
@@ -49574,6 +50001,22 @@
       <x:c r="Y18" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z18" s="165" t="n">
+        <x:f>IF(A18="","",ROUND(V18/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>84.5</x:v>
+      </x:c>
+      <x:c r="AA18" s="167" t="n">
+        <x:f>IF(V18="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V18)+1)</x:f>
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="AB18" s="163" t="str">
+        <x:f>IF(Z18="","",IF(Z18&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z18&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z18&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z18&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC18" s="165" t="n">
+        <x:f>IF(OR(V18="",X18="",X18=0),"",ROUND(V18/X18,1))</x:f>
+        <x:v>99.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
       <x:c r="A19" s="12" t="str">
@@ -49647,6 +50090,22 @@
       <x:c r="Y19" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z19" s="164" t="n">
+        <x:f>IF(A19="","",ROUND(V19/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>88.9</x:v>
+      </x:c>
+      <x:c r="AA19" s="166" t="n">
+        <x:f>IF(V19="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V19)+1)</x:f>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="AB19" s="162" t="str">
+        <x:f>IF(Z19="","",IF(Z19&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z19&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z19&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z19&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC19" s="164" t="n">
+        <x:f>IF(OR(V19="",X19="",X19=0),"",ROUND(V19/X19,1))</x:f>
+        <x:v>91.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="38" customHeight="1">
       <x:c r="A20" s="12" t="str">
@@ -49720,6 +50179,22 @@
       <x:c r="Y20" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z20" s="165" t="n">
+        <x:f>IF(A20="","",ROUND(V20/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>116.4</x:v>
+      </x:c>
+      <x:c r="AA20" s="167" t="n">
+        <x:f>IF(V20="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V20)+1)</x:f>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="AB20" s="163" t="str">
+        <x:f>IF(Z20="","",IF(Z20&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z20&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z20&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z20&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC20" s="165" t="n">
+        <x:f>IF(OR(V20="",X20="",X20=0),"",ROUND(V20/X20,1))</x:f>
+        <x:v>92.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
       <x:c r="A21" s="12" t="str">
@@ -49793,6 +50268,22 @@
       <x:c r="Y21" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z21" s="164" t="n">
+        <x:f>IF(A21="","",ROUND(V21/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>125.2</x:v>
+      </x:c>
+      <x:c r="AA21" s="166" t="n">
+        <x:f>IF(V21="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V21)+1)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="AB21" s="162" t="str">
+        <x:f>IF(Z21="","",IF(Z21&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z21&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z21&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z21&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC21" s="164" t="n">
+        <x:f>IF(OR(V21="",X21="",X21=0),"",ROUND(V21/X21,1))</x:f>
+        <x:v>92.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="12" t="str">
@@ -49866,6 +50357,22 @@
       <x:c r="Y22" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z22" s="165" t="n">
+        <x:f>IF(A22="","",ROUND(V22/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>140.8</x:v>
+      </x:c>
+      <x:c r="AA22" s="167" t="n">
+        <x:f>IF(V22="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V22)+1)</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="AB22" s="163" t="str">
+        <x:f>IF(Z22="","",IF(Z22&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z22&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z22&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z22&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC22" s="165" t="n">
+        <x:f>IF(OR(V22="",X22="",X22=0),"",ROUND(V22/X22,1))</x:f>
+        <x:v>105.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="38" customHeight="1">
       <x:c r="A23" s="12" t="str">
@@ -49939,6 +50446,22 @@
       <x:c r="Y23" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z23" s="164" t="n">
+        <x:f>IF(A23="","",ROUND(V23/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>149.1</x:v>
+      </x:c>
+      <x:c r="AA23" s="166" t="n">
+        <x:f>IF(V23="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V23)+1)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="AB23" s="162" t="str">
+        <x:f>IF(Z23="","",IF(Z23&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z23&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z23&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z23&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC23" s="164" t="n">
+        <x:f>IF(OR(V23="",X23="",X23=0),"",ROUND(V23/X23,1))</x:f>
+        <x:v>92.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
       <x:c r="A24" s="12" t="str">
@@ -50012,6 +50535,22 @@
       <x:c r="Y24" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z24" s="165" t="n">
+        <x:f>IF(A24="","",ROUND(V24/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>161.2</x:v>
+      </x:c>
+      <x:c r="AA24" s="167" t="n">
+        <x:f>IF(V24="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V24)+1)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="AB24" s="163" t="str">
+        <x:f>IF(Z24="","",IF(Z24&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z24&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z24&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z24&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC24" s="165" t="n">
+        <x:f>IF(OR(V24="",X24="",X24=0),"",ROUND(V24/X24,1))</x:f>
+        <x:v>88.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
       <x:c r="A25" s="12" t="str">
@@ -50083,6 +50622,22 @@
       <x:c r="Y25" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z25" s="164" t="n">
+        <x:f>IF(A25="","",ROUND(V25/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>90.5</x:v>
+      </x:c>
+      <x:c r="AA25" s="166" t="n">
+        <x:f>IF(V25="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V25)+1)</x:f>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="AB25" s="162" t="str">
+        <x:f>IF(Z25="","",IF(Z25&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z25&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z25&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z25&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC25" s="164" t="n">
+        <x:f>IF(OR(V25="",X25="",X25=0),"",ROUND(V25/X25,1))</x:f>
+        <x:v>133.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="38" customHeight="1">
       <x:c r="A26" s="12" t="str">
@@ -50156,6 +50711,22 @@
       <x:c r="Y26" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z26" s="165" t="n">
+        <x:f>IF(A26="","",ROUND(V26/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>101.4</x:v>
+      </x:c>
+      <x:c r="AA26" s="167" t="n">
+        <x:f>IF(V26="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V26)+1)</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="AB26" s="163" t="str">
+        <x:f>IF(Z26="","",IF(Z26&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z26&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z26&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z26&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC26" s="165" t="n">
+        <x:f>IF(OR(V26="",X26="",X26=0),"",ROUND(V26/X26,1))</x:f>
+        <x:v>131.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="38" customHeight="1">
       <x:c r="A27" s="12" t="str">
@@ -50229,6 +50800,22 @@
       <x:c r="Y27" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z27" s="164" t="n">
+        <x:f>IF(A27="","",ROUND(V27/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="AA27" s="166" t="n">
+        <x:f>IF(V27="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V27)+1)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="AB27" s="162" t="str">
+        <x:f>IF(Z27="","",IF(Z27&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z27&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z27&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z27&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC27" s="164" t="n">
+        <x:f>IF(OR(V27="",X27="",X27=0),"",ROUND(V27/X27,1))</x:f>
+        <x:v>125.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
       <x:c r="A28" s="12" t="str">
@@ -50302,6 +50889,22 @@
       <x:c r="Y28" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z28" s="165" t="n">
+        <x:f>IF(A28="","",ROUND(V28/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>130.2</x:v>
+      </x:c>
+      <x:c r="AA28" s="167" t="n">
+        <x:f>IF(V28="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V28)+1)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="AB28" s="163" t="str">
+        <x:f>IF(Z28="","",IF(Z28&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z28&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z28&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z28&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC28" s="165" t="n">
+        <x:f>IF(OR(V28="",X28="",X28=0),"",ROUND(V28/X28,1))</x:f>
+        <x:v>115.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="38" customHeight="1">
       <x:c r="A29" s="12" t="str">
@@ -50375,6 +50978,22 @@
       <x:c r="Y29" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z29" s="164" t="n">
+        <x:f>IF(A29="","",ROUND(V29/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>124.4</x:v>
+      </x:c>
+      <x:c r="AA29" s="166" t="n">
+        <x:f>IF(V29="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V29)+1)</x:f>
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="AB29" s="162" t="str">
+        <x:f>IF(Z29="","",IF(Z29&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z29&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z29&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z29&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC29" s="164" t="n">
+        <x:f>IF(OR(V29="",X29="",X29=0),"",ROUND(V29/X29,1))</x:f>
+        <x:v>110.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="38" customHeight="1">
       <x:c r="A30" s="12" t="str">
@@ -50448,6 +51067,22 @@
       <x:c r="Y30" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z30" s="165" t="n">
+        <x:f>IF(A30="","",ROUND(V30/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>138.1</x:v>
+      </x:c>
+      <x:c r="AA30" s="167" t="n">
+        <x:f>IF(V30="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V30)+1)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="AB30" s="163" t="str">
+        <x:f>IF(Z30="","",IF(Z30&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z30&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z30&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z30&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC30" s="165" t="n">
+        <x:f>IF(OR(V30="",X30="",X30=0),"",ROUND(V30/X30,1))</x:f>
+        <x:v>88.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="38" customHeight="1">
       <x:c r="A31" s="12" t="str">
@@ -50522,6 +51157,22 @@
       <x:c r="Y31" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z31" s="164" t="n">
+        <x:f>IF(A31="","",ROUND(V31/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>72.3</x:v>
+      </x:c>
+      <x:c r="AA31" s="166" t="n">
+        <x:f>IF(V31="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V31)+1)</x:f>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="AB31" s="162" t="str">
+        <x:f>IF(Z31="","",IF(Z31&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z31&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z31&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z31&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AC31" s="164" t="n">
+        <x:f>IF(OR(V31="",X31="",X31=0),"",ROUND(V31/X31,1))</x:f>
+        <x:v>88.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
       <x:c r="A32" s="12" t="str">
@@ -50595,6 +51246,22 @@
       <x:c r="Y32" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z32" s="165" t="n">
+        <x:f>IF(A32="","",ROUND(V32/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>81.7</x:v>
+      </x:c>
+      <x:c r="AA32" s="167" t="n">
+        <x:f>IF(V32="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V32)+1)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="AB32" s="163" t="str">
+        <x:f>IF(Z32="","",IF(Z32&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z32&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z32&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z32&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC32" s="165" t="n">
+        <x:f>IF(OR(V32="",X32="",X32=0),"",ROUND(V32/X32,1))</x:f>
+        <x:v>86.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="38" customHeight="1">
       <x:c r="A33" s="12" t="str">
@@ -50668,6 +51335,22 @@
       <x:c r="Y33" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z33" s="164" t="n">
+        <x:f>IF(A33="","",ROUND(V33/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>84.5</x:v>
+      </x:c>
+      <x:c r="AA33" s="166" t="n">
+        <x:f>IF(V33="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V33)+1)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="AB33" s="162" t="str">
+        <x:f>IF(Z33="","",IF(Z33&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z33&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z33&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z33&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC33" s="164" t="n">
+        <x:f>IF(OR(V33="",X33="",X33=0),"",ROUND(V33/X33,1))</x:f>
+        <x:v>94.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="38" customHeight="1">
       <x:c r="A34" s="12" t="str">
@@ -50741,6 +51424,22 @@
       <x:c r="Y34" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z34" s="165" t="n">
+        <x:f>IF(A34="","",ROUND(V34/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>82.4</x:v>
+      </x:c>
+      <x:c r="AA34" s="167" t="n">
+        <x:f>IF(V34="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V34)+1)</x:f>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="AB34" s="163" t="str">
+        <x:f>IF(Z34="","",IF(Z34&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z34&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z34&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z34&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC34" s="165" t="n">
+        <x:f>IF(OR(V34="",X34="",X34=0),"",ROUND(V34/X34,1))</x:f>
+        <x:v>91.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="38" customHeight="1">
       <x:c r="A35" s="12" t="str">
@@ -50814,6 +51513,22 @@
       <x:c r="Y35" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z35" s="164" t="n">
+        <x:f>IF(A35="","",ROUND(V35/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="AA35" s="166" t="n">
+        <x:f>IF(V35="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V35)+1)</x:f>
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="AB35" s="162" t="str">
+        <x:f>IF(Z35="","",IF(Z35&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z35&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z35&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z35&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC35" s="164" t="n">
+        <x:f>IF(OR(V35="",X35="",X35=0),"",ROUND(V35/X35,1))</x:f>
+        <x:v>84.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="38" customHeight="1">
       <x:c r="A36" s="12" t="str">
@@ -50887,6 +51602,22 @@
       <x:c r="Y36" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z36" s="165" t="n">
+        <x:f>IF(A36="","",ROUND(V36/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>95.2</x:v>
+      </x:c>
+      <x:c r="AA36" s="167" t="n">
+        <x:f>IF(V36="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V36)+1)</x:f>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AB36" s="163" t="str">
+        <x:f>IF(Z36="","",IF(Z36&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z36&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z36&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z36&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC36" s="165" t="n">
+        <x:f>IF(OR(V36="",X36="",X36=0),"",ROUND(V36/X36,1))</x:f>
+        <x:v>74.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="38" customHeight="1">
       <x:c r="A37" s="12" t="str">
@@ -50960,6 +51691,22 @@
       <x:c r="Y37" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z37" s="164" t="n">
+        <x:f>IF(A37="","",ROUND(V37/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>99.6</x:v>
+      </x:c>
+      <x:c r="AA37" s="166" t="n">
+        <x:f>IF(V37="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V37)+1)</x:f>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="AB37" s="162" t="str">
+        <x:f>IF(Z37="","",IF(Z37&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z37&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z37&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z37&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC37" s="164" t="n">
+        <x:f>IF(OR(V37="",X37="",X37=0),"",ROUND(V37/X37,1))</x:f>
+        <x:v>77.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="38" customHeight="1">
       <x:c r="A38" s="12" t="str">
@@ -51033,6 +51780,22 @@
       <x:c r="Y38" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z38" s="165" t="n">
+        <x:f>IF(A38="","",ROUND(V38/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="AA38" s="167" t="n">
+        <x:f>IF(V38="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V38)+1)</x:f>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="AB38" s="163" t="str">
+        <x:f>IF(Z38="","",IF(Z38&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z38&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z38&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z38&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC38" s="165" t="n">
+        <x:f>IF(OR(V38="",X38="",X38=0),"",ROUND(V38/X38,1))</x:f>
+        <x:v>85.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="38" customHeight="1">
       <x:c r="A39" s="12" t="str">
@@ -51104,6 +51867,22 @@
       <x:c r="Y39" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z39" s="164" t="n">
+        <x:f>IF(A39="","",ROUND(V39/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>55.1</x:v>
+      </x:c>
+      <x:c r="AA39" s="166" t="n">
+        <x:f>IF(V39="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V39)+1)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="AB39" s="162" t="str">
+        <x:f>IF(Z39="","",IF(Z39&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z39&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z39&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z39&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AC39" s="164" t="n">
+        <x:f>IF(OR(V39="",X39="",X39=0),"",ROUND(V39/X39,1))</x:f>
+        <x:v>153.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="38" customHeight="1">
       <x:c r="A40" s="12" t="str">
@@ -51177,6 +51956,22 @@
       <x:c r="Y40" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z40" s="165" t="n">
+        <x:f>IF(A40="","",ROUND(V40/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="AA40" s="167" t="n">
+        <x:f>IF(V40="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V40)+1)</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="AB40" s="163" t="str">
+        <x:f>IF(Z40="","",IF(Z40&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z40&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z40&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z40&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>エントリー</x:v>
+      </x:c>
+      <x:c r="AC40" s="165" t="n">
+        <x:f>IF(OR(V40="",X40="",X40=0),"",ROUND(V40/X40,1))</x:f>
+        <x:v>96</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="38" customHeight="1">
       <x:c r="A41" s="12" t="str">
@@ -51248,6 +52043,22 @@
       <x:c r="Y41" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z41" s="164" t="n">
+        <x:f>IF(A41="","",ROUND(V41/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="AA41" s="166" t="n">
+        <x:f>IF(V41="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V41)+1)</x:f>
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="AB41" s="162" t="str">
+        <x:f>IF(Z41="","",IF(Z41&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z41&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z41&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z41&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC41" s="164" t="n">
+        <x:f>IF(OR(V41="",X41="",X41=0),"",ROUND(V41/X41,1))</x:f>
+        <x:v>89.4</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="38" customHeight="1">
       <x:c r="A42" s="12" t="str">
@@ -51321,6 +52132,22 @@
       <x:c r="Y42" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z42" s="165" t="n">
+        <x:f>IF(A42="","",ROUND(V42/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>85.7</x:v>
+      </x:c>
+      <x:c r="AA42" s="167" t="n">
+        <x:f>IF(V42="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V42)+1)</x:f>
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AB42" s="163" t="str">
+        <x:f>IF(Z42="","",IF(Z42&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z42&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z42&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z42&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC42" s="165" t="n">
+        <x:f>IF(OR(V42="",X42="",X42=0),"",ROUND(V42/X42,1))</x:f>
+        <x:v>98.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="38" customHeight="1">
       <x:c r="A43" s="12" t="str">
@@ -51394,6 +52221,22 @@
       <x:c r="Y43" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z43" s="164" t="n">
+        <x:f>IF(A43="","",ROUND(V43/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>103.8</x:v>
+      </x:c>
+      <x:c r="AA43" s="166" t="n">
+        <x:f>IF(V43="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V43)+1)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="AB43" s="162" t="str">
+        <x:f>IF(Z43="","",IF(Z43&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z43&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z43&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z43&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC43" s="164" t="n">
+        <x:f>IF(OR(V43="",X43="",X43=0),"",ROUND(V43/X43,1))</x:f>
+        <x:v>101.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="38" customHeight="1">
       <x:c r="A44" s="12" t="str">
@@ -51467,6 +52310,22 @@
       <x:c r="Y44" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z44" s="165" t="n">
+        <x:f>IF(A44="","",ROUND(V44/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>113.3</x:v>
+      </x:c>
+      <x:c r="AA44" s="167" t="n">
+        <x:f>IF(V44="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V44)+1)</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="AB44" s="163" t="str">
+        <x:f>IF(Z44="","",IF(Z44&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z44&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z44&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z44&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC44" s="165" t="n">
+        <x:f>IF(OR(V44="",X44="",X44=0),"",ROUND(V44/X44,1))</x:f>
+        <x:v>100.4</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="38" customHeight="1">
       <x:c r="A45" s="12" t="str">
@@ -51540,6 +52399,22 @@
       <x:c r="Y45" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z45" s="164" t="n">
+        <x:f>IF(A45="","",ROUND(V45/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="AA45" s="166" t="n">
+        <x:f>IF(V45="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V45)+1)</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="AB45" s="162" t="str">
+        <x:f>IF(Z45="","",IF(Z45&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z45&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z45&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z45&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC45" s="164" t="n">
+        <x:f>IF(OR(V45="",X45="",X45=0),"",ROUND(V45/X45,1))</x:f>
+        <x:v>80</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="38" customHeight="1">
       <x:c r="A46" s="12" t="str">
@@ -51613,6 +52488,22 @@
       <x:c r="Y46" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z46" s="165" t="n">
+        <x:f>IF(A46="","",ROUND(V46/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>128.2</x:v>
+      </x:c>
+      <x:c r="AA46" s="167" t="n">
+        <x:f>IF(V46="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V46)+1)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="AB46" s="163" t="str">
+        <x:f>IF(Z46="","",IF(Z46&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z46&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z46&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z46&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC46" s="165" t="n">
+        <x:f>IF(OR(V46="",X46="",X46=0),"",ROUND(V46/X46,1))</x:f>
+        <x:v>78.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="38" customHeight="1">
       <x:c r="A47" s="12" t="str">
@@ -51686,6 +52577,22 @@
       <x:c r="Y47" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z47" s="164" t="n">
+        <x:f>IF(A47="","",ROUND(V47/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>136.2</x:v>
+      </x:c>
+      <x:c r="AA47" s="166" t="n">
+        <x:f>IF(V47="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V47)+1)</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="AB47" s="162" t="str">
+        <x:f>IF(Z47="","",IF(Z47&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z47&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z47&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z47&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC47" s="164" t="n">
+        <x:f>IF(OR(V47="",X47="",X47=0),"",ROUND(V47/X47,1))</x:f>
+        <x:v>75.9</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="38" customHeight="1">
       <x:c r="A48" s="12" t="str">
@@ -51759,6 +52666,22 @@
       <x:c r="Y48" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z48" s="165" t="n">
+        <x:f>IF(A48="","",ROUND(V48/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>137.2</x:v>
+      </x:c>
+      <x:c r="AA48" s="167" t="n">
+        <x:f>IF(V48="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V48)+1)</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AB48" s="163" t="str">
+        <x:f>IF(Z48="","",IF(Z48&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z48&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z48&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z48&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC48" s="165" t="n">
+        <x:f>IF(OR(V48="",X48="",X48=0),"",ROUND(V48/X48,1))</x:f>
+        <x:v>76.4</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="38" customHeight="1">
       <x:c r="A49" s="12" t="str">
@@ -51832,6 +52755,22 @@
       <x:c r="Y49" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z49" s="164" t="n">
+        <x:f>IF(A49="","",ROUND(V49/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="AA49" s="166" t="n">
+        <x:f>IF(V49="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V49)+1)</x:f>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="AB49" s="162" t="str">
+        <x:f>IF(Z49="","",IF(Z49&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z49&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z49&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z49&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC49" s="164" t="n">
+        <x:f>IF(OR(V49="",X49="",X49=0),"",ROUND(V49/X49,1))</x:f>
+        <x:v>75.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="38" customHeight="1">
       <x:c r="A50" s="12" t="str">
@@ -51905,6 +52844,22 @@
       <x:c r="Y50" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z50" s="165" t="n">
+        <x:f>IF(A50="","",ROUND(V50/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>150.2</x:v>
+      </x:c>
+      <x:c r="AA50" s="167" t="n">
+        <x:f>IF(V50="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V50)+1)</x:f>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="AB50" s="163" t="str">
+        <x:f>IF(Z50="","",IF(Z50&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z50&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z50&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z50&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC50" s="165" t="n">
+        <x:f>IF(OR(V50="",X50="",X50=0),"",ROUND(V50/X50,1))</x:f>
+        <x:v>65</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="38" customHeight="1">
       <x:c r="A51" s="12" t="str">
@@ -51978,6 +52933,22 @@
       <x:c r="Y51" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z51" s="164" t="n">
+        <x:f>IF(A51="","",ROUND(V51/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AA51" s="166" t="n">
+        <x:f>IF(V51="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V51)+1)</x:f>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="AB51" s="162" t="str">
+        <x:f>IF(Z51="","",IF(Z51&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z51&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z51&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z51&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC51" s="164" t="n">
+        <x:f>IF(OR(V51="",X51="",X51=0),"",ROUND(V51/X51,1))</x:f>
+        <x:v>169.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="38" customHeight="1">
       <x:c r="A52" s="12" t="str">
@@ -52052,6 +53023,22 @@
       <x:c r="Y52" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z52" s="165" t="n">
+        <x:f>IF(A52="","",ROUND(V52/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>115.9</x:v>
+      </x:c>
+      <x:c r="AA52" s="167" t="n">
+        <x:f>IF(V52="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V52)+1)</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="AB52" s="163" t="str">
+        <x:f>IF(Z52="","",IF(Z52&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z52&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z52&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z52&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC52" s="165" t="n">
+        <x:f>IF(OR(V52="",X52="",X52=0),"",ROUND(V52/X52,1))</x:f>
+        <x:v>141.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="38" customHeight="1">
       <x:c r="A53" s="12" t="str">
@@ -52125,6 +53112,22 @@
       <x:c r="Y53" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z53" s="164" t="n">
+        <x:f>IF(A53="","",ROUND(V53/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>115.9</x:v>
+      </x:c>
+      <x:c r="AA53" s="166" t="n">
+        <x:f>IF(V53="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V53)+1)</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="AB53" s="162" t="str">
+        <x:f>IF(Z53="","",IF(Z53&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z53&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z53&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z53&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC53" s="164" t="n">
+        <x:f>IF(OR(V53="",X53="",X53=0),"",ROUND(V53/X53,1))</x:f>
+        <x:v>136.9</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="38" customHeight="1">
       <x:c r="A54" s="12" t="str">
@@ -52198,6 +53201,22 @@
       <x:c r="Y54" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z54" s="165" t="n">
+        <x:f>IF(A54="","",ROUND(V54/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>137.9</x:v>
+      </x:c>
+      <x:c r="AA54" s="167" t="n">
+        <x:f>IF(V54="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V54)+1)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="AB54" s="163" t="str">
+        <x:f>IF(Z54="","",IF(Z54&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z54&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z54&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z54&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC54" s="165" t="n">
+        <x:f>IF(OR(V54="",X54="",X54=0),"",ROUND(V54/X54,1))</x:f>
+        <x:v>134.4</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="38" customHeight="1">
       <x:c r="A55" s="12" t="str">
@@ -52271,6 +53290,22 @@
       <x:c r="Y55" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z55" s="164" t="n">
+        <x:f>IF(A55="","",ROUND(V55/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>153.6</x:v>
+      </x:c>
+      <x:c r="AA55" s="166" t="n">
+        <x:f>IF(V55="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V55)+1)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="AB55" s="162" t="str">
+        <x:f>IF(Z55="","",IF(Z55&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z55&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z55&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z55&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC55" s="164" t="n">
+        <x:f>IF(OR(V55="",X55="",X55=0),"",ROUND(V55/X55,1))</x:f>
+        <x:v>136.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="38" customHeight="1">
       <x:c r="A56" s="12" t="str">
@@ -52344,6 +53379,22 @@
       <x:c r="Y56" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z56" s="165" t="n">
+        <x:f>IF(A56="","",ROUND(V56/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>161.8</x:v>
+      </x:c>
+      <x:c r="AA56" s="167" t="n">
+        <x:f>IF(V56="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V56)+1)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="AB56" s="163" t="str">
+        <x:f>IF(Z56="","",IF(Z56&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z56&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z56&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z56&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC56" s="165" t="n">
+        <x:f>IF(OR(V56="",X56="",X56=0),"",ROUND(V56/X56,1))</x:f>
+        <x:v>110.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="38" customHeight="1">
       <x:c r="A57" s="12" t="str">
@@ -52417,6 +53468,22 @@
       <x:c r="Y57" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z57" s="164" t="n">
+        <x:f>IF(A57="","",ROUND(V57/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>163.4</x:v>
+      </x:c>
+      <x:c r="AA57" s="166" t="n">
+        <x:f>IF(V57="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V57)+1)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="AB57" s="162" t="str">
+        <x:f>IF(Z57="","",IF(Z57&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z57&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z57&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z57&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC57" s="164" t="n">
+        <x:f>IF(OR(V57="",X57="",X57=0),"",ROUND(V57/X57,1))</x:f>
+        <x:v>111.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="38" customHeight="1">
       <x:c r="A58" s="12" t="str">
@@ -52490,6 +53557,22 @@
       <x:c r="Y58" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z58" s="165" t="n">
+        <x:f>IF(A58="","",ROUND(V58/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>176.7</x:v>
+      </x:c>
+      <x:c r="AA58" s="167" t="n">
+        <x:f>IF(V58="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V58)+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AB58" s="163" t="str">
+        <x:f>IF(Z58="","",IF(Z58&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z58&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z58&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z58&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>フラッグシップ</x:v>
+      </x:c>
+      <x:c r="AC58" s="165" t="n">
+        <x:f>IF(OR(V58="",X58="",X58=0),"",ROUND(V58/X58,1))</x:f>
+        <x:v>107.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="38" customHeight="1">
       <x:c r="A59" s="12" t="str">
@@ -52563,6 +53646,22 @@
       <x:c r="Y59" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z59" s="164" t="n">
+        <x:f>IF(A59="","",ROUND(V59/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>175.6</x:v>
+      </x:c>
+      <x:c r="AA59" s="166" t="n">
+        <x:f>IF(V59="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V59)+1)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="AB59" s="162" t="str">
+        <x:f>IF(Z59="","",IF(Z59&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z59&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z59&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z59&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>フラッグシップ</x:v>
+      </x:c>
+      <x:c r="AC59" s="164" t="n">
+        <x:f>IF(OR(V59="",X59="",X59=0),"",ROUND(V59/X59,1))</x:f>
+        <x:v>107</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="38" customHeight="1">
       <x:c r="A60" s="12" t="str">
@@ -52636,6 +53735,22 @@
       <x:c r="Y60" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z60" s="165" t="n">
+        <x:f>IF(A60="","",ROUND(V60/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>195.2</x:v>
+      </x:c>
+      <x:c r="AA60" s="167" t="n">
+        <x:f>IF(V60="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V60)+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="AB60" s="163" t="str">
+        <x:f>IF(Z60="","",IF(Z60&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z60&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z60&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z60&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>フラッグシップ</x:v>
+      </x:c>
+      <x:c r="AC60" s="165" t="n">
+        <x:f>IF(OR(V60="",X60="",X60=0),"",ROUND(V60/X60,1))</x:f>
+        <x:v>84.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="38" customHeight="1">
       <x:c r="A61" s="12" t="str">
@@ -52707,6 +53822,22 @@
       <x:c r="Y61" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z61" s="164" t="n">
+        <x:f>IF(A61="","",ROUND(V61/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="AA61" s="166" t="n">
+        <x:f>IF(V61="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V61)+1)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AB61" s="162" t="str">
+        <x:f>IF(Z61="","",IF(Z61&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z61&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z61&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z61&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC61" s="164" t="n">
+        <x:f>IF(OR(V61="",X61="",X61=0),"",ROUND(V61/X61,1))</x:f>
+        <x:v>130.4</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="38" customHeight="1">
       <x:c r="A62" s="12" t="str">
@@ -52780,6 +53911,22 @@
       <x:c r="Y62" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z62" s="165" t="n">
+        <x:f>IF(A62="","",ROUND(V62/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>106.1</x:v>
+      </x:c>
+      <x:c r="AA62" s="167" t="n">
+        <x:f>IF(V62="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V62)+1)</x:f>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="AB62" s="163" t="str">
+        <x:f>IF(Z62="","",IF(Z62&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z62&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z62&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z62&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>メインストリーム</x:v>
+      </x:c>
+      <x:c r="AC62" s="165" t="n">
+        <x:f>IF(OR(V62="",X62="",X62=0),"",ROUND(V62/X62,1))</x:f>
+        <x:v>121.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="38" customHeight="1">
       <x:c r="A63" s="12" t="str">
@@ -52853,6 +54000,22 @@
       <x:c r="Y63" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z63" s="164" t="n">
+        <x:f>IF(A63="","",ROUND(V63/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>113.2</x:v>
+      </x:c>
+      <x:c r="AA63" s="166" t="n">
+        <x:f>IF(V63="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V63)+1)</x:f>
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="AB63" s="162" t="str">
+        <x:f>IF(Z63="","",IF(Z63&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z63&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z63&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z63&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC63" s="164" t="n">
+        <x:f>IF(OR(V63="",X63="",X63=0),"",ROUND(V63/X63,1))</x:f>
+        <x:v>122.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="38" customHeight="1">
       <x:c r="A64" s="12" t="str">
@@ -52926,6 +54089,22 @@
       <x:c r="Y64" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z64" s="165" t="n">
+        <x:f>IF(A64="","",ROUND(V64/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>116.1</x:v>
+      </x:c>
+      <x:c r="AA64" s="167" t="n">
+        <x:f>IF(V64="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V64)+1)</x:f>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="AB64" s="163" t="str">
+        <x:f>IF(Z64="","",IF(Z64&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z64&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z64&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z64&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ミドルレンジ</x:v>
+      </x:c>
+      <x:c r="AC64" s="165" t="n">
+        <x:f>IF(OR(V64="",X64="",X64=0),"",ROUND(V64/X64,1))</x:f>
+        <x:v>125.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="38" customHeight="1">
       <x:c r="A65" s="12" t="str">
@@ -52999,6 +54178,22 @@
       <x:c r="Y65" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z65" s="164" t="n">
+        <x:f>IF(A65="","",ROUND(V65/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>147.1</x:v>
+      </x:c>
+      <x:c r="AA65" s="166" t="n">
+        <x:f>IF(V65="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V65)+1)</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="AB65" s="162" t="str">
+        <x:f>IF(Z65="","",IF(Z65&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z65&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z65&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z65&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC65" s="164" t="n">
+        <x:f>IF(OR(V65="",X65="",X65=0),"",ROUND(V65/X65,1))</x:f>
+        <x:v>114.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="38" customHeight="1">
       <x:c r="A66" s="12" t="str">
@@ -53072,6 +54267,22 @@
       <x:c r="Y66" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z66" s="165" t="n">
+        <x:f>IF(A66="","",ROUND(V66/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="AA66" s="167" t="n">
+        <x:f>IF(V66="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V66)+1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="AB66" s="163" t="str">
+        <x:f>IF(Z66="","",IF(Z66&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z66&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z66&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z66&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>ハイエンド</x:v>
+      </x:c>
+      <x:c r="AC66" s="165" t="n">
+        <x:f>IF(OR(V66="",X66="",X66=0),"",ROUND(V66/X66,1))</x:f>
+        <x:v>107.9</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="38" customHeight="1">
       <x:c r="A67" s="12" t="str">
@@ -53145,6 +54356,22 @@
       <x:c r="Y67" s="102" t="n">
         <x:v>46218</x:v>
       </x:c>
+      <x:c r="Z67" s="164" t="n">
+        <x:f>IF(A67="","",ROUND(V67/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>182.9</x:v>
+      </x:c>
+      <x:c r="AA67" s="166" t="n">
+        <x:f>IF(V67="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V67)+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="AB67" s="162" t="str">
+        <x:f>IF(Z67="","",IF(Z67&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z67&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z67&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z67&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>フラッグシップ</x:v>
+      </x:c>
+      <x:c r="AC67" s="164" t="n">
+        <x:f>IF(OR(V67="",X67="",X67=0),"",ROUND(V67/X67,1))</x:f>
+        <x:v>99</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="38" customHeight="1">
       <x:c r="A68" s="12" t="str">
@@ -53217,6 +54444,22 @@
       </x:c>
       <x:c r="Y68" s="102" t="n">
         <x:v>46218</x:v>
+      </x:c>
+      <x:c r="Z68" s="165" t="n">
+        <x:f>IF(A68="","",ROUND(V68/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+        <x:v>199.9</x:v>
+      </x:c>
+      <x:c r="AA68" s="167" t="n">
+        <x:f>IF(V68="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V68)+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB68" s="163" t="str">
+        <x:f>IF(Z68="","",IF(Z68&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z68&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z68&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z68&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+        <x:v>フラッグシップ</x:v>
+      </x:c>
+      <x:c r="AC68" s="165" t="n">
+        <x:f>IF(OR(V68="",X68="",X68=0),"",ROUND(V68/X68,1))</x:f>
+        <x:v>67.8</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -53245,6 +54488,18 @@
       <x:c r="W69" s="105"/>
       <x:c r="X69" s="105"/>
       <x:c r="Y69" s="102"/>
+      <x:c r="Z69" s="164" t="str">
+        <x:f>IF(A69="","",ROUND(V69/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA69" s="166" t="str">
+        <x:f>IF(V69="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V69)+1)</x:f>
+      </x:c>
+      <x:c r="AB69" s="162" t="str">
+        <x:f>IF(Z69="","",IF(Z69&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z69&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z69&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z69&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC69" s="164" t="str">
+        <x:f>IF(OR(V69="",X69="",X69=0),"",ROUND(V69/X69,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="12"/>
@@ -53272,6 +54527,18 @@
       <x:c r="W70" s="105"/>
       <x:c r="X70" s="105"/>
       <x:c r="Y70" s="102"/>
+      <x:c r="Z70" s="165" t="str">
+        <x:f>IF(A70="","",ROUND(V70/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA70" s="167" t="str">
+        <x:f>IF(V70="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V70)+1)</x:f>
+      </x:c>
+      <x:c r="AB70" s="163" t="str">
+        <x:f>IF(Z70="","",IF(Z70&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z70&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z70&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z70&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC70" s="165" t="str">
+        <x:f>IF(OR(V70="",X70="",X70=0),"",ROUND(V70/X70,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="12"/>
@@ -53299,6 +54566,18 @@
       <x:c r="W71" s="105"/>
       <x:c r="X71" s="105"/>
       <x:c r="Y71" s="102"/>
+      <x:c r="Z71" s="164" t="str">
+        <x:f>IF(A71="","",ROUND(V71/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA71" s="166" t="str">
+        <x:f>IF(V71="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V71)+1)</x:f>
+      </x:c>
+      <x:c r="AB71" s="162" t="str">
+        <x:f>IF(Z71="","",IF(Z71&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z71&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z71&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z71&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC71" s="164" t="str">
+        <x:f>IF(OR(V71="",X71="",X71=0),"",ROUND(V71/X71,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="12"/>
@@ -53326,6 +54605,18 @@
       <x:c r="W72" s="105"/>
       <x:c r="X72" s="105"/>
       <x:c r="Y72" s="102"/>
+      <x:c r="Z72" s="165" t="str">
+        <x:f>IF(A72="","",ROUND(V72/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA72" s="167" t="str">
+        <x:f>IF(V72="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V72)+1)</x:f>
+      </x:c>
+      <x:c r="AB72" s="163" t="str">
+        <x:f>IF(Z72="","",IF(Z72&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z72&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z72&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z72&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC72" s="165" t="str">
+        <x:f>IF(OR(V72="",X72="",X72=0),"",ROUND(V72/X72,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="12"/>
@@ -53353,6 +54644,18 @@
       <x:c r="W73" s="105"/>
       <x:c r="X73" s="105"/>
       <x:c r="Y73" s="102"/>
+      <x:c r="Z73" s="164" t="str">
+        <x:f>IF(A73="","",ROUND(V73/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA73" s="166" t="str">
+        <x:f>IF(V73="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V73)+1)</x:f>
+      </x:c>
+      <x:c r="AB73" s="162" t="str">
+        <x:f>IF(Z73="","",IF(Z73&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z73&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z73&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z73&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC73" s="164" t="str">
+        <x:f>IF(OR(V73="",X73="",X73=0),"",ROUND(V73/X73,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="12"/>
@@ -53380,6 +54683,18 @@
       <x:c r="W74" s="105"/>
       <x:c r="X74" s="105"/>
       <x:c r="Y74" s="102"/>
+      <x:c r="Z74" s="165" t="str">
+        <x:f>IF(A74="","",ROUND(V74/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA74" s="167" t="str">
+        <x:f>IF(V74="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V74)+1)</x:f>
+      </x:c>
+      <x:c r="AB74" s="163" t="str">
+        <x:f>IF(Z74="","",IF(Z74&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z74&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z74&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z74&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC74" s="165" t="str">
+        <x:f>IF(OR(V74="",X74="",X74=0),"",ROUND(V74/X74,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="12"/>
@@ -53407,6 +54722,18 @@
       <x:c r="W75" s="105"/>
       <x:c r="X75" s="105"/>
       <x:c r="Y75" s="102"/>
+      <x:c r="Z75" s="164" t="str">
+        <x:f>IF(A75="","",ROUND(V75/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA75" s="166" t="str">
+        <x:f>IF(V75="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V75)+1)</x:f>
+      </x:c>
+      <x:c r="AB75" s="162" t="str">
+        <x:f>IF(Z75="","",IF(Z75&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z75&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z75&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z75&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC75" s="164" t="str">
+        <x:f>IF(OR(V75="",X75="",X75=0),"",ROUND(V75/X75,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="12"/>
@@ -53434,6 +54761,18 @@
       <x:c r="W76" s="105"/>
       <x:c r="X76" s="105"/>
       <x:c r="Y76" s="102"/>
+      <x:c r="Z76" s="165" t="str">
+        <x:f>IF(A76="","",ROUND(V76/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA76" s="167" t="str">
+        <x:f>IF(V76="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V76)+1)</x:f>
+      </x:c>
+      <x:c r="AB76" s="163" t="str">
+        <x:f>IF(Z76="","",IF(Z76&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z76&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z76&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z76&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC76" s="165" t="str">
+        <x:f>IF(OR(V76="",X76="",X76=0),"",ROUND(V76/X76,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="12"/>
@@ -53461,6 +54800,18 @@
       <x:c r="W77" s="105"/>
       <x:c r="X77" s="105"/>
       <x:c r="Y77" s="102"/>
+      <x:c r="Z77" s="164" t="str">
+        <x:f>IF(A77="","",ROUND(V77/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA77" s="166" t="str">
+        <x:f>IF(V77="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V77)+1)</x:f>
+      </x:c>
+      <x:c r="AB77" s="162" t="str">
+        <x:f>IF(Z77="","",IF(Z77&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z77&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z77&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z77&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC77" s="164" t="str">
+        <x:f>IF(OR(V77="",X77="",X77=0),"",ROUND(V77/X77,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="12"/>
@@ -53488,6 +54839,18 @@
       <x:c r="W78" s="105"/>
       <x:c r="X78" s="105"/>
       <x:c r="Y78" s="102"/>
+      <x:c r="Z78" s="165" t="str">
+        <x:f>IF(A78="","",ROUND(V78/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA78" s="167" t="str">
+        <x:f>IF(V78="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V78)+1)</x:f>
+      </x:c>
+      <x:c r="AB78" s="163" t="str">
+        <x:f>IF(Z78="","",IF(Z78&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z78&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z78&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z78&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC78" s="165" t="str">
+        <x:f>IF(OR(V78="",X78="",X78=0),"",ROUND(V78/X78,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="12"/>
@@ -53515,6 +54878,18 @@
       <x:c r="W79" s="105"/>
       <x:c r="X79" s="105"/>
       <x:c r="Y79" s="102"/>
+      <x:c r="Z79" s="164" t="str">
+        <x:f>IF(A79="","",ROUND(V79/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA79" s="166" t="str">
+        <x:f>IF(V79="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V79)+1)</x:f>
+      </x:c>
+      <x:c r="AB79" s="162" t="str">
+        <x:f>IF(Z79="","",IF(Z79&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z79&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z79&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z79&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC79" s="164" t="str">
+        <x:f>IF(OR(V79="",X79="",X79=0),"",ROUND(V79/X79,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="12"/>
@@ -53542,6 +54917,18 @@
       <x:c r="W80" s="105"/>
       <x:c r="X80" s="105"/>
       <x:c r="Y80" s="102"/>
+      <x:c r="Z80" s="165" t="str">
+        <x:f>IF(A80="","",ROUND(V80/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA80" s="167" t="str">
+        <x:f>IF(V80="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V80)+1)</x:f>
+      </x:c>
+      <x:c r="AB80" s="163" t="str">
+        <x:f>IF(Z80="","",IF(Z80&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z80&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z80&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z80&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC80" s="165" t="str">
+        <x:f>IF(OR(V80="",X80="",X80=0),"",ROUND(V80/X80,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="12"/>
@@ -53569,6 +54956,18 @@
       <x:c r="W81" s="105"/>
       <x:c r="X81" s="105"/>
       <x:c r="Y81" s="102"/>
+      <x:c r="Z81" s="164" t="str">
+        <x:f>IF(A81="","",ROUND(V81/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA81" s="166" t="str">
+        <x:f>IF(V81="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V81)+1)</x:f>
+      </x:c>
+      <x:c r="AB81" s="162" t="str">
+        <x:f>IF(Z81="","",IF(Z81&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z81&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z81&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z81&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC81" s="164" t="str">
+        <x:f>IF(OR(V81="",X81="",X81=0),"",ROUND(V81/X81,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="12"/>
@@ -53596,6 +54995,18 @@
       <x:c r="W82" s="105"/>
       <x:c r="X82" s="105"/>
       <x:c r="Y82" s="102"/>
+      <x:c r="Z82" s="165" t="str">
+        <x:f>IF(A82="","",ROUND(V82/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA82" s="167" t="str">
+        <x:f>IF(V82="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V82)+1)</x:f>
+      </x:c>
+      <x:c r="AB82" s="163" t="str">
+        <x:f>IF(Z82="","",IF(Z82&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z82&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z82&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z82&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC82" s="165" t="str">
+        <x:f>IF(OR(V82="",X82="",X82=0),"",ROUND(V82/X82,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="12"/>
@@ -53623,6 +55034,18 @@
       <x:c r="W83" s="105"/>
       <x:c r="X83" s="105"/>
       <x:c r="Y83" s="102"/>
+      <x:c r="Z83" s="164" t="str">
+        <x:f>IF(A83="","",ROUND(V83/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA83" s="166" t="str">
+        <x:f>IF(V83="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V83)+1)</x:f>
+      </x:c>
+      <x:c r="AB83" s="162" t="str">
+        <x:f>IF(Z83="","",IF(Z83&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z83&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z83&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z83&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC83" s="164" t="str">
+        <x:f>IF(OR(V83="",X83="",X83=0),"",ROUND(V83/X83,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="12"/>
@@ -53650,6 +55073,18 @@
       <x:c r="W84" s="105"/>
       <x:c r="X84" s="105"/>
       <x:c r="Y84" s="102"/>
+      <x:c r="Z84" s="165" t="str">
+        <x:f>IF(A84="","",ROUND(V84/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA84" s="167" t="str">
+        <x:f>IF(V84="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V84)+1)</x:f>
+      </x:c>
+      <x:c r="AB84" s="163" t="str">
+        <x:f>IF(Z84="","",IF(Z84&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z84&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z84&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z84&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC84" s="165" t="str">
+        <x:f>IF(OR(V84="",X84="",X84=0),"",ROUND(V84/X84,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="12"/>
@@ -53677,6 +55112,18 @@
       <x:c r="W85" s="105"/>
       <x:c r="X85" s="105"/>
       <x:c r="Y85" s="102"/>
+      <x:c r="Z85" s="164" t="str">
+        <x:f>IF(A85="","",ROUND(V85/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA85" s="166" t="str">
+        <x:f>IF(V85="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V85)+1)</x:f>
+      </x:c>
+      <x:c r="AB85" s="162" t="str">
+        <x:f>IF(Z85="","",IF(Z85&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z85&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z85&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z85&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC85" s="164" t="str">
+        <x:f>IF(OR(V85="",X85="",X85=0),"",ROUND(V85/X85,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="12"/>
@@ -53704,6 +55151,18 @@
       <x:c r="W86" s="105"/>
       <x:c r="X86" s="105"/>
       <x:c r="Y86" s="102"/>
+      <x:c r="Z86" s="165" t="str">
+        <x:f>IF(A86="","",ROUND(V86/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA86" s="167" t="str">
+        <x:f>IF(V86="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V86)+1)</x:f>
+      </x:c>
+      <x:c r="AB86" s="163" t="str">
+        <x:f>IF(Z86="","",IF(Z86&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z86&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z86&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z86&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC86" s="165" t="str">
+        <x:f>IF(OR(V86="",X86="",X86=0),"",ROUND(V86/X86,1))</x:f>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="12"/>
@@ -53731,11 +55190,26 @@
       <x:c r="W87" s="105"/>
       <x:c r="X87" s="105"/>
       <x:c r="Y87" s="102"/>
+      <x:c r="Z87" s="164" t="str">
+        <x:f>IF(A87="","",ROUND(V87/INDEX($V$5:$V$87,MATCH($AA$3,$A$5:$A$87,0))*100,1))</x:f>
+      </x:c>
+      <x:c r="AA87" s="166" t="str">
+        <x:f>IF(V87="","",COUNTIF($V$5:$V$87,"&gt;"&amp;V87)+1)</x:f>
+      </x:c>
+      <x:c r="AB87" s="162" t="str">
+        <x:f>IF(Z87="","",IF(Z87&gt;='Lists'!$AL$9,'Lists'!$AK$9,IF(Z87&gt;='Lists'!$AL$8,'Lists'!$AK$8,IF(Z87&gt;='Lists'!$AL$7,'Lists'!$AK$7,IF(Z87&gt;='Lists'!$AL$6,'Lists'!$AK$6,'Lists'!$AK$5)))))</x:f>
+      </x:c>
+      <x:c r="AC87" s="164" t="str">
+        <x:f>IF(OR(V87="",X87="",X87=0),"",ROUND(V87/X87,1))</x:f>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Y1"/>
     <x:mergeCell ref="A2:Y2"/>
+    <x:mergeCell ref="Z1:AC1"/>
+    <x:mergeCell ref="Z2:AC2"/>
+    <x:mergeCell ref="AA3:AC3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="V5:V87">
     <x:cfRule type="dataBar" priority="1">
@@ -53765,6 +55239,30 @@
       </x:extLst>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="Z5:Z68">
+    <x:cfRule type="colorScale" priority="3">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8696B"/>
+        <x:color rgb="FFFFEB84"/>
+        <x:color rgb="FF63BE7B"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="AC5:AC68">
+    <x:cfRule type="colorScale" priority="4">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8696B"/>
+        <x:color rgb="FFFFEB84"/>
+        <x:color rgb="FF63BE7B"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="F5:F87">
       <x:formula1>"research_required,approved,preferred,rejected,discontinued"</x:formula1>
@@ -53778,7 +55276,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73bcd74fee214faf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6677125bfc34060"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -55437,7 +56935,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5ee3d2d217d454e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7d9f276a4794565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -56316,7 +57814,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d9dd579fd844508"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13f241c0ea704479"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -57149,7 +58647,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9fe8da79dac4e29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87aa2ee8966e4a94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -58028,7 +59526,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d721a1e48e64105"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46fbbd52ca44eeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>